<commit_message>
PPRTV September 2026 (links corrected)
Every link was one row too high: a chemical's name opened the next
chemical's page, and the header row carried the first chemical's links.
Each link is now on its own row, checked against EPA's page.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PPRTV.xlsx
+++ b/PPRTV.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d4d1dc82d6709298/Documents/Code/RiskResources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AADBB007-4D49-40F2-AC0F-9C6D2FE83327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{670687DC-8C23-4725-AB39-3A96F9E225B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{0970D201-5B99-4FE3-A1B9-35D4DEBF3B63}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{55ED2829-6C41-442F-B1B0-43CAFF6AE9F6}"/>
   </bookViews>
   <sheets>
     <sheet name="PPRTV 0926" sheetId="1" r:id="rId1"/>
@@ -4524,7 +4524,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4541,15 +4541,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <u/>
       <sz val="11"/>
       <color theme="10"/>
@@ -4579,15 +4570,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -4927,7 +4915,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{745DC08D-AE8B-4C75-9243-B69FF27649B3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBE45523-6C76-4660-A56E-2F9D5B1EE8BB}">
   <dimension ref="A1:M411"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -4952,7 +4940,7 @@
       <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
@@ -4964,19 +4952,19 @@
       <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="5" t="s">
@@ -4999,7 +4987,7 @@
       <c r="D2">
         <v>2011</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G2" s="1" t="s">
@@ -5052,7 +5040,7 @@
       <c r="L3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="M3" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -5069,7 +5057,7 @@
       <c r="D4">
         <v>2012</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G4" s="1" t="s">
@@ -5087,7 +5075,7 @@
       <c r="L4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="M4" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -5110,7 +5098,7 @@
       <c r="G5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J5" s="1" t="s">
@@ -5174,13 +5162,13 @@
       <c r="D7">
         <v>2010</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J7" s="1" t="s">
@@ -5209,7 +5197,7 @@
       <c r="D8">
         <v>2005</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G8" s="1" t="s">
@@ -5247,7 +5235,7 @@
       <c r="D9">
         <v>2005</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G9" s="1" t="s">
@@ -5265,7 +5253,7 @@
       <c r="L9" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="M9" s="1" t="s">
+      <c r="M9" s="2" t="s">
         <v>51</v>
       </c>
     </row>
@@ -5282,7 +5270,7 @@
       <c r="D10">
         <v>2004</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G10" s="1" t="s">
@@ -5300,7 +5288,7 @@
       <c r="L10" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="M10" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -5317,7 +5305,7 @@
       <c r="D11">
         <v>2009</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G11" s="1" t="s">
@@ -5335,7 +5323,7 @@
       <c r="L11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="M11" s="1" t="s">
+      <c r="M11" s="2" t="s">
         <v>58</v>
       </c>
     </row>
@@ -5636,7 +5624,7 @@
       <c r="L19" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="M19" s="2" t="s">
+      <c r="M19" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -5659,7 +5647,7 @@
       <c r="G20" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="H20" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J20" s="1" t="s">
@@ -5694,7 +5682,7 @@
       <c r="G21" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="H21" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J21" s="1" t="s">
@@ -5706,7 +5694,7 @@
       <c r="L21" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="M21" s="1" t="s">
+      <c r="M21" s="2" t="s">
         <v>98</v>
       </c>
     </row>
@@ -5805,7 +5793,7 @@
       <c r="G24" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H24" s="2" t="s">
+      <c r="H24" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J24" s="1" t="s">
@@ -5817,7 +5805,7 @@
       <c r="L24" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="M24" s="2" t="s">
+      <c r="M24" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -5843,7 +5831,7 @@
       <c r="G25" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H25" s="1" t="s">
+      <c r="H25" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J25" s="1" t="s">
@@ -5855,7 +5843,7 @@
       <c r="L25" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="M25" s="1" t="s">
+      <c r="M25" s="2" t="s">
         <v>115</v>
       </c>
     </row>
@@ -5872,7 +5860,7 @@
       <c r="D26">
         <v>2005</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G26" s="1" t="s">
@@ -5890,7 +5878,7 @@
       <c r="L26" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="M26" s="2" t="s">
+      <c r="M26" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -5907,7 +5895,7 @@
       <c r="D27">
         <v>2009</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="E27" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G27" s="1" t="s">
@@ -5925,7 +5913,7 @@
       <c r="L27" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="M27" s="1" t="s">
+      <c r="M27" s="2" t="s">
         <v>122</v>
       </c>
     </row>
@@ -5942,7 +5930,7 @@
       <c r="D28">
         <v>2011</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G28" s="1" t="s">
@@ -5960,7 +5948,7 @@
       <c r="L28" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="M28" s="2" t="s">
+      <c r="M28" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -5977,13 +5965,13 @@
       <c r="D29">
         <v>2008</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="E29" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H29" s="2" t="s">
+      <c r="H29" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J29" s="1" t="s">
@@ -6018,7 +6006,7 @@
       <c r="G30" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="H30" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J30" s="1" t="s">
@@ -6030,7 +6018,7 @@
       <c r="L30" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="M30" s="1" t="s">
+      <c r="M30" s="2" t="s">
         <v>135</v>
       </c>
     </row>
@@ -6106,7 +6094,7 @@
       <c r="L32" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="M32" s="2" t="s">
+      <c r="M32" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -6123,7 +6111,7 @@
       <c r="D33">
         <v>2007</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="E33" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G33" s="1" t="s">
@@ -6164,7 +6152,7 @@
       <c r="G34" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H34" s="2" t="s">
+      <c r="H34" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J34" s="1" t="s">
@@ -6193,13 +6181,13 @@
       <c r="D35">
         <v>2009</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="E35" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G35" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H35" s="1" t="s">
+      <c r="H35" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J35" s="1" t="s">
@@ -6211,7 +6199,7 @@
       <c r="L35" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="M35" s="1" t="s">
+      <c r="M35" s="2" t="s">
         <v>154</v>
       </c>
     </row>
@@ -6284,7 +6272,7 @@
       <c r="L37" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="M37" s="2" t="s">
+      <c r="M37" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -6319,7 +6307,7 @@
       <c r="L38" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="M38" s="1" t="s">
+      <c r="M38" s="2" t="s">
         <v>166</v>
       </c>
     </row>
@@ -6360,7 +6348,7 @@
       <c r="L39" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="M39" s="2" t="s">
+      <c r="M39" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -6395,7 +6383,7 @@
       <c r="L40" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="M40" s="1" t="s">
+      <c r="M40" s="2" t="s">
         <v>176</v>
       </c>
     </row>
@@ -6412,7 +6400,7 @@
       <c r="D41">
         <v>2024</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="E41" s="1" t="s">
         <v>179</v>
       </c>
       <c r="F41">
@@ -6433,7 +6421,7 @@
       <c r="L41" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="M41" s="2" t="s">
+      <c r="M41" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -6450,7 +6438,7 @@
       <c r="D42">
         <v>2005</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="E42" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G42" s="1" t="s">
@@ -6468,7 +6456,7 @@
       <c r="L42" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="M42" s="1" t="s">
+      <c r="M42" s="2" t="s">
         <v>184</v>
       </c>
     </row>
@@ -6503,7 +6491,7 @@
       <c r="L43" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="M43" s="2" t="s">
+      <c r="M43" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -6579,7 +6567,7 @@
       <c r="L45" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="M45" s="1" t="s">
+      <c r="M45" s="2" t="s">
         <v>198</v>
       </c>
     </row>
@@ -6634,7 +6622,7 @@
       <c r="D47">
         <v>2006</v>
       </c>
-      <c r="E47" s="2" t="s">
+      <c r="E47" s="1" t="s">
         <v>205</v>
       </c>
       <c r="F47">
@@ -6655,7 +6643,7 @@
       <c r="L47" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="M47" s="2" t="s">
+      <c r="M47" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -6707,7 +6695,7 @@
       <c r="D49">
         <v>2011</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="E49" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G49" s="1" t="s">
@@ -6763,7 +6751,7 @@
       <c r="L50" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="M50" s="1" t="s">
+      <c r="M50" s="2" t="s">
         <v>219</v>
       </c>
     </row>
@@ -6950,7 +6938,7 @@
       <c r="L55" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="M55" s="2" t="s">
+      <c r="M55" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -6967,7 +6955,7 @@
       <c r="D56">
         <v>2009</v>
       </c>
-      <c r="E56" s="2" t="s">
+      <c r="E56" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G56" s="1" t="s">
@@ -7002,7 +6990,7 @@
       <c r="D57">
         <v>2009</v>
       </c>
-      <c r="E57" s="1" t="s">
+      <c r="E57" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G57" s="1" t="s">
@@ -7055,7 +7043,7 @@
       <c r="L58" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="M58" s="1" t="s">
+      <c r="M58" s="2" t="s">
         <v>250</v>
       </c>
     </row>
@@ -7072,7 +7060,7 @@
       <c r="D59">
         <v>2017</v>
       </c>
-      <c r="E59" s="2" t="s">
+      <c r="E59" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G59" s="1" t="s">
@@ -7090,7 +7078,7 @@
       <c r="L59" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="M59" s="2" t="s">
+      <c r="M59" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -7113,7 +7101,7 @@
       <c r="G60" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H60" s="2" t="s">
+      <c r="H60" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J60" s="1" t="s">
@@ -7142,13 +7130,13 @@
       <c r="D61">
         <v>2007</v>
       </c>
-      <c r="E61" s="1" t="s">
+      <c r="E61" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G61" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H61" s="1" t="s">
+      <c r="H61" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J61" s="1" t="s">
@@ -7160,7 +7148,7 @@
       <c r="L61" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="M61" s="1" t="s">
+      <c r="M61" s="2" t="s">
         <v>262</v>
       </c>
     </row>
@@ -7247,7 +7235,7 @@
       <c r="D64">
         <v>2009</v>
       </c>
-      <c r="E64" s="2" t="s">
+      <c r="E64" s="1" t="s">
         <v>222</v>
       </c>
       <c r="F64">
@@ -7271,7 +7259,7 @@
       <c r="L64" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="M64" s="2" t="s">
+      <c r="M64" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -7288,7 +7276,7 @@
       <c r="D65">
         <v>2002</v>
       </c>
-      <c r="E65" s="1" t="s">
+      <c r="E65" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G65" s="1" t="s">
@@ -7306,7 +7294,7 @@
       <c r="L65" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="M65" s="1" t="s">
+      <c r="M65" s="2" t="s">
         <v>277</v>
       </c>
     </row>
@@ -7703,7 +7691,7 @@
       <c r="L76" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="M76" s="2" t="s">
+      <c r="M76" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -7741,7 +7729,7 @@
       <c r="L77" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="M77" s="1" t="s">
+      <c r="M77" s="2" t="s">
         <v>314</v>
       </c>
     </row>
@@ -7895,7 +7883,7 @@
       <c r="D82">
         <v>2004</v>
       </c>
-      <c r="E82" s="2" t="s">
+      <c r="E82" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G82" s="1" t="s">
@@ -7913,7 +7901,7 @@
       <c r="L82" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="M82" s="2" t="s">
+      <c r="M82" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -7965,7 +7953,7 @@
       <c r="D84">
         <v>2006</v>
       </c>
-      <c r="E84" s="1" t="s">
+      <c r="E84" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G84" s="1" t="s">
@@ -7986,7 +7974,7 @@
       <c r="L84" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="M84" s="1" t="s">
+      <c r="M84" s="2" t="s">
         <v>339</v>
       </c>
     </row>
@@ -8167,7 +8155,7 @@
       <c r="L89" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="M89" s="2" t="s">
+      <c r="M89" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -8228,7 +8216,7 @@
       <c r="G91" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H91" s="2" t="s">
+      <c r="H91" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J91" s="1" t="s">
@@ -8263,7 +8251,7 @@
       <c r="G92" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H92" s="1" t="s">
+      <c r="H92" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J92" s="1" t="s">
@@ -8275,7 +8263,7 @@
       <c r="L92" s="2" t="s">
         <v>367</v>
       </c>
-      <c r="M92" s="1" t="s">
+      <c r="M92" s="2" t="s">
         <v>368</v>
       </c>
     </row>
@@ -8301,7 +8289,7 @@
       <c r="G93" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H93" s="2" t="s">
+      <c r="H93" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J93" s="1" t="s">
@@ -8313,7 +8301,7 @@
       <c r="L93" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="M93" s="2" t="s">
+      <c r="M93" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -8330,13 +8318,13 @@
       <c r="D94">
         <v>2012</v>
       </c>
-      <c r="E94" s="2" t="s">
+      <c r="E94" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G94" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H94" s="1" t="s">
+      <c r="H94" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J94" s="1" t="s">
@@ -8365,7 +8353,7 @@
       <c r="D95">
         <v>2009</v>
       </c>
-      <c r="E95" s="1" t="s">
+      <c r="E95" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G95" s="1" t="s">
@@ -8383,7 +8371,7 @@
       <c r="L95" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="M95" s="1" t="s">
+      <c r="M95" s="2" t="s">
         <v>379</v>
       </c>
     </row>
@@ -8479,7 +8467,7 @@
       <c r="D98">
         <v>2015</v>
       </c>
-      <c r="E98" s="2" t="s">
+      <c r="E98" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G98" s="1" t="s">
@@ -8497,7 +8485,7 @@
       <c r="L98" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="M98" s="2" t="s">
+      <c r="M98" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -8514,7 +8502,7 @@
       <c r="D99">
         <v>2007</v>
       </c>
-      <c r="E99" s="1" t="s">
+      <c r="E99" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G99" s="1" t="s">
@@ -8532,7 +8520,7 @@
       <c r="L99" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="M99" s="1" t="s">
+      <c r="M99" s="2" t="s">
         <v>394</v>
       </c>
     </row>
@@ -8584,7 +8572,7 @@
       <c r="D101">
         <v>2010</v>
       </c>
-      <c r="E101" s="2" t="s">
+      <c r="E101" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G101" s="1" t="s">
@@ -8602,7 +8590,7 @@
       <c r="L101" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="M101" s="2" t="s">
+      <c r="M101" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -8619,7 +8607,7 @@
       <c r="D102">
         <v>2010</v>
       </c>
-      <c r="E102" s="1" t="s">
+      <c r="E102" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G102" s="1" t="s">
@@ -8672,7 +8660,7 @@
       <c r="L103" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="M103" s="1" t="s">
+      <c r="M103" s="2" t="s">
         <v>409</v>
       </c>
     </row>
@@ -8783,7 +8771,7 @@
       <c r="L106" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="M106" s="2" t="s">
+      <c r="M106" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -8800,7 +8788,7 @@
       <c r="D107">
         <v>2021</v>
       </c>
-      <c r="E107" s="2" t="s">
+      <c r="E107" s="1" t="s">
         <v>160</v>
       </c>
       <c r="F107">
@@ -8838,13 +8826,13 @@
       <c r="D108">
         <v>2012</v>
       </c>
-      <c r="E108" s="1" t="s">
+      <c r="E108" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G108" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H108" s="2" t="s">
+      <c r="H108" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J108" s="1" t="s">
@@ -8873,13 +8861,13 @@
       <c r="D109">
         <v>2010</v>
       </c>
-      <c r="E109" s="2" t="s">
+      <c r="E109" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G109" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H109" s="1" t="s">
+      <c r="H109" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J109" s="1" t="s">
@@ -8908,7 +8896,7 @@
       <c r="D110">
         <v>2010</v>
       </c>
-      <c r="E110" s="1" t="s">
+      <c r="E110" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G110" s="1" t="s">
@@ -8929,7 +8917,7 @@
       <c r="L110" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="M110" s="1" t="s">
+      <c r="M110" s="2" t="s">
         <v>436</v>
       </c>
     </row>
@@ -8967,7 +8955,7 @@
       <c r="L111" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="M111" s="2" t="s">
+      <c r="M111" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -9002,7 +8990,7 @@
       <c r="L112" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="M112" s="1" t="s">
+      <c r="M112" s="2" t="s">
         <v>444</v>
       </c>
     </row>
@@ -9037,7 +9025,7 @@
       <c r="L113" s="2" t="s">
         <v>447</v>
       </c>
-      <c r="M113" s="2" t="s">
+      <c r="M113" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -9072,7 +9060,7 @@
       <c r="L114" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="M114" s="1" t="s">
+      <c r="M114" s="2" t="s">
         <v>452</v>
       </c>
     </row>
@@ -9177,7 +9165,7 @@
       <c r="L117" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="M117" s="2" t="s">
+      <c r="M117" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -9212,7 +9200,7 @@
       <c r="L118" s="2" t="s">
         <v>464</v>
       </c>
-      <c r="M118" s="1" t="s">
+      <c r="M118" s="2" t="s">
         <v>465</v>
       </c>
     </row>
@@ -9235,7 +9223,7 @@
       <c r="G119" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H119" s="2" t="s">
+      <c r="H119" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J119" s="1" t="s">
@@ -9247,7 +9235,7 @@
       <c r="L119" s="2" t="s">
         <v>468</v>
       </c>
-      <c r="M119" s="2" t="s">
+      <c r="M119" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -9273,7 +9261,7 @@
       <c r="G120" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H120" s="1" t="s">
+      <c r="H120" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J120" s="1" t="s">
@@ -9285,7 +9273,7 @@
       <c r="L120" s="2" t="s">
         <v>472</v>
       </c>
-      <c r="M120" s="1" t="s">
+      <c r="M120" s="2" t="s">
         <v>473</v>
       </c>
     </row>
@@ -9302,7 +9290,7 @@
       <c r="D121">
         <v>2014</v>
       </c>
-      <c r="E121" s="2" t="s">
+      <c r="E121" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G121" s="1" t="s">
@@ -9320,7 +9308,7 @@
       <c r="L121" s="2" t="s">
         <v>476</v>
       </c>
-      <c r="M121" s="2" t="s">
+      <c r="M121" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -9337,7 +9325,7 @@
       <c r="D122">
         <v>2009</v>
       </c>
-      <c r="E122" s="1" t="s">
+      <c r="E122" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G122" s="1" t="s">
@@ -9355,7 +9343,7 @@
       <c r="L122" s="2" t="s">
         <v>480</v>
       </c>
-      <c r="M122" s="1" t="s">
+      <c r="M122" s="2" t="s">
         <v>481</v>
       </c>
     </row>
@@ -9547,7 +9535,7 @@
       <c r="D128">
         <v>2013</v>
       </c>
-      <c r="E128" s="2" t="s">
+      <c r="E128" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G128" s="1" t="s">
@@ -9565,7 +9553,7 @@
       <c r="L128" s="2" t="s">
         <v>499</v>
       </c>
-      <c r="M128" s="2" t="s">
+      <c r="M128" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -9582,7 +9570,7 @@
       <c r="D129">
         <v>2010</v>
       </c>
-      <c r="E129" s="1" t="s">
+      <c r="E129" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G129" s="1" t="s">
@@ -9655,7 +9643,7 @@
       <c r="D131">
         <v>2006</v>
       </c>
-      <c r="E131" s="2" t="s">
+      <c r="E131" s="1" t="s">
         <v>512</v>
       </c>
       <c r="F131">
@@ -9731,7 +9719,7 @@
       <c r="D133">
         <v>2022</v>
       </c>
-      <c r="E133" s="1" t="s">
+      <c r="E133" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G133" s="1" t="s">
@@ -9752,7 +9740,7 @@
       <c r="L133" s="2" t="s">
         <v>524</v>
       </c>
-      <c r="M133" s="1" t="s">
+      <c r="M133" s="2" t="s">
         <v>525</v>
       </c>
     </row>
@@ -9769,7 +9757,7 @@
       <c r="D134">
         <v>2002</v>
       </c>
-      <c r="E134" s="2" t="s">
+      <c r="E134" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G134" s="1" t="s">
@@ -9787,7 +9775,7 @@
       <c r="L134" s="2" t="s">
         <v>528</v>
       </c>
-      <c r="M134" s="2" t="s">
+      <c r="M134" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -9804,13 +9792,13 @@
       <c r="D135">
         <v>2007</v>
       </c>
-      <c r="E135" s="1" t="s">
+      <c r="E135" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G135" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H135" s="2" t="s">
+      <c r="H135" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J135" s="1" t="s">
@@ -9848,7 +9836,7 @@
       <c r="G136" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H136" s="1" t="s">
+      <c r="H136" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J136" s="1" t="s">
@@ -9860,7 +9848,7 @@
       <c r="L136" s="2" t="s">
         <v>535</v>
       </c>
-      <c r="M136" s="1" t="s">
+      <c r="M136" s="2" t="s">
         <v>536</v>
       </c>
     </row>
@@ -10327,7 +10315,7 @@
       <c r="D149">
         <v>2011</v>
       </c>
-      <c r="E149" s="2" t="s">
+      <c r="E149" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G149" s="1" t="s">
@@ -10348,7 +10336,7 @@
       <c r="L149" s="2" t="s">
         <v>580</v>
       </c>
-      <c r="M149" s="2" t="s">
+      <c r="M149" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -10365,7 +10353,7 @@
       <c r="D150">
         <v>2013</v>
       </c>
-      <c r="E150" s="1" t="s">
+      <c r="E150" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G150" s="1" t="s">
@@ -10383,7 +10371,7 @@
       <c r="L150" s="2" t="s">
         <v>583</v>
       </c>
-      <c r="M150" s="1" t="s">
+      <c r="M150" s="2" t="s">
         <v>584</v>
       </c>
     </row>
@@ -10514,7 +10502,7 @@
       <c r="D154">
         <v>2006</v>
       </c>
-      <c r="E154" s="2" t="s">
+      <c r="E154" s="1" t="s">
         <v>563</v>
       </c>
       <c r="F154">
@@ -10535,7 +10523,7 @@
       <c r="L154" s="2" t="s">
         <v>596</v>
       </c>
-      <c r="M154" s="2" t="s">
+      <c r="M154" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -10552,7 +10540,7 @@
       <c r="D155">
         <v>2016</v>
       </c>
-      <c r="E155" s="1" t="s">
+      <c r="E155" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G155" s="1" t="s">
@@ -10570,7 +10558,7 @@
       <c r="L155" s="2" t="s">
         <v>599</v>
       </c>
-      <c r="M155" s="1" t="s">
+      <c r="M155" s="2" t="s">
         <v>600</v>
       </c>
     </row>
@@ -10605,7 +10593,7 @@
       <c r="L156" s="2" t="s">
         <v>603</v>
       </c>
-      <c r="M156" s="2" t="s">
+      <c r="M156" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -10640,7 +10628,7 @@
       <c r="L157" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="M157" s="1" t="s">
+      <c r="M157" s="2" t="s">
         <v>607</v>
       </c>
     </row>
@@ -10663,7 +10651,7 @@
       <c r="G158" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H158" s="2" t="s">
+      <c r="H158" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J158" s="1" t="s">
@@ -10675,7 +10663,7 @@
       <c r="L158" s="2" t="s">
         <v>610</v>
       </c>
-      <c r="M158" s="2" t="s">
+      <c r="M158" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -10701,7 +10689,7 @@
       <c r="G159" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H159" s="1" t="s">
+      <c r="H159" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J159" s="1" t="s">
@@ -10713,7 +10701,7 @@
       <c r="L159" s="2" t="s">
         <v>613</v>
       </c>
-      <c r="M159" s="1" t="s">
+      <c r="M159" s="2" t="s">
         <v>614</v>
       </c>
     </row>
@@ -10800,7 +10788,7 @@
       <c r="D162">
         <v>2004</v>
       </c>
-      <c r="E162" s="2" t="s">
+      <c r="E162" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G162" s="1" t="s">
@@ -10818,7 +10806,7 @@
       <c r="L162" s="2" t="s">
         <v>623</v>
       </c>
-      <c r="M162" s="2" t="s">
+      <c r="M162" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -10835,7 +10823,7 @@
       <c r="D163">
         <v>2007</v>
       </c>
-      <c r="E163" s="1" t="s">
+      <c r="E163" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G163" s="1" t="s">
@@ -10888,7 +10876,7 @@
       <c r="L164" s="2" t="s">
         <v>631</v>
       </c>
-      <c r="M164" s="1" t="s">
+      <c r="M164" s="2" t="s">
         <v>632</v>
       </c>
     </row>
@@ -10964,7 +10952,7 @@
       <c r="L166" s="2" t="s">
         <v>639</v>
       </c>
-      <c r="M166" s="2" t="s">
+      <c r="M166" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -11002,7 +10990,7 @@
       <c r="L167" s="2" t="s">
         <v>642</v>
       </c>
-      <c r="M167" s="1" t="s">
+      <c r="M167" s="2" t="s">
         <v>643</v>
       </c>
     </row>
@@ -11019,7 +11007,7 @@
       <c r="D168">
         <v>2006</v>
       </c>
-      <c r="E168" s="2" t="s">
+      <c r="E168" s="1" t="s">
         <v>71</v>
       </c>
       <c r="F168">
@@ -11040,7 +11028,7 @@
       <c r="L168" s="2" t="s">
         <v>646</v>
       </c>
-      <c r="M168" s="2" t="s">
+      <c r="M168" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -11057,7 +11045,7 @@
       <c r="D169">
         <v>2007</v>
       </c>
-      <c r="E169" s="1" t="s">
+      <c r="E169" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G169" s="1" t="s">
@@ -11075,7 +11063,7 @@
       <c r="L169" s="2" t="s">
         <v>649</v>
       </c>
-      <c r="M169" s="1" t="s">
+      <c r="M169" s="2" t="s">
         <v>650</v>
       </c>
     </row>
@@ -11162,7 +11150,7 @@
       <c r="D172">
         <v>2013</v>
       </c>
-      <c r="E172" s="2" t="s">
+      <c r="E172" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G172" s="1" t="s">
@@ -11180,7 +11168,7 @@
       <c r="L172" s="2" t="s">
         <v>659</v>
       </c>
-      <c r="M172" s="2" t="s">
+      <c r="M172" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -11197,7 +11185,7 @@
       <c r="D173">
         <v>2002</v>
       </c>
-      <c r="E173" s="1" t="s">
+      <c r="E173" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G173" s="1" t="s">
@@ -11215,7 +11203,7 @@
       <c r="L173" s="2" t="s">
         <v>663</v>
       </c>
-      <c r="M173" s="1" t="s">
+      <c r="M173" s="2" t="s">
         <v>664</v>
       </c>
     </row>
@@ -11302,7 +11290,7 @@
       <c r="D176">
         <v>2009</v>
       </c>
-      <c r="E176" s="2" t="s">
+      <c r="E176" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G176" s="1" t="s">
@@ -11320,7 +11308,7 @@
       <c r="L176" s="2" t="s">
         <v>673</v>
       </c>
-      <c r="M176" s="2" t="s">
+      <c r="M176" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -11372,7 +11360,7 @@
       <c r="D178">
         <v>2002</v>
       </c>
-      <c r="E178" s="1" t="s">
+      <c r="E178" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G178" s="1" t="s">
@@ -11390,7 +11378,7 @@
       <c r="L178" s="2" t="s">
         <v>680</v>
       </c>
-      <c r="M178" s="1" t="s">
+      <c r="M178" s="2" t="s">
         <v>681</v>
       </c>
     </row>
@@ -11407,7 +11395,7 @@
       <c r="D179">
         <v>2015</v>
       </c>
-      <c r="E179" s="2" t="s">
+      <c r="E179" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G179" s="1" t="s">
@@ -11425,7 +11413,7 @@
       <c r="L179" s="2" t="s">
         <v>684</v>
       </c>
-      <c r="M179" s="2" t="s">
+      <c r="M179" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -11442,7 +11430,7 @@
       <c r="D180">
         <v>2009</v>
       </c>
-      <c r="E180" s="1" t="s">
+      <c r="E180" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G180" s="1" t="s">
@@ -11460,7 +11448,7 @@
       <c r="L180" s="2" t="s">
         <v>687</v>
       </c>
-      <c r="M180" s="1" t="s">
+      <c r="M180" s="2" t="s">
         <v>688</v>
       </c>
     </row>
@@ -11477,7 +11465,7 @@
       <c r="D181">
         <v>2013</v>
       </c>
-      <c r="E181" s="2" t="s">
+      <c r="E181" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G181" s="1" t="s">
@@ -11495,7 +11483,7 @@
       <c r="L181" s="2" t="s">
         <v>691</v>
       </c>
-      <c r="M181" s="2" t="s">
+      <c r="M181" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -11512,7 +11500,7 @@
       <c r="D182">
         <v>2002</v>
       </c>
-      <c r="E182" s="1" t="s">
+      <c r="E182" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G182" s="1" t="s">
@@ -11530,7 +11518,7 @@
       <c r="L182" s="2" t="s">
         <v>695</v>
       </c>
-      <c r="M182" s="1" t="s">
+      <c r="M182" s="2" t="s">
         <v>696</v>
       </c>
     </row>
@@ -11588,7 +11576,7 @@
       <c r="G184" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H184" s="2" t="s">
+      <c r="H184" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J184" s="1" t="s">
@@ -11600,7 +11588,7 @@
       <c r="L184" s="2" t="s">
         <v>702</v>
       </c>
-      <c r="M184" s="2" t="s">
+      <c r="M184" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -11664,7 +11652,7 @@
       <c r="G186" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H186" s="1" t="s">
+      <c r="H186" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J186" s="1" t="s">
@@ -11676,7 +11664,7 @@
       <c r="L186" s="2" t="s">
         <v>711</v>
       </c>
-      <c r="M186" s="1" t="s">
+      <c r="M186" s="2" t="s">
         <v>712</v>
       </c>
     </row>
@@ -11693,7 +11681,7 @@
       <c r="D187">
         <v>2010</v>
       </c>
-      <c r="E187" s="2" t="s">
+      <c r="E187" s="1" t="s">
         <v>201</v>
       </c>
       <c r="F187">
@@ -11717,7 +11705,7 @@
       <c r="L187" s="2" t="s">
         <v>716</v>
       </c>
-      <c r="M187" s="2" t="s">
+      <c r="M187" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -11734,7 +11722,7 @@
       <c r="D188">
         <v>2013</v>
       </c>
-      <c r="E188" s="1" t="s">
+      <c r="E188" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G188" s="1" t="s">
@@ -11755,7 +11743,7 @@
       <c r="L188" s="2" t="s">
         <v>720</v>
       </c>
-      <c r="M188" s="1" t="s">
+      <c r="M188" s="2" t="s">
         <v>721</v>
       </c>
     </row>
@@ -11772,7 +11760,7 @@
       <c r="D189">
         <v>2014</v>
       </c>
-      <c r="E189" s="2" t="s">
+      <c r="E189" s="1" t="s">
         <v>179</v>
       </c>
       <c r="F189">
@@ -11796,7 +11784,7 @@
       <c r="L189" s="2" t="s">
         <v>725</v>
       </c>
-      <c r="M189" s="2" t="s">
+      <c r="M189" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -11813,7 +11801,7 @@
       <c r="D190">
         <v>2009</v>
       </c>
-      <c r="E190" s="1" t="s">
+      <c r="E190" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G190" s="1" t="s">
@@ -11831,7 +11819,7 @@
       <c r="L190" s="2" t="s">
         <v>728</v>
       </c>
-      <c r="M190" s="1" t="s">
+      <c r="M190" s="2" t="s">
         <v>729</v>
       </c>
     </row>
@@ -11848,13 +11836,13 @@
       <c r="D191">
         <v>2010</v>
       </c>
-      <c r="E191" s="2" t="s">
+      <c r="E191" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G191" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H191" s="2" t="s">
+      <c r="H191" s="1" t="s">
         <v>351</v>
       </c>
       <c r="I191">
@@ -11869,7 +11857,7 @@
       <c r="L191" s="2" t="s">
         <v>732</v>
       </c>
-      <c r="M191" s="2" t="s">
+      <c r="M191" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -11886,13 +11874,13 @@
       <c r="D192">
         <v>2009</v>
       </c>
-      <c r="E192" s="1" t="s">
+      <c r="E192" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G192" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H192" s="1" t="s">
+      <c r="H192" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J192" s="1" t="s">
@@ -11904,7 +11892,7 @@
       <c r="L192" s="2" t="s">
         <v>736</v>
       </c>
-      <c r="M192" s="1" t="s">
+      <c r="M192" s="2" t="s">
         <v>737</v>
       </c>
     </row>
@@ -11942,7 +11930,7 @@
       <c r="L193" s="2" t="s">
         <v>741</v>
       </c>
-      <c r="M193" s="2" t="s">
+      <c r="M193" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -11980,7 +11968,7 @@
       <c r="L194" s="2" t="s">
         <v>744</v>
       </c>
-      <c r="M194" s="1" t="s">
+      <c r="M194" s="2" t="s">
         <v>745</v>
       </c>
     </row>
@@ -11997,7 +11985,7 @@
       <c r="D195">
         <v>2019</v>
       </c>
-      <c r="E195" s="2" t="s">
+      <c r="E195" s="1" t="s">
         <v>740</v>
       </c>
       <c r="F195">
@@ -12021,7 +12009,7 @@
       <c r="L195" s="2" t="s">
         <v>749</v>
       </c>
-      <c r="M195" s="2" t="s">
+      <c r="M195" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -12073,7 +12061,7 @@
       <c r="D197">
         <v>2023</v>
       </c>
-      <c r="E197" s="1" t="s">
+      <c r="E197" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G197" s="1" t="s">
@@ -12091,7 +12079,7 @@
       <c r="L197" s="2" t="s">
         <v>757</v>
       </c>
-      <c r="M197" s="1" t="s">
+      <c r="M197" s="2" t="s">
         <v>758</v>
       </c>
     </row>
@@ -12196,7 +12184,7 @@
       <c r="L200" s="2" t="s">
         <v>767</v>
       </c>
-      <c r="M200" s="2" t="s">
+      <c r="M200" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -12234,7 +12222,7 @@
       <c r="L201" s="2" t="s">
         <v>771</v>
       </c>
-      <c r="M201" s="1" t="s">
+      <c r="M201" s="2" t="s">
         <v>772</v>
       </c>
     </row>
@@ -12251,7 +12239,7 @@
       <c r="D202">
         <v>2018</v>
       </c>
-      <c r="E202" s="2" t="s">
+      <c r="E202" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G202" s="1" t="s">
@@ -12269,7 +12257,7 @@
       <c r="L202" s="2" t="s">
         <v>775</v>
       </c>
-      <c r="M202" s="2" t="s">
+      <c r="M202" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -12286,7 +12274,7 @@
       <c r="D203">
         <v>2020</v>
       </c>
-      <c r="E203" s="1" t="s">
+      <c r="E203" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G203" s="1" t="s">
@@ -12307,7 +12295,7 @@
       <c r="L203" s="2" t="s">
         <v>779</v>
       </c>
-      <c r="M203" s="1" t="s">
+      <c r="M203" s="2" t="s">
         <v>780</v>
       </c>
     </row>
@@ -12447,7 +12435,7 @@
       <c r="L207" s="2" t="s">
         <v>792</v>
       </c>
-      <c r="M207" s="2" t="s">
+      <c r="M207" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -12464,7 +12452,7 @@
       <c r="D208">
         <v>2016</v>
       </c>
-      <c r="E208" s="2" t="s">
+      <c r="E208" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G208" s="1" t="s">
@@ -12502,7 +12490,7 @@
       <c r="D209">
         <v>2010</v>
       </c>
-      <c r="E209" s="1" t="s">
+      <c r="E209" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G209" s="1" t="s">
@@ -12596,7 +12584,7 @@
       <c r="L211" s="2" t="s">
         <v>812</v>
       </c>
-      <c r="M211" s="1" t="s">
+      <c r="M211" s="2" t="s">
         <v>813</v>
       </c>
     </row>
@@ -12657,7 +12645,7 @@
       <c r="G213" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H213" s="2" t="s">
+      <c r="H213" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J213" s="1" t="s">
@@ -12669,7 +12657,7 @@
       <c r="L213" s="2" t="s">
         <v>819</v>
       </c>
-      <c r="M213" s="2" t="s">
+      <c r="M213" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -12692,7 +12680,7 @@
       <c r="G214" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H214" s="1" t="s">
+      <c r="H214" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J214" s="1" t="s">
@@ -12704,7 +12692,7 @@
       <c r="L214" s="2" t="s">
         <v>823</v>
       </c>
-      <c r="M214" s="1" t="s">
+      <c r="M214" s="2" t="s">
         <v>824</v>
       </c>
     </row>
@@ -12780,7 +12768,7 @@
       <c r="L216" s="2" t="s">
         <v>830</v>
       </c>
-      <c r="M216" s="2" t="s">
+      <c r="M216" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -12926,7 +12914,7 @@
       <c r="L220" s="2" t="s">
         <v>848</v>
       </c>
-      <c r="M220" s="1" t="s">
+      <c r="M220" s="2" t="s">
         <v>849</v>
       </c>
     </row>
@@ -12978,7 +12966,7 @@
       <c r="D222">
         <v>2006</v>
       </c>
-      <c r="E222" s="2" t="s">
+      <c r="E222" s="1" t="s">
         <v>855</v>
       </c>
       <c r="F222">
@@ -12999,7 +12987,7 @@
       <c r="L222" s="2" t="s">
         <v>856</v>
       </c>
-      <c r="M222" s="2" t="s">
+      <c r="M222" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -13016,7 +13004,7 @@
       <c r="D223">
         <v>2023</v>
       </c>
-      <c r="E223" s="1" t="s">
+      <c r="E223" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G223" s="1" t="s">
@@ -13037,7 +13025,7 @@
       <c r="L223" s="2" t="s">
         <v>859</v>
       </c>
-      <c r="M223" s="1" t="s">
+      <c r="M223" s="2" t="s">
         <v>860</v>
       </c>
     </row>
@@ -13396,7 +13384,7 @@
       <c r="D233">
         <v>2002</v>
       </c>
-      <c r="E233" s="2" t="s">
+      <c r="E233" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G233" s="1" t="s">
@@ -13414,7 +13402,7 @@
       <c r="L233" s="2" t="s">
         <v>894</v>
       </c>
-      <c r="M233" s="2" t="s">
+      <c r="M233" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -13431,13 +13419,13 @@
       <c r="D234">
         <v>2012</v>
       </c>
-      <c r="E234" s="1" t="s">
+      <c r="E234" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G234" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H234" s="2" t="s">
+      <c r="H234" s="1" t="s">
         <v>897</v>
       </c>
       <c r="I234">
@@ -13478,7 +13466,7 @@
       <c r="G235" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H235" s="1" t="s">
+      <c r="H235" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J235" s="1" t="s">
@@ -13490,7 +13478,7 @@
       <c r="L235" s="2" t="s">
         <v>903</v>
       </c>
-      <c r="M235" s="1" t="s">
+      <c r="M235" s="2" t="s">
         <v>904</v>
       </c>
     </row>
@@ -13566,7 +13554,7 @@
       <c r="L237" s="2" t="s">
         <v>911</v>
       </c>
-      <c r="M237" s="2" t="s">
+      <c r="M237" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -13604,7 +13592,7 @@
       <c r="L238" s="2" t="s">
         <v>915</v>
       </c>
-      <c r="M238" s="1" t="s">
+      <c r="M238" s="2" t="s">
         <v>916</v>
       </c>
     </row>
@@ -14088,7 +14076,7 @@
       <c r="D252">
         <v>2024</v>
       </c>
-      <c r="E252" s="2" t="s">
+      <c r="E252" s="1" t="s">
         <v>958</v>
       </c>
       <c r="F252">
@@ -14112,7 +14100,7 @@
       <c r="L252" s="2" t="s">
         <v>960</v>
       </c>
-      <c r="M252" s="2" t="s">
+      <c r="M252" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -14199,7 +14187,7 @@
       <c r="D255">
         <v>2016</v>
       </c>
-      <c r="E255" s="1" t="s">
+      <c r="E255" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G255" s="1" t="s">
@@ -14252,7 +14240,7 @@
       <c r="L256" s="2" t="s">
         <v>978</v>
       </c>
-      <c r="M256" s="1" t="s">
+      <c r="M256" s="2" t="s">
         <v>979</v>
       </c>
     </row>
@@ -14780,7 +14768,7 @@
       <c r="D271">
         <v>2006</v>
       </c>
-      <c r="E271" s="2" t="s">
+      <c r="E271" s="1" t="s">
         <v>71</v>
       </c>
       <c r="F271">
@@ -14801,7 +14789,7 @@
       <c r="L271" s="2" t="s">
         <v>1025</v>
       </c>
-      <c r="M271" s="2" t="s">
+      <c r="M271" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -14818,7 +14806,7 @@
       <c r="D272">
         <v>2009</v>
       </c>
-      <c r="E272" s="1" t="s">
+      <c r="E272" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G272" s="1" t="s">
@@ -14836,7 +14824,7 @@
       <c r="L272" s="2" t="s">
         <v>1028</v>
       </c>
-      <c r="M272" s="1" t="s">
+      <c r="M272" s="2" t="s">
         <v>1029</v>
       </c>
     </row>
@@ -14874,7 +14862,7 @@
       <c r="L273" s="2" t="s">
         <v>1032</v>
       </c>
-      <c r="M273" s="2" t="s">
+      <c r="M273" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -14909,7 +14897,7 @@
       <c r="L274" s="2" t="s">
         <v>1035</v>
       </c>
-      <c r="M274" s="1" t="s">
+      <c r="M274" s="2" t="s">
         <v>1036</v>
       </c>
     </row>
@@ -14932,7 +14920,7 @@
       <c r="G275" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H275" s="2" t="s">
+      <c r="H275" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J275" s="1" t="s">
@@ -14944,7 +14932,7 @@
       <c r="L275" s="2" t="s">
         <v>1039</v>
       </c>
-      <c r="M275" s="2" t="s">
+      <c r="M275" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -14967,7 +14955,7 @@
       <c r="G276" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H276" s="1" t="s">
+      <c r="H276" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J276" s="1" t="s">
@@ -15087,7 +15075,7 @@
       <c r="L279" s="2" t="s">
         <v>1058</v>
       </c>
-      <c r="M279" s="1" t="s">
+      <c r="M279" s="2" t="s">
         <v>1059</v>
       </c>
     </row>
@@ -15680,7 +15668,7 @@
       <c r="L295" s="2" t="s">
         <v>1109</v>
       </c>
-      <c r="M295" s="2" t="s">
+      <c r="M295" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -15715,7 +15703,7 @@
       <c r="L296" s="2" t="s">
         <v>1112</v>
       </c>
-      <c r="M296" s="1" t="s">
+      <c r="M296" s="2" t="s">
         <v>1113</v>
       </c>
     </row>
@@ -15916,7 +15904,7 @@
       <c r="G302" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H302" s="2" t="s">
+      <c r="H302" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J302" s="1" t="s">
@@ -15928,7 +15916,7 @@
       <c r="L302" s="2" t="s">
         <v>1131</v>
       </c>
-      <c r="M302" s="2" t="s">
+      <c r="M302" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -15954,7 +15942,7 @@
       <c r="G303" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H303" s="1" t="s">
+      <c r="H303" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J303" s="1" t="s">
@@ -15966,7 +15954,7 @@
       <c r="L303" s="2" t="s">
         <v>1135</v>
       </c>
-      <c r="M303" s="1" t="s">
+      <c r="M303" s="2" t="s">
         <v>1136</v>
       </c>
     </row>
@@ -16433,7 +16421,7 @@
       <c r="L316" s="2" t="s">
         <v>1176</v>
       </c>
-      <c r="M316" s="2" t="s">
+      <c r="M316" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -16506,7 +16494,7 @@
       <c r="L318" s="2" t="s">
         <v>1184</v>
       </c>
-      <c r="M318" s="1" t="s">
+      <c r="M318" s="2" t="s">
         <v>1185</v>
       </c>
     </row>
@@ -16558,7 +16546,7 @@
       <c r="D320">
         <v>2005</v>
       </c>
-      <c r="E320" s="2" t="s">
+      <c r="E320" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G320" s="1" t="s">
@@ -16576,7 +16564,7 @@
       <c r="L320" s="2" t="s">
         <v>1191</v>
       </c>
-      <c r="M320" s="2" t="s">
+      <c r="M320" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -16593,7 +16581,7 @@
       <c r="D321">
         <v>2007</v>
       </c>
-      <c r="E321" s="1" t="s">
+      <c r="E321" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G321" s="1" t="s">
@@ -16611,7 +16599,7 @@
       <c r="L321" s="2" t="s">
         <v>1195</v>
       </c>
-      <c r="M321" s="1" t="s">
+      <c r="M321" s="2" t="s">
         <v>1196</v>
       </c>
     </row>
@@ -16821,7 +16809,7 @@
       <c r="L327" s="2" t="s">
         <v>1214</v>
       </c>
-      <c r="M327" s="2" t="s">
+      <c r="M327" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -16856,7 +16844,7 @@
       <c r="L328" s="2" t="s">
         <v>1217</v>
       </c>
-      <c r="M328" s="1" t="s">
+      <c r="M328" s="2" t="s">
         <v>1218</v>
       </c>
     </row>
@@ -17168,7 +17156,7 @@
       <c r="D337">
         <v>2009</v>
       </c>
-      <c r="E337" s="2" t="s">
+      <c r="E337" s="1" t="s">
         <v>1221</v>
       </c>
       <c r="F337">
@@ -17189,7 +17177,7 @@
       <c r="L337" s="2" t="s">
         <v>1244</v>
       </c>
-      <c r="M337" s="2" t="s">
+      <c r="M337" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -17241,7 +17229,7 @@
       <c r="D339">
         <v>2009</v>
       </c>
-      <c r="E339" s="1" t="s">
+      <c r="E339" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G339" s="1" t="s">
@@ -17259,7 +17247,7 @@
       <c r="L339" s="2" t="s">
         <v>1251</v>
       </c>
-      <c r="M339" s="1" t="s">
+      <c r="M339" s="2" t="s">
         <v>1252</v>
       </c>
     </row>
@@ -17405,7 +17393,7 @@
       <c r="L343" s="2" t="s">
         <v>1265</v>
       </c>
-      <c r="M343" s="2" t="s">
+      <c r="M343" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -17440,7 +17428,7 @@
       <c r="L344" s="2" t="s">
         <v>1268</v>
       </c>
-      <c r="M344" s="1" t="s">
+      <c r="M344" s="2" t="s">
         <v>1269</v>
       </c>
     </row>
@@ -17475,7 +17463,7 @@
       <c r="L345" s="2" t="s">
         <v>1272</v>
       </c>
-      <c r="M345" s="2" t="s">
+      <c r="M345" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -17615,7 +17603,7 @@
       <c r="L349" s="2" t="s">
         <v>1287</v>
       </c>
-      <c r="M349" s="1" t="s">
+      <c r="M349" s="2" t="s">
         <v>1288</v>
       </c>
     </row>
@@ -17775,13 +17763,13 @@
       <c r="D354">
         <v>2010</v>
       </c>
-      <c r="E354" s="2" t="s">
+      <c r="E354" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G354" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H354" s="2" t="s">
+      <c r="H354" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J354" s="1" t="s">
@@ -17793,7 +17781,7 @@
       <c r="L354" s="2" t="s">
         <v>1301</v>
       </c>
-      <c r="M354" s="2" t="s">
+      <c r="M354" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -17810,13 +17798,13 @@
       <c r="D355">
         <v>2009</v>
       </c>
-      <c r="E355" s="1" t="s">
+      <c r="E355" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G355" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H355" s="1" t="s">
+      <c r="H355" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J355" s="1" t="s">
@@ -17828,7 +17816,7 @@
       <c r="L355" s="2" t="s">
         <v>1304</v>
       </c>
-      <c r="M355" s="1" t="s">
+      <c r="M355" s="2" t="s">
         <v>1305</v>
       </c>
     </row>
@@ -18395,7 +18383,7 @@
       <c r="L370" s="2" t="s">
         <v>1346</v>
       </c>
-      <c r="M370" s="2" t="s">
+      <c r="M370" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -18433,7 +18421,7 @@
       <c r="L371" s="2" t="s">
         <v>1350</v>
       </c>
-      <c r="M371" s="1" t="s">
+      <c r="M371" s="2" t="s">
         <v>1351</v>
       </c>
     </row>
@@ -18593,7 +18581,7 @@
       <c r="D376">
         <v>2011</v>
       </c>
-      <c r="E376" s="2" t="s">
+      <c r="E376" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G376" s="1" t="s">
@@ -18611,7 +18599,7 @@
       <c r="L376" s="2" t="s">
         <v>1366</v>
       </c>
-      <c r="M376" s="2" t="s">
+      <c r="M376" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -18628,7 +18616,7 @@
       <c r="D377">
         <v>2016</v>
       </c>
-      <c r="E377" s="1" t="s">
+      <c r="E377" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G377" s="1" t="s">
@@ -18649,7 +18637,7 @@
       <c r="L377" s="2" t="s">
         <v>1370</v>
       </c>
-      <c r="M377" s="1" t="s">
+      <c r="M377" s="2" t="s">
         <v>1371</v>
       </c>
     </row>
@@ -18666,7 +18654,7 @@
       <c r="D378">
         <v>2010</v>
       </c>
-      <c r="E378" s="2" t="s">
+      <c r="E378" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G378" s="1" t="s">
@@ -18684,7 +18672,7 @@
       <c r="L378" s="2" t="s">
         <v>1374</v>
       </c>
-      <c r="M378" s="2" t="s">
+      <c r="M378" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -18701,7 +18689,7 @@
       <c r="D379">
         <v>2009</v>
       </c>
-      <c r="E379" s="1" t="s">
+      <c r="E379" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G379" s="1" t="s">
@@ -18722,7 +18710,7 @@
       <c r="L379" s="2" t="s">
         <v>1377</v>
       </c>
-      <c r="M379" s="1" t="s">
+      <c r="M379" s="2" t="s">
         <v>1378</v>
       </c>
     </row>
@@ -18739,7 +18727,7 @@
       <c r="D380">
         <v>2009</v>
       </c>
-      <c r="E380" s="2" t="s">
+      <c r="E380" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G380" s="1" t="s">
@@ -18757,7 +18745,7 @@
       <c r="L380" s="2" t="s">
         <v>1381</v>
       </c>
-      <c r="M380" s="2" t="s">
+      <c r="M380" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -18844,7 +18832,7 @@
       <c r="D383">
         <v>2007</v>
       </c>
-      <c r="E383" s="1" t="s">
+      <c r="E383" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G383" s="1" t="s">
@@ -18879,7 +18867,7 @@
       <c r="D384">
         <v>2007</v>
       </c>
-      <c r="E384" s="2" t="s">
+      <c r="E384" s="1" t="s">
         <v>160</v>
       </c>
       <c r="F384">
@@ -18917,7 +18905,7 @@
       <c r="D385">
         <v>2012</v>
       </c>
-      <c r="E385" s="1" t="s">
+      <c r="E385" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G385" s="1" t="s">
@@ -18935,7 +18923,7 @@
       <c r="L385" s="2" t="s">
         <v>1402</v>
       </c>
-      <c r="M385" s="1" t="s">
+      <c r="M385" s="2" t="s">
         <v>1403</v>
       </c>
     </row>
@@ -19247,13 +19235,13 @@
       <c r="D394">
         <v>2011</v>
       </c>
-      <c r="E394" s="2" t="s">
+      <c r="E394" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G394" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H394" s="2" t="s">
+      <c r="H394" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J394" s="1" t="s">
@@ -19265,7 +19253,7 @@
       <c r="L394" s="2" t="s">
         <v>1431</v>
       </c>
-      <c r="M394" s="2" t="s">
+      <c r="M394" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -19352,13 +19340,13 @@
       <c r="D397">
         <v>2007</v>
       </c>
-      <c r="E397" s="1" t="s">
+      <c r="E397" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G397" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H397" s="1" t="s">
+      <c r="H397" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J397" s="1" t="s">
@@ -19370,7 +19358,7 @@
       <c r="L397" s="2" t="s">
         <v>1444</v>
       </c>
-      <c r="M397" s="1" t="s">
+      <c r="M397" s="2" t="s">
         <v>1445</v>
       </c>
     </row>
@@ -19682,7 +19670,7 @@
       <c r="D406">
         <v>2009</v>
       </c>
-      <c r="E406" s="2" t="s">
+      <c r="E406" s="1" t="s">
         <v>1472</v>
       </c>
       <c r="F406">
@@ -19703,7 +19691,7 @@
       <c r="L406" s="2" t="s">
         <v>1473</v>
       </c>
-      <c r="M406" s="2" t="s">
+      <c r="M406" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -19720,13 +19708,13 @@
       <c r="D407">
         <v>2008</v>
       </c>
-      <c r="E407" s="1" t="s">
+      <c r="E407" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G407" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H407" s="2" t="s">
+      <c r="H407" s="1" t="s">
         <v>141</v>
       </c>
       <c r="I407">
@@ -19764,7 +19752,7 @@
       <c r="G408" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H408" s="1" t="s">
+      <c r="H408" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J408" s="1" t="s">
@@ -19776,7 +19764,7 @@
       <c r="L408" s="2" t="s">
         <v>1480</v>
       </c>
-      <c r="M408" s="1" t="s">
+      <c r="M408" s="2" t="s">
         <v>1481</v>
       </c>
     </row>
@@ -19793,7 +19781,7 @@
       <c r="D409">
         <v>2009</v>
       </c>
-      <c r="E409" s="2" t="s">
+      <c r="E409" s="1" t="s">
         <v>1334</v>
       </c>
       <c r="F409">
@@ -19802,7 +19790,7 @@
       <c r="G409" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H409" s="2" t="s">
+      <c r="H409" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J409" s="1" t="s">
@@ -19814,7 +19802,7 @@
       <c r="L409" s="2" t="s">
         <v>1484</v>
       </c>
-      <c r="M409" s="2" t="s">
+      <c r="M409" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -19831,13 +19819,13 @@
       <c r="D410">
         <v>2009</v>
       </c>
-      <c r="E410" s="1" t="s">
+      <c r="E410" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G410" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H410" s="1" t="s">
+      <c r="H410" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J410" s="1" t="s">
@@ -19849,7 +19837,7 @@
       <c r="L410" s="2" t="s">
         <v>1487</v>
       </c>
-      <c r="M410" s="1" t="s">
+      <c r="M410" s="2" t="s">
         <v>1488</v>
       </c>
     </row>
@@ -19857,7 +19845,7 @@
       <c r="A411">
         <v>1963</v>
       </c>
-      <c r="B411" s="1" t="s">
+      <c r="B411" s="2" t="s">
         <v>1489</v>
       </c>
       <c r="C411" s="1" t="s">
@@ -19881,7 +19869,7 @@
       <c r="K411" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="L411" s="1" t="s">
+      <c r="L411" s="2" t="s">
         <v>1491</v>
       </c>
       <c r="M411" s="1" t="s">
@@ -19889,1052 +19877,1052 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M1" xr:uid="{745DC08D-AE8B-4C75-9243-B69FF27649B3}"/>
+  <autoFilter ref="A1:M1" xr:uid="{BBE45523-6C76-4660-A56E-2F9D5B1EE8BB}"/>
   <hyperlinks>
-    <hyperlink ref="B1" r:id="rId1" xr:uid="{C9C14143-0247-4B9D-8BDB-CA5D6E6F9A92}"/>
-    <hyperlink ref="E1" r:id="rId2" xr:uid="{D0F508BE-95CC-4D80-A0F7-6F0B3F107B65}"/>
-    <hyperlink ref="L1" r:id="rId3" xr:uid="{46D7236D-6263-4F09-9358-63D4AC2FE5D9}"/>
-    <hyperlink ref="M1" r:id="rId4" xr:uid="{2199B84E-1F78-4FB3-856D-B73A8F8210A7}"/>
-    <hyperlink ref="B2" r:id="rId5" xr:uid="{CCCD3E82-1EFE-4AFC-AF47-AB79D3FF0A18}"/>
-    <hyperlink ref="L2" r:id="rId6" xr:uid="{25CA67C1-B92D-4EB6-9419-C16DEF0931CC}"/>
-    <hyperlink ref="M2" r:id="rId7" xr:uid="{0E111863-F4D5-413E-962E-5FE4031316D1}"/>
-    <hyperlink ref="B3" r:id="rId8" xr:uid="{37A40087-AB22-47FB-8D23-A1032679E396}"/>
-    <hyperlink ref="L3" r:id="rId9" xr:uid="{417820F1-08C0-43CF-92A7-271D38C48041}"/>
-    <hyperlink ref="B4" r:id="rId10" xr:uid="{FF0D7F0A-B9E7-481F-9E60-E898F3BA34C2}"/>
-    <hyperlink ref="E4" r:id="rId11" xr:uid="{83296A01-EEA3-4310-BDB9-B13580B8E844}"/>
-    <hyperlink ref="L4" r:id="rId12" xr:uid="{DBECBA3B-DF29-4820-B086-79232312DAE8}"/>
-    <hyperlink ref="M4" r:id="rId13" xr:uid="{83EDA145-2A74-4ED2-9BB3-DEDCB7AE556B}"/>
-    <hyperlink ref="B5" r:id="rId14" xr:uid="{1F4FD076-8694-48D0-89F0-5550124D2EC9}"/>
-    <hyperlink ref="E5" r:id="rId15" xr:uid="{78523326-4EC8-4212-8B8D-8756AB41E35C}"/>
-    <hyperlink ref="H5" r:id="rId16" xr:uid="{C2C92D55-45A2-4983-8D96-6D82D85FE93C}"/>
-    <hyperlink ref="L5" r:id="rId17" xr:uid="{3980BA4C-821B-4F0D-82B0-4EA2EC4919D0}"/>
-    <hyperlink ref="M5" r:id="rId18" xr:uid="{80DB7200-1117-469A-9D60-8260E81D61F5}"/>
-    <hyperlink ref="B6" r:id="rId19" xr:uid="{46F0DA9A-B703-49D4-837C-2F6B590DC70D}"/>
-    <hyperlink ref="E6" r:id="rId20" xr:uid="{46513BC2-7FED-4AB2-88AC-8ED178DE06D6}"/>
-    <hyperlink ref="H6" r:id="rId21" xr:uid="{F2245913-2C4E-4A96-88ED-7A087E78E7D4}"/>
-    <hyperlink ref="L6" r:id="rId22" xr:uid="{ED0775BC-C3B8-499D-9545-2F92EBA2A721}"/>
-    <hyperlink ref="M6" r:id="rId23" xr:uid="{FCFD3180-BA67-4BE4-BFA0-8A0B9F6981DF}"/>
-    <hyperlink ref="B7" r:id="rId24" xr:uid="{2AB7EE4F-9A92-4AA4-9464-B23260AEA06E}"/>
-    <hyperlink ref="L7" r:id="rId25" xr:uid="{3BB5926E-DA6C-4749-ABA9-97A3CC746E03}"/>
-    <hyperlink ref="M7" r:id="rId26" xr:uid="{81014465-0CB3-491F-8B61-625B70D19AA8}"/>
-    <hyperlink ref="B8" r:id="rId27" xr:uid="{CE0B7E69-4B6B-4B4B-BAD0-EFA49A73B70A}"/>
-    <hyperlink ref="E8" r:id="rId28" xr:uid="{167747A3-11D1-47B9-B3E7-8AD39EA55B56}"/>
-    <hyperlink ref="L8" r:id="rId29" xr:uid="{5BD0B654-8CCE-4316-878A-D557892BD426}"/>
-    <hyperlink ref="M8" r:id="rId30" xr:uid="{AFABD157-F538-45B0-933F-202131903E4A}"/>
-    <hyperlink ref="B9" r:id="rId31" xr:uid="{00A949B4-DCB9-42F1-A608-1EE1B0562AF4}"/>
-    <hyperlink ref="L9" r:id="rId32" xr:uid="{7C32FD6A-C22F-4C4D-85A7-A36D2F5D22CA}"/>
-    <hyperlink ref="B10" r:id="rId33" xr:uid="{AD298E54-B14D-4695-8DF3-A9A21E512B51}"/>
-    <hyperlink ref="E10" r:id="rId34" xr:uid="{E6BA4601-4164-4085-9122-E3E63BF214CC}"/>
-    <hyperlink ref="L10" r:id="rId35" xr:uid="{D2207D9D-553F-4005-9E2D-747CA12BD859}"/>
-    <hyperlink ref="M10" r:id="rId36" xr:uid="{FE395AAB-221C-40EC-85FE-61FBB185BB47}"/>
-    <hyperlink ref="B11" r:id="rId37" xr:uid="{A79227A7-0C16-47BD-AD2B-814B29E9A02D}"/>
-    <hyperlink ref="L11" r:id="rId38" xr:uid="{A78C0A26-EC7D-40F2-8131-65C17EBD1070}"/>
-    <hyperlink ref="B12" r:id="rId39" xr:uid="{CDA7C7AA-2226-422C-81C6-F787E5034F81}"/>
-    <hyperlink ref="L12" r:id="rId40" xr:uid="{6353A950-4E4F-4A1C-B1E5-B9434CA66769}"/>
-    <hyperlink ref="B13" r:id="rId41" xr:uid="{158F132D-C952-49A3-A1FD-1496357D424B}"/>
-    <hyperlink ref="L13" r:id="rId42" xr:uid="{FD6568EE-249A-45D5-9F78-1733D408E567}"/>
-    <hyperlink ref="B14" r:id="rId43" xr:uid="{F221C616-FA11-4F44-A55C-2C1EE93EF369}"/>
-    <hyperlink ref="L14" r:id="rId44" xr:uid="{4160EA6D-254A-492F-A5D6-038EDFA356C0}"/>
-    <hyperlink ref="B15" r:id="rId45" xr:uid="{F5BE7F38-13E0-4023-A3AF-EC92FAB2CC10}"/>
-    <hyperlink ref="L15" r:id="rId46" xr:uid="{28928EC1-7C7C-4411-AB83-E6107DBB053A}"/>
-    <hyperlink ref="B16" r:id="rId47" xr:uid="{AD64D9F9-8803-4E11-8CEB-1C1DD0C7569C}"/>
-    <hyperlink ref="L16" r:id="rId48" xr:uid="{EBECB84C-A420-4368-9132-50BFD4DE3DE2}"/>
-    <hyperlink ref="B17" r:id="rId49" xr:uid="{A55EFB9C-B002-49F7-8248-6CB96D0F5D00}"/>
-    <hyperlink ref="L17" r:id="rId50" xr:uid="{1614DE5B-9FF3-4719-82DD-33A6DECF425A}"/>
-    <hyperlink ref="B18" r:id="rId51" xr:uid="{CB0BBF7A-7137-415A-B5B5-44A21C5043AE}"/>
-    <hyperlink ref="L18" r:id="rId52" xr:uid="{493FC858-2E7F-465F-94F8-E6CBD780A87A}"/>
-    <hyperlink ref="B19" r:id="rId53" xr:uid="{18BA2BFB-E6D5-4E5B-9533-2442385B3830}"/>
-    <hyperlink ref="L19" r:id="rId54" xr:uid="{E911C792-6939-4B36-B551-231045C53D2C}"/>
-    <hyperlink ref="M19" r:id="rId55" xr:uid="{A1F20C3A-1E53-423E-A8BF-53893836C608}"/>
-    <hyperlink ref="B20" r:id="rId56" xr:uid="{0294F07D-655A-4343-A017-02F4A07B7DC2}"/>
-    <hyperlink ref="H20" r:id="rId57" xr:uid="{430DC55D-B571-47B9-A2CA-29B53C019CA9}"/>
-    <hyperlink ref="L20" r:id="rId58" xr:uid="{662E56D7-B339-4E87-B8D4-DDEB9775C0A8}"/>
-    <hyperlink ref="M20" r:id="rId59" xr:uid="{6129AB72-36DF-409C-B4A6-5DC5F0607CED}"/>
-    <hyperlink ref="B21" r:id="rId60" xr:uid="{7598A5A1-5E3D-4C98-8AA8-3F0F5DC1255D}"/>
-    <hyperlink ref="L21" r:id="rId61" xr:uid="{95DEE957-B4F3-4AB8-9DF5-26DD5AA53E30}"/>
-    <hyperlink ref="B22" r:id="rId62" xr:uid="{EDE9DDA4-ED92-4330-B91B-D1682EC99380}"/>
-    <hyperlink ref="L22" r:id="rId63" xr:uid="{4DB97269-107C-44E4-9E40-EA91B7B94CC0}"/>
-    <hyperlink ref="B23" r:id="rId64" xr:uid="{B22B34CC-8949-4F80-9B7F-303DFCC4142C}"/>
-    <hyperlink ref="L23" r:id="rId65" xr:uid="{E0A13189-B682-4D80-9FF2-00934E550368}"/>
-    <hyperlink ref="B24" r:id="rId66" xr:uid="{50007E6D-1172-41E6-922A-9A3A0D33A945}"/>
-    <hyperlink ref="H24" r:id="rId67" xr:uid="{30915B0B-1457-48DA-8C2F-B528E5738D85}"/>
-    <hyperlink ref="L24" r:id="rId68" xr:uid="{727BD84B-DDF7-463F-AF0B-D55EE71D068A}"/>
-    <hyperlink ref="M24" r:id="rId69" xr:uid="{7A95324D-8E2B-4CB8-B1FC-AD278AD2A84F}"/>
-    <hyperlink ref="B25" r:id="rId70" xr:uid="{AE5C0B36-6D5E-4C9D-9D7B-4470A9FF4B30}"/>
-    <hyperlink ref="L25" r:id="rId71" xr:uid="{E38E2D3C-9E2F-4C4F-A4D9-4210D0A07B6B}"/>
-    <hyperlink ref="B26" r:id="rId72" xr:uid="{70DCF356-8D2E-409C-91CB-25B1ADEBF271}"/>
-    <hyperlink ref="E26" r:id="rId73" xr:uid="{32FC1D81-6DF9-4484-A8EF-375CA39BF591}"/>
-    <hyperlink ref="L26" r:id="rId74" xr:uid="{5A271B5C-C6E2-43C8-8E06-75D611C85BB2}"/>
-    <hyperlink ref="M26" r:id="rId75" xr:uid="{A2CFFD87-8524-4AA0-B96E-523EC4D908D7}"/>
-    <hyperlink ref="B27" r:id="rId76" xr:uid="{3657D698-813C-489E-905E-E14D5E930D12}"/>
-    <hyperlink ref="L27" r:id="rId77" xr:uid="{2DAA0AB9-E4AE-44B9-938E-DDE3CEBB2CF9}"/>
-    <hyperlink ref="B28" r:id="rId78" xr:uid="{67D375F6-81CB-43F2-A648-E64DEA193CB4}"/>
-    <hyperlink ref="E28" r:id="rId79" xr:uid="{E8F5A4B1-FCD2-4B19-B60F-9E2F7C4FA0D0}"/>
-    <hyperlink ref="L28" r:id="rId80" xr:uid="{A0932844-A4FC-493D-9D81-32750092E650}"/>
-    <hyperlink ref="M28" r:id="rId81" xr:uid="{76D29148-9D1E-4DA0-BDF8-CBFD0FD824D2}"/>
-    <hyperlink ref="B29" r:id="rId82" xr:uid="{00F8A225-8D6C-4942-A9A4-B0428D8A9296}"/>
-    <hyperlink ref="H29" r:id="rId83" xr:uid="{BD26EB32-5312-41F6-9A5D-9FA39AACFFC1}"/>
-    <hyperlink ref="L29" r:id="rId84" xr:uid="{FFFE6E98-926B-447B-9A8E-90942A0EE5BD}"/>
-    <hyperlink ref="M29" r:id="rId85" xr:uid="{5D0ADD5F-6153-4206-8A65-771F844E04B4}"/>
-    <hyperlink ref="B30" r:id="rId86" xr:uid="{A153B7A1-6E6A-4B61-B1EA-181701CDBF29}"/>
-    <hyperlink ref="L30" r:id="rId87" xr:uid="{502FC828-6D91-4C95-83A5-521D818CCF74}"/>
-    <hyperlink ref="B31" r:id="rId88" xr:uid="{CF185BE9-BA78-48FD-B38B-01A1D71FA350}"/>
-    <hyperlink ref="L31" r:id="rId89" xr:uid="{D7F82748-36D8-4531-975A-47BAB944AAB8}"/>
-    <hyperlink ref="B32" r:id="rId90" xr:uid="{F869B253-4556-4452-B940-EA6D7019A795}"/>
-    <hyperlink ref="L32" r:id="rId91" xr:uid="{D490D77C-755D-4EFC-A806-63068C4CC479}"/>
-    <hyperlink ref="M32" r:id="rId92" xr:uid="{775C074D-D92E-4FA3-8CC3-4E3005CF6AFC}"/>
-    <hyperlink ref="B33" r:id="rId93" xr:uid="{068C10FC-7A7E-40D9-9D2A-985E9F44F169}"/>
-    <hyperlink ref="E33" r:id="rId94" xr:uid="{80B04818-83CA-43E2-99EA-4FD3FE684C9C}"/>
-    <hyperlink ref="L33" r:id="rId95" xr:uid="{082FE4E0-C4C3-45C1-9F46-E16D73A181D9}"/>
-    <hyperlink ref="M33" r:id="rId96" xr:uid="{54A3C53F-44F2-416F-ABA4-6D9E2875184E}"/>
-    <hyperlink ref="B34" r:id="rId97" xr:uid="{4C8B9DB0-880A-4067-9B9B-3EDEC69B5AAE}"/>
-    <hyperlink ref="E34" r:id="rId98" xr:uid="{E5C5582E-D81E-4D55-8270-FCA9471D0A03}"/>
-    <hyperlink ref="H34" r:id="rId99" xr:uid="{8171340C-9C64-4D69-A1B3-F38F0FEDF29F}"/>
-    <hyperlink ref="L34" r:id="rId100" xr:uid="{EC513D00-66C9-4CC9-BA3E-D3A406805409}"/>
-    <hyperlink ref="M34" r:id="rId101" xr:uid="{50A9EB18-6C7D-4328-86DB-4766C4126FAE}"/>
-    <hyperlink ref="B35" r:id="rId102" xr:uid="{626322A2-A213-4460-AA4C-59627584A017}"/>
-    <hyperlink ref="L35" r:id="rId103" xr:uid="{57B85D0A-AE19-47E9-BCE6-F7754F412209}"/>
-    <hyperlink ref="B36" r:id="rId104" xr:uid="{45D03503-176B-4939-AFF9-BC92E6DF2DFB}"/>
-    <hyperlink ref="L36" r:id="rId105" xr:uid="{BCE2FB66-E991-4D26-9D32-2E5EA4CC5327}"/>
-    <hyperlink ref="B37" r:id="rId106" xr:uid="{D04FB519-4D98-40B6-BA39-EE96B10F9DF0}"/>
-    <hyperlink ref="L37" r:id="rId107" xr:uid="{B60B7E7A-3F83-4CF8-9395-17848BCB61E1}"/>
-    <hyperlink ref="M37" r:id="rId108" xr:uid="{2BA59781-BF3A-4458-8A5B-9CC1E94D9840}"/>
-    <hyperlink ref="B38" r:id="rId109" xr:uid="{50D7E25C-1FAF-4E9E-A9CE-E605247C10A3}"/>
-    <hyperlink ref="L38" r:id="rId110" xr:uid="{085C9B07-B9F4-4C91-B5FC-8CBEBD44FB02}"/>
-    <hyperlink ref="B39" r:id="rId111" xr:uid="{2535F753-A834-47D1-8FF7-173396A21DB1}"/>
-    <hyperlink ref="L39" r:id="rId112" xr:uid="{A90CEEB0-8F0B-4B7B-898A-C43D93354530}"/>
-    <hyperlink ref="M39" r:id="rId113" xr:uid="{848F34D2-319C-466D-B6B4-F8B440246789}"/>
-    <hyperlink ref="B40" r:id="rId114" xr:uid="{836ED3A2-2762-4811-9733-730DACC73A5C}"/>
-    <hyperlink ref="L40" r:id="rId115" xr:uid="{190F799A-FD1C-4122-9009-312718516A30}"/>
-    <hyperlink ref="B41" r:id="rId116" xr:uid="{502BD352-121C-467D-8D80-CFDA52EAAFB8}"/>
-    <hyperlink ref="E41" r:id="rId117" xr:uid="{F4E68FEE-2009-496B-96BF-463C3BBE9350}"/>
-    <hyperlink ref="L41" r:id="rId118" xr:uid="{E4CA1FE2-5D02-4A0E-B73A-48F259FBF6AA}"/>
-    <hyperlink ref="M41" r:id="rId119" xr:uid="{20FF3987-4F0F-47AA-B4F5-9FC25DC8493F}"/>
-    <hyperlink ref="B42" r:id="rId120" xr:uid="{B23D69F1-9F4F-4DBA-92FE-FB3B69F2D957}"/>
-    <hyperlink ref="L42" r:id="rId121" xr:uid="{4E2B27C3-57CD-4BE8-A4B1-DD1F2E1D224F}"/>
-    <hyperlink ref="B43" r:id="rId122" xr:uid="{4ADF9441-6F49-49F3-8F37-C9854D2EC7C3}"/>
-    <hyperlink ref="L43" r:id="rId123" xr:uid="{C8C1E724-3325-4D3E-A58F-4F53E29CE22A}"/>
-    <hyperlink ref="M43" r:id="rId124" xr:uid="{D7C299FF-BF60-4651-847A-DB7AD8F06961}"/>
-    <hyperlink ref="B44" r:id="rId125" xr:uid="{B9F7E903-77B8-47D4-BD94-6ED7A0780DBD}"/>
-    <hyperlink ref="L44" r:id="rId126" xr:uid="{4E9A2C98-D518-463E-A6D0-50AF63575FFD}"/>
-    <hyperlink ref="M44" r:id="rId127" xr:uid="{64770562-9BC3-46FF-9E5A-25C5BEA28CC9}"/>
-    <hyperlink ref="B45" r:id="rId128" xr:uid="{ECC1F8CA-FBE7-438B-875B-31692A21789E}"/>
-    <hyperlink ref="L45" r:id="rId129" xr:uid="{36AEE80B-5B5A-4458-A54D-B80EEA5297A4}"/>
-    <hyperlink ref="B46" r:id="rId130" xr:uid="{E00DEBEF-3226-441C-95AC-356E4FD5DE73}"/>
-    <hyperlink ref="L46" r:id="rId131" xr:uid="{A1682F66-238F-4F56-83AA-5A376ED0E6E9}"/>
-    <hyperlink ref="B47" r:id="rId132" xr:uid="{ED2B8A76-4A08-4ED9-A9A1-0519E1C7A4D1}"/>
-    <hyperlink ref="E47" r:id="rId133" xr:uid="{871801D9-2FAB-4D46-A512-9451AC0D0249}"/>
-    <hyperlink ref="L47" r:id="rId134" xr:uid="{5A2FC794-1566-44AE-B471-D7FB23831804}"/>
-    <hyperlink ref="M47" r:id="rId135" xr:uid="{8B12C211-7A68-4A46-ABBD-7E8B4E6B9741}"/>
-    <hyperlink ref="B48" r:id="rId136" xr:uid="{347B17F9-B485-4D79-ADE1-A49F0F8D1E5F}"/>
-    <hyperlink ref="E48" r:id="rId137" xr:uid="{E1B6C454-AE60-47FD-877B-110F0B5F1E03}"/>
-    <hyperlink ref="L48" r:id="rId138" xr:uid="{6C726C7F-50AC-4687-8EA7-09B2BA134DE1}"/>
-    <hyperlink ref="M48" r:id="rId139" xr:uid="{5DFE3BFB-7D2E-4513-ACCE-6A179293D46E}"/>
-    <hyperlink ref="B49" r:id="rId140" xr:uid="{70AB73EE-7BF7-4459-912E-A48D2116733F}"/>
-    <hyperlink ref="L49" r:id="rId141" xr:uid="{1EC7573B-3B6A-40B3-B245-D3FDC031AF13}"/>
-    <hyperlink ref="M49" r:id="rId142" xr:uid="{880D5F39-FF50-4F75-AC16-8814516727FF}"/>
-    <hyperlink ref="B50" r:id="rId143" xr:uid="{DA146018-01A5-4F6A-8A23-43F7074B6C68}"/>
-    <hyperlink ref="L50" r:id="rId144" xr:uid="{2B7E484F-FF71-47DB-ACC7-E1EBD0A87944}"/>
-    <hyperlink ref="B51" r:id="rId145" xr:uid="{4FB99745-5698-45A8-A015-ED0A4639BAFD}"/>
-    <hyperlink ref="L51" r:id="rId146" xr:uid="{C6868AB7-9C7E-4039-9BEA-5CCF03B8680C}"/>
-    <hyperlink ref="B52" r:id="rId147" xr:uid="{B6960A06-93AF-4F10-8B9E-327B0228DCD5}"/>
-    <hyperlink ref="L52" r:id="rId148" xr:uid="{1C785B36-4359-4067-82B1-A9C1F5713C85}"/>
-    <hyperlink ref="B53" r:id="rId149" xr:uid="{02B51947-FEC3-46AA-9883-25694C4D3334}"/>
-    <hyperlink ref="L53" r:id="rId150" xr:uid="{85FE2568-4B38-43F5-9147-2F6BDCFB946A}"/>
-    <hyperlink ref="B54" r:id="rId151" xr:uid="{6EAA93A5-16EA-44AB-A69E-E8F7236B16F2}"/>
-    <hyperlink ref="L54" r:id="rId152" xr:uid="{0BE7A3D5-47A6-4486-8380-8C230B1A0FCD}"/>
-    <hyperlink ref="B55" r:id="rId153" xr:uid="{7AC26CE5-CAEC-4D6F-850F-B33C362C20C0}"/>
-    <hyperlink ref="L55" r:id="rId154" xr:uid="{52B413D2-2C9B-4134-911A-EA2C0B81A9C0}"/>
-    <hyperlink ref="M55" r:id="rId155" xr:uid="{27AF1946-7E57-4AA4-979C-D8F3FCCDB5CB}"/>
-    <hyperlink ref="B56" r:id="rId156" xr:uid="{796F65E7-6354-4A64-B055-6AEE84EA3841}"/>
-    <hyperlink ref="E56" r:id="rId157" xr:uid="{DEDAB2B1-8C85-40A4-B0C1-81B6DD3001E0}"/>
-    <hyperlink ref="L56" r:id="rId158" xr:uid="{53672236-F7D5-43D8-B9A1-07A882885DEC}"/>
-    <hyperlink ref="M56" r:id="rId159" xr:uid="{D4F7F641-681F-40F6-A19F-1274CED3587A}"/>
-    <hyperlink ref="B57" r:id="rId160" xr:uid="{003903C8-D2D2-43D3-AA25-C6D13376920D}"/>
-    <hyperlink ref="L57" r:id="rId161" xr:uid="{047E5BF7-A31B-4949-AFDD-13DD1DD1FB0D}"/>
-    <hyperlink ref="M57" r:id="rId162" xr:uid="{A6EAC2FE-C82C-406C-8C5B-DE8B10424E8E}"/>
-    <hyperlink ref="B58" r:id="rId163" xr:uid="{A41330D8-D536-4BA0-A210-55C792C2E298}"/>
-    <hyperlink ref="L58" r:id="rId164" xr:uid="{B217A759-A246-41EB-8CA2-F9DF17DA4B93}"/>
-    <hyperlink ref="B59" r:id="rId165" xr:uid="{ABBCABD2-8EA4-4723-8223-74584487B63A}"/>
-    <hyperlink ref="E59" r:id="rId166" xr:uid="{73B4B400-B97A-476B-AC3F-F6027249038E}"/>
-    <hyperlink ref="L59" r:id="rId167" xr:uid="{87EC17C6-EDC5-4F1C-948A-F40737E9EB35}"/>
-    <hyperlink ref="M59" r:id="rId168" xr:uid="{D225074D-C2BF-4D37-838F-54BEE0E37F4E}"/>
-    <hyperlink ref="B60" r:id="rId169" xr:uid="{AE2EC83D-A648-4341-A2DD-6B6D098F3710}"/>
-    <hyperlink ref="E60" r:id="rId170" xr:uid="{2A1A9837-00D8-4CA7-A1AC-FD0C55722C8F}"/>
-    <hyperlink ref="H60" r:id="rId171" xr:uid="{E6DFFDE8-FE5B-4C70-ADA3-CB9604B69E8A}"/>
-    <hyperlink ref="L60" r:id="rId172" xr:uid="{B95BD397-62E0-4462-9C7E-CBCE20146F08}"/>
-    <hyperlink ref="M60" r:id="rId173" xr:uid="{225C73E2-4284-482E-844E-D57AB2367D3A}"/>
-    <hyperlink ref="B61" r:id="rId174" xr:uid="{0DDC700F-FCE0-4116-B1EC-7D893F6BCD41}"/>
-    <hyperlink ref="L61" r:id="rId175" xr:uid="{9AD277FF-2133-48D2-BBD5-E6A5BCD0EA0D}"/>
-    <hyperlink ref="B62" r:id="rId176" xr:uid="{E1CCE4E6-9A0D-4E58-AE00-4112421EB931}"/>
-    <hyperlink ref="L62" r:id="rId177" xr:uid="{3169F3D1-F72B-44E9-B9BC-5783E5D6A1ED}"/>
-    <hyperlink ref="B63" r:id="rId178" xr:uid="{D4718AC5-447A-4B27-883A-EE60A52BCD9B}"/>
-    <hyperlink ref="L63" r:id="rId179" xr:uid="{0A6344EC-A028-485B-9C56-9AD82D0A867E}"/>
-    <hyperlink ref="B64" r:id="rId180" xr:uid="{CF13DA05-D7EA-45F3-84CA-3873F3E83782}"/>
-    <hyperlink ref="E64" r:id="rId181" xr:uid="{F58893CE-2F31-435F-8020-70A6764C28E0}"/>
-    <hyperlink ref="L64" r:id="rId182" xr:uid="{DD87077A-861D-465D-97CD-26E97D93C177}"/>
-    <hyperlink ref="M64" r:id="rId183" xr:uid="{1D5B62E4-A7A2-493D-8E2C-988B7CFC9EFB}"/>
-    <hyperlink ref="B65" r:id="rId184" xr:uid="{BC376CFA-3682-4C5E-AA0E-237B7DA05307}"/>
-    <hyperlink ref="L65" r:id="rId185" xr:uid="{1A869C3C-9428-47F5-AC85-C798784AE4FC}"/>
-    <hyperlink ref="B66" r:id="rId186" xr:uid="{7A39D466-56CA-4ADF-AFEC-9191F5B4AD44}"/>
-    <hyperlink ref="L66" r:id="rId187" xr:uid="{E98D7016-AA72-4E84-996F-881EE6297EAA}"/>
-    <hyperlink ref="B67" r:id="rId188" xr:uid="{576EE0A1-48E5-46E9-BAF1-98D595240CE9}"/>
-    <hyperlink ref="L67" r:id="rId189" xr:uid="{48B2E3CB-7498-42D8-84E9-83AA0A334D1B}"/>
-    <hyperlink ref="B68" r:id="rId190" xr:uid="{4E9DF589-DE68-4CFF-870E-34A90290CFF2}"/>
-    <hyperlink ref="L68" r:id="rId191" xr:uid="{BBEC19E0-387F-4B76-BF87-6775EC662708}"/>
-    <hyperlink ref="B69" r:id="rId192" xr:uid="{23638DA0-B9D2-4484-A63D-571A8D46B6A9}"/>
-    <hyperlink ref="L69" r:id="rId193" xr:uid="{50533C8C-B334-4A2C-BD8F-9B1B69AF5FCA}"/>
-    <hyperlink ref="B70" r:id="rId194" xr:uid="{C5C519C7-F566-4907-986D-665D0A5C1594}"/>
-    <hyperlink ref="L70" r:id="rId195" xr:uid="{05F7973E-84B0-4B77-905F-4D400C234A6D}"/>
-    <hyperlink ref="B71" r:id="rId196" xr:uid="{790E3A8E-3A8E-4249-94EA-281317346AEE}"/>
-    <hyperlink ref="L71" r:id="rId197" xr:uid="{0D268E6F-E7D7-41F2-96E1-6F4A8601E7AF}"/>
-    <hyperlink ref="B72" r:id="rId198" xr:uid="{955A65AA-4C4B-4FFC-A91D-3BCF3319F4F4}"/>
-    <hyperlink ref="L72" r:id="rId199" xr:uid="{FDD2EF1D-F4E6-47E7-804E-1A5E235E61C7}"/>
-    <hyperlink ref="B73" r:id="rId200" xr:uid="{40098B95-6AB8-4FC2-8191-AAEC492D013C}"/>
-    <hyperlink ref="L73" r:id="rId201" xr:uid="{D3A9A788-B621-4D14-B6F8-19F95237BD43}"/>
-    <hyperlink ref="B74" r:id="rId202" xr:uid="{98FD7EE9-1D03-4C65-AF92-4F17EEAAFED2}"/>
-    <hyperlink ref="L74" r:id="rId203" xr:uid="{BA3A50A4-790E-415A-8628-55BE77854874}"/>
-    <hyperlink ref="B75" r:id="rId204" xr:uid="{32EA5D28-DEF6-4FA2-8F39-4F886D250142}"/>
-    <hyperlink ref="L75" r:id="rId205" xr:uid="{6FA9D464-68CA-4A49-9D0D-3AA9691E9002}"/>
-    <hyperlink ref="B76" r:id="rId206" xr:uid="{0CA47F5A-2FCF-4629-82DD-D056FC4ACBFE}"/>
-    <hyperlink ref="L76" r:id="rId207" xr:uid="{7FA88714-5F4F-476D-8BD2-41D34F5408B5}"/>
-    <hyperlink ref="M76" r:id="rId208" xr:uid="{C8AA4697-FB23-41AF-895C-48416DF0B5EB}"/>
-    <hyperlink ref="B77" r:id="rId209" xr:uid="{285B433E-6952-49D0-92E1-99D5090F02FE}"/>
-    <hyperlink ref="L77" r:id="rId210" xr:uid="{259441CC-43CF-4721-95DA-B98B9522FFA2}"/>
-    <hyperlink ref="B78" r:id="rId211" xr:uid="{0F62FC1A-D81E-4724-9AF8-72095CDB0335}"/>
-    <hyperlink ref="L78" r:id="rId212" xr:uid="{4A98CE5E-7C17-4D09-BD13-D9BF70A8F147}"/>
-    <hyperlink ref="B79" r:id="rId213" xr:uid="{C93C1862-2866-49CE-BED1-ED5159E94FE9}"/>
-    <hyperlink ref="L79" r:id="rId214" xr:uid="{7393C2A4-0852-401A-9198-4FC0825FF652}"/>
-    <hyperlink ref="B80" r:id="rId215" xr:uid="{9408721E-ADFB-433A-9D07-8DBF0B33E4D5}"/>
-    <hyperlink ref="L80" r:id="rId216" xr:uid="{84E21384-34EB-44C2-8880-893B06A12C70}"/>
-    <hyperlink ref="B81" r:id="rId217" xr:uid="{FEB7D3EF-CAF0-4F50-910D-575A0B745FD1}"/>
-    <hyperlink ref="L81" r:id="rId218" xr:uid="{FCF68482-75F4-44D3-B9E9-082464711FD9}"/>
-    <hyperlink ref="B82" r:id="rId219" xr:uid="{CF64D1F3-00BD-45A2-B3EF-90D89F8E5E54}"/>
-    <hyperlink ref="E82" r:id="rId220" xr:uid="{E496D6CF-AAEB-4B7D-B1DE-462D7AF37D07}"/>
-    <hyperlink ref="L82" r:id="rId221" xr:uid="{052448D1-BD8F-4E32-89ED-7D3F0197303F}"/>
-    <hyperlink ref="M82" r:id="rId222" xr:uid="{F6F16616-020A-473C-8F58-DA60A9446BFA}"/>
-    <hyperlink ref="B83" r:id="rId223" xr:uid="{559F900C-296F-4E3C-A81F-917B1B0C0477}"/>
-    <hyperlink ref="E83" r:id="rId224" xr:uid="{12ACF4CB-4623-4DDB-AB25-D6775F40228D}"/>
-    <hyperlink ref="L83" r:id="rId225" xr:uid="{0FD6FA86-7C2C-4E76-9784-12B259D0DD8E}"/>
-    <hyperlink ref="M83" r:id="rId226" xr:uid="{70A9510B-D1AC-4D2E-9E85-3C243CC572DD}"/>
-    <hyperlink ref="B84" r:id="rId227" xr:uid="{FBD62BC5-710F-4E45-A9B5-0472AF2FD999}"/>
-    <hyperlink ref="L84" r:id="rId228" xr:uid="{E684BA2F-E242-4C1F-8231-226961399BC6}"/>
-    <hyperlink ref="B85" r:id="rId229" xr:uid="{DCEAC20B-3F61-4BEE-B02B-858757F24EBD}"/>
-    <hyperlink ref="L85" r:id="rId230" xr:uid="{C50A02AD-481D-42A4-BEC6-0D1A6E2118CE}"/>
-    <hyperlink ref="B86" r:id="rId231" xr:uid="{E661FAD6-203D-476A-AAC3-2EA272E35688}"/>
-    <hyperlink ref="L86" r:id="rId232" xr:uid="{A622F3C1-0497-4DBB-9031-9C0527C05F8A}"/>
-    <hyperlink ref="B87" r:id="rId233" xr:uid="{7ED22BC1-38D4-404C-A58E-C9A4CEA83F85}"/>
-    <hyperlink ref="L87" r:id="rId234" xr:uid="{4F7183E2-5FE5-49E7-AF4A-EC10185FE37D}"/>
-    <hyperlink ref="B88" r:id="rId235" xr:uid="{39D8409A-861E-427F-AD2C-60C5054F83AD}"/>
-    <hyperlink ref="L88" r:id="rId236" xr:uid="{4DEBC4B0-2F36-4A5B-A1AA-D53503E58BCB}"/>
-    <hyperlink ref="B89" r:id="rId237" xr:uid="{B5EA4FBA-2C93-404F-8B93-78D518E2F456}"/>
-    <hyperlink ref="L89" r:id="rId238" xr:uid="{FB572C23-317A-496E-AF6A-E24CAEBD56BC}"/>
-    <hyperlink ref="M89" r:id="rId239" xr:uid="{33F56599-5FF5-4524-806A-02609F15C08C}"/>
-    <hyperlink ref="B90" r:id="rId240" xr:uid="{5EEAE30C-F631-41BD-AC5A-EEB3B47F7AAE}"/>
-    <hyperlink ref="L90" r:id="rId241" xr:uid="{BD58DA74-1BAE-449F-8EFA-1F33B737D39F}"/>
-    <hyperlink ref="M90" r:id="rId242" xr:uid="{36EEA4E3-539D-4422-B3AD-B8172B906168}"/>
-    <hyperlink ref="B91" r:id="rId243" xr:uid="{ECA44C41-6700-4AB5-9D32-3AC60F2E04CB}"/>
-    <hyperlink ref="H91" r:id="rId244" xr:uid="{CDC8CEE4-F42E-4A92-B1BA-BCC23F964A3C}"/>
-    <hyperlink ref="L91" r:id="rId245" xr:uid="{10E938E1-6869-4718-92F8-B3BD8BE8813C}"/>
-    <hyperlink ref="M91" r:id="rId246" xr:uid="{0B36D963-61A0-4899-8034-DF83E5C1AAC5}"/>
-    <hyperlink ref="B92" r:id="rId247" xr:uid="{00939B24-BB4D-40AE-A2E4-2B3F6289BFEA}"/>
-    <hyperlink ref="L92" r:id="rId248" xr:uid="{365892CA-36F5-47EC-8E11-85E0A4F3448C}"/>
-    <hyperlink ref="B93" r:id="rId249" xr:uid="{0D2DB9EF-0745-425B-B6DB-061019A09F8B}"/>
-    <hyperlink ref="H93" r:id="rId250" xr:uid="{5AA145FA-D8D9-4E36-A5BC-95D1D6028485}"/>
-    <hyperlink ref="L93" r:id="rId251" xr:uid="{423AB6F7-1572-4EFE-B580-CC0AF15B448F}"/>
-    <hyperlink ref="M93" r:id="rId252" xr:uid="{F573A521-FF3A-4199-83BF-21839404C8F6}"/>
-    <hyperlink ref="B94" r:id="rId253" xr:uid="{07D604C4-13B0-407C-88E1-77AA9DD285E6}"/>
-    <hyperlink ref="E94" r:id="rId254" xr:uid="{DDCEF32B-3D20-44A4-B469-2BD51A1C2D0B}"/>
-    <hyperlink ref="L94" r:id="rId255" xr:uid="{B7CF8A73-8385-412A-8326-A95637AE64CF}"/>
-    <hyperlink ref="M94" r:id="rId256" xr:uid="{2A82CAFD-75F7-4CB6-B1CB-002B05AFD999}"/>
-    <hyperlink ref="B95" r:id="rId257" xr:uid="{6FB6A9C0-B971-4E13-9020-C46C0BAF9368}"/>
-    <hyperlink ref="L95" r:id="rId258" xr:uid="{C8F18531-AF72-4D1A-B76C-A5197F0DD567}"/>
-    <hyperlink ref="B96" r:id="rId259" xr:uid="{5F9DA90F-B92E-4347-9870-72D71983D9E7}"/>
-    <hyperlink ref="L96" r:id="rId260" xr:uid="{21EC90F1-E863-48A7-A0FA-B2DC0225819B}"/>
-    <hyperlink ref="B97" r:id="rId261" xr:uid="{F612BAED-D501-4F82-B5E8-E266ACCA969C}"/>
-    <hyperlink ref="L97" r:id="rId262" xr:uid="{3B86D692-B32C-41F5-A141-E2870BE601FD}"/>
-    <hyperlink ref="B98" r:id="rId263" xr:uid="{69FFB2AA-5897-40ED-A251-7D9EAA3D5AD4}"/>
-    <hyperlink ref="E98" r:id="rId264" xr:uid="{5A18D035-0101-4CCA-A710-A8CA3FB5A888}"/>
-    <hyperlink ref="L98" r:id="rId265" xr:uid="{52165E19-2B7D-4E7C-8EE0-9B7B147DFD2E}"/>
-    <hyperlink ref="M98" r:id="rId266" xr:uid="{AF45CD71-49BD-414C-A610-FFE7ADCC45FB}"/>
-    <hyperlink ref="B99" r:id="rId267" xr:uid="{4631A115-3AFB-4DBB-95F3-764EC19459D8}"/>
-    <hyperlink ref="L99" r:id="rId268" xr:uid="{CFA204B9-376A-4866-B6C0-1DD5537DD122}"/>
-    <hyperlink ref="B100" r:id="rId269" xr:uid="{4F5B7434-DC36-43BB-A246-EB590DDAA331}"/>
-    <hyperlink ref="L100" r:id="rId270" xr:uid="{0258E799-5731-4E3A-8558-2AE7BC8C75BC}"/>
-    <hyperlink ref="B101" r:id="rId271" xr:uid="{92E0334F-5D6C-4022-8A12-4989147727C9}"/>
-    <hyperlink ref="E101" r:id="rId272" xr:uid="{4846B354-A106-4E71-A5D8-B19933ED82F8}"/>
-    <hyperlink ref="L101" r:id="rId273" xr:uid="{9F474963-8EC5-4D56-A7A5-57B147369F60}"/>
-    <hyperlink ref="M101" r:id="rId274" xr:uid="{4EC6719A-2CAB-4FC2-A59F-0EE9C831ABF2}"/>
-    <hyperlink ref="B102" r:id="rId275" xr:uid="{BE75D3E2-B73F-46EB-BE8B-6C83F09875E8}"/>
-    <hyperlink ref="L102" r:id="rId276" xr:uid="{032EAF35-82E4-49F9-9297-968580F245D3}"/>
-    <hyperlink ref="M102" r:id="rId277" xr:uid="{6E1722A8-B71E-4707-BEF7-0F597046059B}"/>
-    <hyperlink ref="B103" r:id="rId278" xr:uid="{6BE0F2AF-60A5-467E-8900-10BE095B4A4E}"/>
-    <hyperlink ref="L103" r:id="rId279" xr:uid="{F3C008B6-80F8-4A9E-AF5E-2044724FA3FC}"/>
-    <hyperlink ref="B104" r:id="rId280" xr:uid="{CD280032-9648-434D-8C88-2B41802A1821}"/>
-    <hyperlink ref="L104" r:id="rId281" xr:uid="{8BEAD859-4D72-49C5-B1D6-AEE4B740EB3B}"/>
-    <hyperlink ref="B105" r:id="rId282" xr:uid="{69A95AFA-039D-4CE6-9BDA-9AA82A55F70A}"/>
-    <hyperlink ref="L105" r:id="rId283" xr:uid="{36AC8DEE-763C-408C-9475-7BB01FF2F5DB}"/>
-    <hyperlink ref="B106" r:id="rId284" xr:uid="{B865777E-FA02-4879-8C43-06A2FD88FE10}"/>
-    <hyperlink ref="L106" r:id="rId285" xr:uid="{B06DADFF-029C-4946-86A6-F6EB69B5928D}"/>
-    <hyperlink ref="M106" r:id="rId286" xr:uid="{CBE58B53-4351-4ECA-9E12-CEFC44D68EF8}"/>
-    <hyperlink ref="B107" r:id="rId287" xr:uid="{8DFB8162-4C20-4611-AB94-08B69F6C8F91}"/>
-    <hyperlink ref="E107" r:id="rId288" xr:uid="{F7D4EEC8-7BA7-4AA5-8583-95B2C8EB116E}"/>
-    <hyperlink ref="L107" r:id="rId289" xr:uid="{109D0E6B-E793-45B9-976D-4C11A5F3C0AE}"/>
-    <hyperlink ref="M107" r:id="rId290" xr:uid="{D676892F-C0C4-4EA8-B33C-5B9E46D5AFC7}"/>
-    <hyperlink ref="B108" r:id="rId291" xr:uid="{61888E2A-8A8E-416E-8B72-365278080765}"/>
-    <hyperlink ref="H108" r:id="rId292" xr:uid="{960EC7A6-F35D-4375-87A1-5C8E14AACFE7}"/>
-    <hyperlink ref="L108" r:id="rId293" xr:uid="{1FAEA921-C157-45E2-93A2-1217B2944800}"/>
-    <hyperlink ref="M108" r:id="rId294" xr:uid="{1EFD5D0E-DF47-4963-95AA-067E8356B3F4}"/>
-    <hyperlink ref="B109" r:id="rId295" xr:uid="{3C2FD3F3-C77E-4FCD-ADFA-D1A715867874}"/>
-    <hyperlink ref="E109" r:id="rId296" xr:uid="{4EEFF20F-7F2D-4E46-8837-A74BB5D9637B}"/>
-    <hyperlink ref="L109" r:id="rId297" xr:uid="{777E8CB5-562C-47F8-B9B3-1DBE724F1DE6}"/>
-    <hyperlink ref="M109" r:id="rId298" xr:uid="{6E13E913-7A9A-4953-9114-C5815010EB9F}"/>
-    <hyperlink ref="B110" r:id="rId299" xr:uid="{32A74329-3399-412E-9323-1997EB8FF5F4}"/>
-    <hyperlink ref="L110" r:id="rId300" xr:uid="{6F7AE1E1-FB0D-456D-867D-2A60005980A2}"/>
-    <hyperlink ref="B111" r:id="rId301" xr:uid="{C2C25C7C-F801-49D9-9F21-25E808647683}"/>
-    <hyperlink ref="L111" r:id="rId302" xr:uid="{9C30164F-B36D-41EB-B6AF-0BD5885D30B3}"/>
-    <hyperlink ref="M111" r:id="rId303" xr:uid="{56FAC98A-C129-4838-BEBB-D13B331C0E87}"/>
-    <hyperlink ref="B112" r:id="rId304" xr:uid="{A2CA43BC-473A-4064-943C-70419781C5F0}"/>
-    <hyperlink ref="L112" r:id="rId305" xr:uid="{F9036E76-F9F6-4039-B1F8-8B2C4043353D}"/>
-    <hyperlink ref="B113" r:id="rId306" xr:uid="{E0F18F44-DFF5-4A8A-93E0-B6364FA764F5}"/>
-    <hyperlink ref="L113" r:id="rId307" xr:uid="{1ACD26BB-66B1-436A-9741-F1126A0D4C3B}"/>
-    <hyperlink ref="M113" r:id="rId308" xr:uid="{2D312D9F-33CD-4748-BC19-73AAE31D430F}"/>
-    <hyperlink ref="B114" r:id="rId309" xr:uid="{39B857F7-394A-4F3E-8B93-058D09D11089}"/>
-    <hyperlink ref="L114" r:id="rId310" xr:uid="{7FF6925E-95EC-4B7E-BA0C-467A0C2E5820}"/>
-    <hyperlink ref="B115" r:id="rId311" xr:uid="{4B894487-6045-43FF-A584-B7EA92F609B3}"/>
-    <hyperlink ref="L115" r:id="rId312" xr:uid="{13E4912F-80B7-482F-9B8B-683DBD681440}"/>
-    <hyperlink ref="B116" r:id="rId313" xr:uid="{9047B50E-F35F-452E-A943-0D4D99296C75}"/>
-    <hyperlink ref="L116" r:id="rId314" xr:uid="{6F663D6D-BF9C-4787-82F8-7918345F28EF}"/>
-    <hyperlink ref="B117" r:id="rId315" xr:uid="{02334602-28B2-4EAE-82E5-AB0FD71CF48D}"/>
-    <hyperlink ref="L117" r:id="rId316" xr:uid="{1CF24759-861B-4669-ADFF-C4156AAE4E2F}"/>
-    <hyperlink ref="M117" r:id="rId317" xr:uid="{D179D731-7129-48DD-A00F-1348AC3C4ED4}"/>
-    <hyperlink ref="B118" r:id="rId318" xr:uid="{1680DDE9-7579-497E-83E5-087000BF146D}"/>
-    <hyperlink ref="L118" r:id="rId319" xr:uid="{A33E09E5-7ACD-4393-8824-DD31CE3CAE77}"/>
-    <hyperlink ref="B119" r:id="rId320" xr:uid="{CDFBAE7C-5A2C-4092-B983-63911820D354}"/>
-    <hyperlink ref="H119" r:id="rId321" xr:uid="{2CAFEDCD-2D4E-45F7-9D03-93C94582E66B}"/>
-    <hyperlink ref="L119" r:id="rId322" xr:uid="{74F774C9-93F4-4C64-BB01-41D3B0CD11BB}"/>
-    <hyperlink ref="M119" r:id="rId323" xr:uid="{4D8C488D-0B85-471C-ABDD-15E053C5DCC2}"/>
-    <hyperlink ref="B120" r:id="rId324" xr:uid="{8154467C-C314-4C59-951C-9FBF046B45BC}"/>
-    <hyperlink ref="L120" r:id="rId325" xr:uid="{768D332B-9D2A-4150-98F9-0310C4163CA5}"/>
-    <hyperlink ref="B121" r:id="rId326" xr:uid="{87022AE0-ACC9-43EE-B17E-2AA059A8047D}"/>
-    <hyperlink ref="E121" r:id="rId327" xr:uid="{CACBC907-FDC3-4ED4-97F5-648B0FFC68FF}"/>
-    <hyperlink ref="L121" r:id="rId328" xr:uid="{4123DF38-8CC2-4941-8228-6AF8854B72EF}"/>
-    <hyperlink ref="M121" r:id="rId329" xr:uid="{82394FE1-C149-44D5-9D18-676153900727}"/>
-    <hyperlink ref="B122" r:id="rId330" xr:uid="{4E48D8FA-9AD5-4F84-A29B-2B901B99E042}"/>
-    <hyperlink ref="L122" r:id="rId331" xr:uid="{A3F369F1-A993-431A-B0C8-95882791950F}"/>
-    <hyperlink ref="B123" r:id="rId332" xr:uid="{CBA8383D-4B36-484C-A2C8-894B25BEBC45}"/>
-    <hyperlink ref="L123" r:id="rId333" xr:uid="{144D21CC-F11A-47FD-BB95-27B9B6526A7E}"/>
-    <hyperlink ref="B124" r:id="rId334" xr:uid="{416813EA-DF1F-4B21-804E-AC3149CD6890}"/>
-    <hyperlink ref="L124" r:id="rId335" xr:uid="{9AD263B1-9698-4B18-9D57-975996602CA6}"/>
-    <hyperlink ref="B125" r:id="rId336" xr:uid="{99A3DA52-0A78-4D7C-8221-D5969A661D0A}"/>
-    <hyperlink ref="L125" r:id="rId337" xr:uid="{DCB86820-41FA-4DEC-96DA-636AC8783424}"/>
-    <hyperlink ref="B126" r:id="rId338" xr:uid="{09EEC61D-DF2D-402A-8E81-CFDCF8ED390F}"/>
-    <hyperlink ref="L126" r:id="rId339" xr:uid="{8101F16F-087A-4059-B9F2-29CAEBF91DBB}"/>
-    <hyperlink ref="B127" r:id="rId340" xr:uid="{FEC10EC3-A0D2-457F-8F64-E18BA73C53DD}"/>
-    <hyperlink ref="L127" r:id="rId341" xr:uid="{6A71BC24-ED4A-4C00-993F-49EF84C2A60C}"/>
-    <hyperlink ref="B128" r:id="rId342" xr:uid="{EDB4AA45-D64C-4C30-974A-04B97B4783DD}"/>
-    <hyperlink ref="E128" r:id="rId343" xr:uid="{741D5AF2-727D-4974-8B21-E2CC60A61A7E}"/>
-    <hyperlink ref="L128" r:id="rId344" xr:uid="{79C56289-0EBB-487A-9A25-EA424BEA03A2}"/>
-    <hyperlink ref="M128" r:id="rId345" xr:uid="{826BD170-7220-421E-9E59-345A7090F24B}"/>
-    <hyperlink ref="B129" r:id="rId346" xr:uid="{245100B6-E350-40CE-9C75-629307E5DCD7}"/>
-    <hyperlink ref="L129" r:id="rId347" xr:uid="{5B489B99-1C66-44A3-BAD0-52DBFFEE6730}"/>
-    <hyperlink ref="M129" r:id="rId348" xr:uid="{DE157646-5236-43F5-A671-59B3394D0313}"/>
-    <hyperlink ref="B130" r:id="rId349" xr:uid="{79BFF90C-07B0-4EA4-85F4-339B3DACE763}"/>
-    <hyperlink ref="L130" r:id="rId350" xr:uid="{F7CC83C4-2C15-4B28-8775-332ECECD56DB}"/>
-    <hyperlink ref="M130" r:id="rId351" xr:uid="{C6BD178A-3C31-48FC-876E-D46B2454BE71}"/>
-    <hyperlink ref="B131" r:id="rId352" xr:uid="{0FEB1919-22A2-47BF-927A-266E691D2856}"/>
-    <hyperlink ref="E131" r:id="rId353" xr:uid="{A66A1345-A230-4AFE-B0CB-BECD9379EF40}"/>
-    <hyperlink ref="L131" r:id="rId354" xr:uid="{548B52B2-B3B7-43A5-9B9A-D899FCC0A252}"/>
-    <hyperlink ref="M131" r:id="rId355" xr:uid="{47AC3314-7CD4-44C2-8478-9CE0154B7A07}"/>
-    <hyperlink ref="B132" r:id="rId356" xr:uid="{46F10E10-F011-4356-BAE2-8116E9917874}"/>
-    <hyperlink ref="E132" r:id="rId357" xr:uid="{D11824AE-9A5B-43E9-9345-BFF1C7260AC8}"/>
-    <hyperlink ref="L132" r:id="rId358" xr:uid="{BF26EB28-7F01-4339-AF37-27390161DB57}"/>
-    <hyperlink ref="M132" r:id="rId359" xr:uid="{C3E9098C-857F-48C9-B80A-8FD440FF198B}"/>
-    <hyperlink ref="B133" r:id="rId360" xr:uid="{E71716ED-2C5F-46AC-8118-E66F246A9225}"/>
-    <hyperlink ref="L133" r:id="rId361" xr:uid="{19B43415-EE88-459A-8121-0C32772BDA9C}"/>
-    <hyperlink ref="B134" r:id="rId362" xr:uid="{27800E68-043A-48B3-A2C7-6F6FB941F037}"/>
-    <hyperlink ref="E134" r:id="rId363" xr:uid="{7E515852-1107-441C-814E-E559774DA21C}"/>
-    <hyperlink ref="L134" r:id="rId364" xr:uid="{84322BF6-E01F-410D-AAF6-74FF8132B70F}"/>
-    <hyperlink ref="M134" r:id="rId365" xr:uid="{A42760AA-0133-483B-B7DB-F81CD4A13ED8}"/>
-    <hyperlink ref="B135" r:id="rId366" xr:uid="{005C5B41-5F4D-4335-8553-25B982204EDF}"/>
-    <hyperlink ref="H135" r:id="rId367" xr:uid="{05C9422C-CF62-4061-8DA4-671D3675EC70}"/>
-    <hyperlink ref="L135" r:id="rId368" xr:uid="{C40DAFEF-FBB6-4457-BC18-FCCFDFCC8B0D}"/>
-    <hyperlink ref="M135" r:id="rId369" xr:uid="{60701ED5-7E9D-4C2B-90C2-822C3CF759A4}"/>
-    <hyperlink ref="B136" r:id="rId370" xr:uid="{B8BCB3B0-A0F4-469D-A917-BEF25C234D8B}"/>
-    <hyperlink ref="L136" r:id="rId371" xr:uid="{8271C14C-51B1-47A9-A8E7-25414D930F63}"/>
-    <hyperlink ref="B137" r:id="rId372" xr:uid="{579EDC0E-290D-42E8-9D13-DD642909C1DF}"/>
-    <hyperlink ref="L137" r:id="rId373" xr:uid="{9450C728-F256-4CCF-97ED-ED39D72953A3}"/>
-    <hyperlink ref="B138" r:id="rId374" xr:uid="{1732F742-A54A-420C-B0CD-C4A1E1A945DD}"/>
-    <hyperlink ref="L138" r:id="rId375" xr:uid="{BE4B0DAC-92AF-48F1-B61D-CA2B28C72FE8}"/>
-    <hyperlink ref="B139" r:id="rId376" xr:uid="{27AB2C40-ABC6-4719-918A-5CFD41E1C53E}"/>
-    <hyperlink ref="L139" r:id="rId377" xr:uid="{75BAD27E-6354-4E30-874A-AC877AE8B5E3}"/>
-    <hyperlink ref="B140" r:id="rId378" xr:uid="{B231BAC6-6031-411B-819D-3CA2EDDA4622}"/>
-    <hyperlink ref="L140" r:id="rId379" xr:uid="{58DB9950-596D-435C-AD0A-423D96CEB22E}"/>
-    <hyperlink ref="B141" r:id="rId380" xr:uid="{E840CCFB-F041-4811-89AC-AD10C2436837}"/>
-    <hyperlink ref="L141" r:id="rId381" xr:uid="{B9524DC6-A13F-4717-B958-F8C73A68EC15}"/>
-    <hyperlink ref="B142" r:id="rId382" xr:uid="{75ADB35E-7EBF-48DB-99EF-7B10217CCC16}"/>
-    <hyperlink ref="L142" r:id="rId383" xr:uid="{D131CFED-24BE-4B61-B6D3-3FA2A2876456}"/>
-    <hyperlink ref="B143" r:id="rId384" xr:uid="{CD1B8FEE-EB31-4BCA-9782-88BC8D351A5B}"/>
-    <hyperlink ref="L143" r:id="rId385" xr:uid="{DAD94694-A586-445B-A6E3-A708D699D8B5}"/>
-    <hyperlink ref="B144" r:id="rId386" xr:uid="{0A2438FB-9D12-445A-A63A-083CA4F0F2C9}"/>
-    <hyperlink ref="L144" r:id="rId387" xr:uid="{246325B1-9CA9-4F35-ACAB-028028E47522}"/>
-    <hyperlink ref="B145" r:id="rId388" xr:uid="{97488B87-8C2C-479C-98AC-536483653BB6}"/>
-    <hyperlink ref="L145" r:id="rId389" xr:uid="{5E5B1A88-E9F3-46D4-9AD0-6F83BC5654FB}"/>
-    <hyperlink ref="B146" r:id="rId390" xr:uid="{0B20AEF0-543E-4429-B171-749023EA9E17}"/>
-    <hyperlink ref="L146" r:id="rId391" xr:uid="{9B74EBB6-D9B2-4D49-9ABF-123B0054910B}"/>
-    <hyperlink ref="B147" r:id="rId392" xr:uid="{D3F65BB4-4B0D-4924-AA09-15479505BDAE}"/>
-    <hyperlink ref="L147" r:id="rId393" xr:uid="{1121E938-E410-4F34-BC4C-3647E6301076}"/>
-    <hyperlink ref="B148" r:id="rId394" xr:uid="{698B57EF-C136-4F82-84CC-556FCCFF0F99}"/>
-    <hyperlink ref="L148" r:id="rId395" xr:uid="{A90568EC-2803-419A-81D0-1C10B6C23507}"/>
-    <hyperlink ref="B149" r:id="rId396" xr:uid="{67A23531-F7CA-4294-828C-23DCDB1AB758}"/>
-    <hyperlink ref="E149" r:id="rId397" xr:uid="{764FC6B2-B578-4F83-9C94-D116CB05FFB2}"/>
-    <hyperlink ref="L149" r:id="rId398" xr:uid="{EF9C240B-65AC-4FFA-860D-DF63BCF7924F}"/>
-    <hyperlink ref="M149" r:id="rId399" xr:uid="{3C351911-B47A-4674-8CC4-1507B0B33378}"/>
-    <hyperlink ref="B150" r:id="rId400" xr:uid="{47A276D5-5846-4BA5-8CDA-370F6A1A5459}"/>
-    <hyperlink ref="L150" r:id="rId401" xr:uid="{31691F32-D7E8-4496-9A65-9EDEF4015A5B}"/>
-    <hyperlink ref="B151" r:id="rId402" xr:uid="{24D5BDC0-D07F-4E1A-9B33-A09FA373706B}"/>
-    <hyperlink ref="L151" r:id="rId403" xr:uid="{0A99FD7D-3AFE-42EE-8C26-F815149E1EF3}"/>
-    <hyperlink ref="B152" r:id="rId404" xr:uid="{D81C2AFB-41C9-4D2A-BDE1-A9174C777AAD}"/>
-    <hyperlink ref="L152" r:id="rId405" xr:uid="{E54C8E2A-2AFC-4D82-A490-080ECFA76706}"/>
-    <hyperlink ref="B153" r:id="rId406" xr:uid="{0A52915B-3C8D-45EA-BF16-ADA25884D969}"/>
-    <hyperlink ref="L153" r:id="rId407" xr:uid="{114388AE-5816-46C2-A82E-EBED5E07ED61}"/>
-    <hyperlink ref="B154" r:id="rId408" xr:uid="{CB7FC242-65F3-4B12-A9DA-597F1394E8E5}"/>
-    <hyperlink ref="E154" r:id="rId409" xr:uid="{B5675B2B-25EA-4B19-904B-C98C1851F113}"/>
-    <hyperlink ref="L154" r:id="rId410" xr:uid="{C3DD42C8-94EE-4E95-8AA9-BE1DFA507430}"/>
-    <hyperlink ref="M154" r:id="rId411" xr:uid="{03C096EF-92DF-4C2D-A1FE-3E647E927F2C}"/>
-    <hyperlink ref="B155" r:id="rId412" xr:uid="{20AC118F-A07C-4218-A9C4-D18762FEDB22}"/>
-    <hyperlink ref="L155" r:id="rId413" xr:uid="{0770F099-28DE-4F33-BD16-BE01AA341B29}"/>
-    <hyperlink ref="B156" r:id="rId414" xr:uid="{BA3F6744-B769-4469-9DE0-8E1E0541A301}"/>
-    <hyperlink ref="L156" r:id="rId415" xr:uid="{17A4D028-BEA5-4D71-8E9D-7AE00F4150E6}"/>
-    <hyperlink ref="M156" r:id="rId416" xr:uid="{175239C6-6D8E-4FD4-8EA9-CD259560C6EA}"/>
-    <hyperlink ref="B157" r:id="rId417" xr:uid="{24A2C199-379D-4E34-91C7-C9890D0CA846}"/>
-    <hyperlink ref="L157" r:id="rId418" xr:uid="{3C340DE2-5D4C-40C2-88A4-E1DA8519D775}"/>
-    <hyperlink ref="B158" r:id="rId419" xr:uid="{09191A77-4E9E-44DF-834F-AD5A859FA73A}"/>
-    <hyperlink ref="H158" r:id="rId420" xr:uid="{0FBC67A2-DC4D-4A29-BC4C-7E7FB94E3BD8}"/>
-    <hyperlink ref="L158" r:id="rId421" xr:uid="{DD908217-EAF5-4D91-8E41-BEA4EA08984A}"/>
-    <hyperlink ref="M158" r:id="rId422" xr:uid="{6B94E662-E395-4B49-9C36-127011E95370}"/>
-    <hyperlink ref="B159" r:id="rId423" xr:uid="{896DCD7E-6F97-41F3-94CC-FAEB84666AFD}"/>
-    <hyperlink ref="L159" r:id="rId424" xr:uid="{1004395F-2719-4F52-A1DB-8F485B213593}"/>
-    <hyperlink ref="B160" r:id="rId425" xr:uid="{24571C3F-7834-4032-B0A3-687EEFD1815A}"/>
-    <hyperlink ref="L160" r:id="rId426" xr:uid="{7C5C01F5-CAE8-47CC-8985-E97BF658C14A}"/>
-    <hyperlink ref="B161" r:id="rId427" xr:uid="{5EDF2E63-F777-42BA-88E4-09E8415D8F93}"/>
-    <hyperlink ref="L161" r:id="rId428" xr:uid="{00A83275-3006-4941-A78C-B667E6B2CE21}"/>
-    <hyperlink ref="B162" r:id="rId429" xr:uid="{42B28617-9299-4486-9872-7ACA9A866176}"/>
-    <hyperlink ref="E162" r:id="rId430" xr:uid="{6F39E867-4685-460C-9BAC-456E2260CA60}"/>
-    <hyperlink ref="L162" r:id="rId431" xr:uid="{7517B42A-DD79-408F-AE28-C68825B47311}"/>
-    <hyperlink ref="M162" r:id="rId432" xr:uid="{279C519A-E0A2-4558-802C-3ABC71E3EBEB}"/>
-    <hyperlink ref="B163" r:id="rId433" xr:uid="{6AEF4EBB-60DF-447C-B494-877D4547E659}"/>
-    <hyperlink ref="L163" r:id="rId434" xr:uid="{60D1B2BB-7023-4E91-9B1D-92677C4A833A}"/>
-    <hyperlink ref="M163" r:id="rId435" xr:uid="{05C84012-6334-4B45-95D7-AC89485BAD3F}"/>
-    <hyperlink ref="B164" r:id="rId436" xr:uid="{2655ED4C-FA8A-4F8C-A2E6-38BADBC67EAA}"/>
-    <hyperlink ref="L164" r:id="rId437" xr:uid="{E4AF88AE-FFCD-4162-AF3F-CCE195D98B6A}"/>
-    <hyperlink ref="B165" r:id="rId438" xr:uid="{95B108F5-8636-4F73-89AB-E58DBF24B540}"/>
-    <hyperlink ref="L165" r:id="rId439" xr:uid="{6CC8BA5D-303A-4C45-8AE2-6732341AD643}"/>
-    <hyperlink ref="B166" r:id="rId440" xr:uid="{EAA64A0A-C404-45E6-8265-3E1409B184F4}"/>
-    <hyperlink ref="L166" r:id="rId441" xr:uid="{7BCE8D0D-9912-4F25-9CAB-C82C99975A0C}"/>
-    <hyperlink ref="M166" r:id="rId442" xr:uid="{494FEB9B-5AEC-4479-849B-C0123B3B4580}"/>
-    <hyperlink ref="B167" r:id="rId443" xr:uid="{D970A6E6-DD10-4B43-803D-A00F7F20FC39}"/>
-    <hyperlink ref="L167" r:id="rId444" xr:uid="{B80419DA-7E9C-4C6F-BE75-AE7BA4B37F40}"/>
-    <hyperlink ref="B168" r:id="rId445" xr:uid="{F4D498BC-C189-4576-8FF9-43164D5916DF}"/>
-    <hyperlink ref="E168" r:id="rId446" xr:uid="{D0AB8753-3B9D-4372-AE7F-DC6DF6D21A48}"/>
-    <hyperlink ref="L168" r:id="rId447" xr:uid="{7A4FACFB-74A8-4ECA-B0D8-A25F96E47E17}"/>
-    <hyperlink ref="M168" r:id="rId448" xr:uid="{0567F44D-E52D-41E9-A330-2E68492B96B5}"/>
-    <hyperlink ref="B169" r:id="rId449" xr:uid="{090ECF89-C295-461A-A210-9D8AC5085D64}"/>
-    <hyperlink ref="L169" r:id="rId450" xr:uid="{BB307E3B-A8E7-4204-A192-7D69F38E3A0E}"/>
-    <hyperlink ref="B170" r:id="rId451" xr:uid="{71357826-87BB-4758-826C-75156B92EA5B}"/>
-    <hyperlink ref="L170" r:id="rId452" xr:uid="{11FCEA13-D8A7-441B-BFD5-85841F52355E}"/>
-    <hyperlink ref="B171" r:id="rId453" xr:uid="{C4AD90A1-4859-4385-A2F3-42D705FFC100}"/>
-    <hyperlink ref="L171" r:id="rId454" xr:uid="{8AE7CA6F-EF3F-4286-BD17-044AEC2E7A21}"/>
-    <hyperlink ref="B172" r:id="rId455" xr:uid="{A1D588EA-60BC-4BE7-8F0B-09849945ED0B}"/>
-    <hyperlink ref="E172" r:id="rId456" xr:uid="{DE004DFC-3193-48B5-BBFF-2B3F33AE8C32}"/>
-    <hyperlink ref="L172" r:id="rId457" xr:uid="{850EF190-ADAD-4EAB-91E6-77B09E9FB9ED}"/>
-    <hyperlink ref="M172" r:id="rId458" xr:uid="{A8D16C7F-45B4-4519-80C2-4C20FE1E8C6C}"/>
-    <hyperlink ref="B173" r:id="rId459" xr:uid="{83F7327F-A98A-4833-B619-98EC76BBCFF7}"/>
-    <hyperlink ref="L173" r:id="rId460" xr:uid="{B1DC5953-3B3A-4266-9CD2-D63F909F2661}"/>
-    <hyperlink ref="B174" r:id="rId461" xr:uid="{60F09B1F-DC7A-4635-979F-1F47D50C1850}"/>
-    <hyperlink ref="L174" r:id="rId462" xr:uid="{94671165-41B8-4D7E-9C6B-6C0030BBD837}"/>
-    <hyperlink ref="B175" r:id="rId463" xr:uid="{79E41D6D-F6CF-448C-9EFF-FCF0C6A8FCE8}"/>
-    <hyperlink ref="L175" r:id="rId464" xr:uid="{51732E39-C832-4D25-835D-CAAE471286F8}"/>
-    <hyperlink ref="B176" r:id="rId465" xr:uid="{B8760B18-BA3C-4A49-8DE3-3E40AB35538A}"/>
-    <hyperlink ref="E176" r:id="rId466" xr:uid="{8FF13FC4-BE34-400A-9173-78DAB9C24946}"/>
-    <hyperlink ref="L176" r:id="rId467" xr:uid="{CD6D28B6-9ACE-4C37-A16A-66A1F74556D7}"/>
-    <hyperlink ref="M176" r:id="rId468" xr:uid="{0795A1AA-6411-454B-897E-0B2CEC00DC2E}"/>
-    <hyperlink ref="B177" r:id="rId469" xr:uid="{E9DF3F97-4AA8-4286-9C7F-6030C13CB376}"/>
-    <hyperlink ref="E177" r:id="rId470" xr:uid="{71E6504A-B8B6-49D9-A894-9E608EB97652}"/>
-    <hyperlink ref="L177" r:id="rId471" xr:uid="{DCA77050-9831-4B39-8BF7-0554A025A5EE}"/>
-    <hyperlink ref="M177" r:id="rId472" xr:uid="{086A2C1A-16E2-4CAD-B24D-5E1445C1090C}"/>
-    <hyperlink ref="B178" r:id="rId473" xr:uid="{6111ECA8-5A13-42F0-A165-5DCD72D19A12}"/>
-    <hyperlink ref="L178" r:id="rId474" xr:uid="{54A6C083-6253-4943-B995-594D2C2D7858}"/>
-    <hyperlink ref="B179" r:id="rId475" xr:uid="{CCBFEDC6-9B65-4486-ADC0-260A7C97673C}"/>
-    <hyperlink ref="E179" r:id="rId476" xr:uid="{FCDE018E-ECD5-48F6-8744-B06EB58247D7}"/>
-    <hyperlink ref="L179" r:id="rId477" xr:uid="{9F110849-0D1B-42B7-BF03-9FE2F10B216C}"/>
-    <hyperlink ref="M179" r:id="rId478" xr:uid="{83442071-B2A6-4AD1-A6AC-EA82622E321F}"/>
-    <hyperlink ref="B180" r:id="rId479" xr:uid="{08A99911-E7FA-43E6-AF1C-D2D24F04B743}"/>
-    <hyperlink ref="L180" r:id="rId480" xr:uid="{30891317-B2DF-428C-B396-D568F2055225}"/>
-    <hyperlink ref="B181" r:id="rId481" xr:uid="{513C7C0D-3BA1-4A4D-AB4C-2E2DF5CE6768}"/>
-    <hyperlink ref="E181" r:id="rId482" xr:uid="{BF919AF7-DFDF-4381-AC0A-7A07D1BAC1D7}"/>
-    <hyperlink ref="L181" r:id="rId483" xr:uid="{3D4AB93F-27E5-4FB8-9A65-7B078FC94817}"/>
-    <hyperlink ref="M181" r:id="rId484" xr:uid="{8FFF08C0-4B0B-4024-96D0-789B753C601A}"/>
-    <hyperlink ref="B182" r:id="rId485" xr:uid="{AA3D17C0-815F-48EF-9CEA-71BAC54CBDC9}"/>
-    <hyperlink ref="L182" r:id="rId486" xr:uid="{44AFE6F6-B75C-48E7-9DF2-224DB2B948CC}"/>
-    <hyperlink ref="B183" r:id="rId487" xr:uid="{A70334C5-A820-47FB-AAAD-828A6EDAF2C4}"/>
-    <hyperlink ref="L183" r:id="rId488" xr:uid="{851AEB43-3100-4BD4-8CAB-7A089032C351}"/>
-    <hyperlink ref="B184" r:id="rId489" xr:uid="{2D535571-9F81-4ADA-A60F-55D44B62E7F3}"/>
-    <hyperlink ref="H184" r:id="rId490" xr:uid="{6F8DD5B4-5F53-4E34-8E95-E128CFC79E98}"/>
-    <hyperlink ref="L184" r:id="rId491" xr:uid="{EE52E15F-1D63-4F41-B887-6009910C629E}"/>
-    <hyperlink ref="M184" r:id="rId492" xr:uid="{71ED904D-C299-45AB-83E5-D72C13B72B96}"/>
-    <hyperlink ref="B185" r:id="rId493" xr:uid="{5FF3BF63-5BED-4F6A-B04A-ECEBE4B61CC4}"/>
-    <hyperlink ref="H185" r:id="rId494" xr:uid="{DDFCA117-11E3-4C0A-BF15-FF25A2C6B32D}"/>
-    <hyperlink ref="L185" r:id="rId495" xr:uid="{D66985F1-640B-45E7-A261-8B420B466240}"/>
-    <hyperlink ref="M185" r:id="rId496" xr:uid="{8B1B3D7D-627A-4D72-90BB-875BE4B6C33E}"/>
-    <hyperlink ref="B186" r:id="rId497" xr:uid="{97405C74-92B2-4E72-99EC-1D0F7266A589}"/>
-    <hyperlink ref="L186" r:id="rId498" xr:uid="{4A0EB185-2394-4FB9-A13F-6BF7F09A267D}"/>
-    <hyperlink ref="B187" r:id="rId499" xr:uid="{EF60E075-0BFA-4A44-874A-79C19C2572A9}"/>
-    <hyperlink ref="E187" r:id="rId500" xr:uid="{CCEA0781-7539-4AD0-8D20-D9EDC85DE025}"/>
-    <hyperlink ref="L187" r:id="rId501" xr:uid="{3329BCEB-9133-4FEC-8EE3-7078C28EB168}"/>
-    <hyperlink ref="M187" r:id="rId502" xr:uid="{42D82B7E-9D70-4FD1-99B7-21358C0DE55E}"/>
-    <hyperlink ref="B188" r:id="rId503" xr:uid="{C7B44DA9-D9A2-46CF-AC1B-B9E02D2FD7D8}"/>
-    <hyperlink ref="L188" r:id="rId504" xr:uid="{E0EAACB4-FECC-4811-8A00-0C24A4F9C7C5}"/>
-    <hyperlink ref="B189" r:id="rId505" xr:uid="{A74CCB67-1760-411F-8537-2E0AA014D048}"/>
-    <hyperlink ref="E189" r:id="rId506" xr:uid="{E40BC0EF-1A6C-43E7-99EA-B66686C9ED73}"/>
-    <hyperlink ref="L189" r:id="rId507" xr:uid="{8708529B-8E03-42A1-8E47-F52529D9D436}"/>
-    <hyperlink ref="M189" r:id="rId508" xr:uid="{5A94DFD2-621F-4377-95D1-882BD7B3A279}"/>
-    <hyperlink ref="B190" r:id="rId509" xr:uid="{842CAD7D-45E0-4063-A06B-0128071F0C02}"/>
-    <hyperlink ref="L190" r:id="rId510" xr:uid="{797DB053-DFB5-415D-9DE0-AA312C56E6DC}"/>
-    <hyperlink ref="B191" r:id="rId511" xr:uid="{F6A2F310-B1CA-4A42-B65F-76EFF67B0BAF}"/>
-    <hyperlink ref="E191" r:id="rId512" xr:uid="{6A251D7E-9309-4141-8843-097672D721E1}"/>
-    <hyperlink ref="H191" r:id="rId513" xr:uid="{45CE5465-7984-40E1-971F-097E1F0AACB3}"/>
-    <hyperlink ref="L191" r:id="rId514" xr:uid="{F0C2A6EB-F223-4A43-BBD6-E89608D361DE}"/>
-    <hyperlink ref="M191" r:id="rId515" xr:uid="{B9A8C6B6-6236-415C-9688-591657E841D2}"/>
-    <hyperlink ref="B192" r:id="rId516" xr:uid="{EB11B652-663C-4C65-976F-7C0F51D2783E}"/>
-    <hyperlink ref="L192" r:id="rId517" xr:uid="{978FDAC7-B6E0-4C94-A7AF-AD1B5F118EC0}"/>
-    <hyperlink ref="B193" r:id="rId518" xr:uid="{C8E87A07-8540-4197-AD57-63E31D9D1F39}"/>
-    <hyperlink ref="L193" r:id="rId519" xr:uid="{6E3B58D9-398F-4358-943C-9BF779D67A4D}"/>
-    <hyperlink ref="M193" r:id="rId520" xr:uid="{CD63E100-F6E6-47F2-8A70-EAAA4A2A9F0C}"/>
-    <hyperlink ref="B194" r:id="rId521" xr:uid="{E9089C5E-CE97-496B-806D-19256111622B}"/>
-    <hyperlink ref="L194" r:id="rId522" xr:uid="{53BDFED7-93CB-4209-84C6-463CE303345D}"/>
-    <hyperlink ref="B195" r:id="rId523" xr:uid="{19A31951-8FFA-4447-AF96-ADE0A6A40D69}"/>
-    <hyperlink ref="E195" r:id="rId524" xr:uid="{4A70F7AD-74A7-44B0-9D3F-64399463B9DE}"/>
-    <hyperlink ref="L195" r:id="rId525" xr:uid="{C607109E-B7B0-42FA-8BDC-0F73418B031D}"/>
-    <hyperlink ref="M195" r:id="rId526" xr:uid="{0BE2EBF5-ADAE-4096-AB59-3FE15F1A80CF}"/>
-    <hyperlink ref="B196" r:id="rId527" xr:uid="{ED6B98C5-0625-43E7-A775-6BE75732F43E}"/>
-    <hyperlink ref="E196" r:id="rId528" xr:uid="{8AE7667E-8B2E-45C8-87AA-547D3D70F94B}"/>
-    <hyperlink ref="L196" r:id="rId529" xr:uid="{2E059331-5CCD-4E19-AECC-3873865BBA2F}"/>
-    <hyperlink ref="M196" r:id="rId530" xr:uid="{84D76D05-B976-418C-BB6D-CDFF70BBA7DC}"/>
-    <hyperlink ref="B197" r:id="rId531" xr:uid="{9C85FD83-994A-4DCD-99B0-D6356C25E84A}"/>
-    <hyperlink ref="L197" r:id="rId532" xr:uid="{277248BD-7010-4BEA-A9CF-9C46C1D35068}"/>
-    <hyperlink ref="B198" r:id="rId533" xr:uid="{1E15FA6A-483B-42EA-8835-71CDC39D3C77}"/>
-    <hyperlink ref="L198" r:id="rId534" xr:uid="{22CB91F1-A048-4CB8-8637-DBC72BE6E43B}"/>
-    <hyperlink ref="B199" r:id="rId535" xr:uid="{9C8250C7-F090-4FE2-AD7A-3FDFAC019EBE}"/>
-    <hyperlink ref="L199" r:id="rId536" xr:uid="{832A2872-9B6D-4F6E-97AC-8C9ADD9CBFA9}"/>
-    <hyperlink ref="B200" r:id="rId537" xr:uid="{5F8C6FFA-E7DC-4655-8D80-AFF7DC931E3B}"/>
-    <hyperlink ref="L200" r:id="rId538" xr:uid="{F7684F7B-44FE-43D1-851F-9C85E9AE47D2}"/>
-    <hyperlink ref="M200" r:id="rId539" xr:uid="{3C4BACFE-2890-4EBC-A2DB-AEB1E551E7C3}"/>
-    <hyperlink ref="B201" r:id="rId540" xr:uid="{7810BB9B-8796-495F-8C51-54208F7D59FF}"/>
-    <hyperlink ref="L201" r:id="rId541" xr:uid="{65942DC7-FBE3-48B0-AE00-F51FBE961930}"/>
-    <hyperlink ref="B202" r:id="rId542" xr:uid="{5AC845B3-C29C-42AF-B5A0-E30FAC67E5BE}"/>
-    <hyperlink ref="E202" r:id="rId543" xr:uid="{8F070A6C-5DB1-4964-BA34-B0B7B0922E48}"/>
-    <hyperlink ref="L202" r:id="rId544" xr:uid="{B71E5467-208F-4A51-8745-3AB1DE727767}"/>
-    <hyperlink ref="M202" r:id="rId545" xr:uid="{E2C28FAE-40D1-49BB-B618-02965916649B}"/>
-    <hyperlink ref="B203" r:id="rId546" xr:uid="{F5AB4946-870D-40A8-9BA8-0758DCA7EA3D}"/>
-    <hyperlink ref="L203" r:id="rId547" xr:uid="{A3CC4617-FA89-40BF-B6B5-C5760B5519D9}"/>
-    <hyperlink ref="B204" r:id="rId548" xr:uid="{B7880F31-B52A-4BEE-8C21-2EF91A453210}"/>
-    <hyperlink ref="L204" r:id="rId549" xr:uid="{A84DC5A8-1DF9-4401-9C6A-482083F14B91}"/>
-    <hyperlink ref="B205" r:id="rId550" xr:uid="{FD16B199-7619-4A35-A062-AFCC2ACD5648}"/>
-    <hyperlink ref="L205" r:id="rId551" xr:uid="{F49D823F-17A2-4CD6-ACD3-6AAC9C997639}"/>
-    <hyperlink ref="B206" r:id="rId552" xr:uid="{64BBAAAF-EC46-48DB-8729-6A0833FC0882}"/>
-    <hyperlink ref="L206" r:id="rId553" xr:uid="{92010D58-F7C5-44AD-84B2-D3AC0BE33DE3}"/>
-    <hyperlink ref="B207" r:id="rId554" xr:uid="{933E59CB-65CE-43BA-86BD-7C75CBB7815C}"/>
-    <hyperlink ref="L207" r:id="rId555" xr:uid="{248CDB57-BC81-4409-87D7-FBDEEDA8D027}"/>
-    <hyperlink ref="M207" r:id="rId556" xr:uid="{C8725875-122F-4635-BBA0-57DFA6694C74}"/>
-    <hyperlink ref="B208" r:id="rId557" xr:uid="{1DDDFF6A-B044-4201-B370-EE50097E2665}"/>
-    <hyperlink ref="E208" r:id="rId558" xr:uid="{5ADD9190-3FF7-469D-9859-0D6B880D51FA}"/>
-    <hyperlink ref="L208" r:id="rId559" xr:uid="{C026A516-34B1-48F8-9CBE-4C97A38251F7}"/>
-    <hyperlink ref="M208" r:id="rId560" xr:uid="{B7DACFB8-7AD0-4677-9CFD-2E15F6A4D897}"/>
-    <hyperlink ref="B209" r:id="rId561" xr:uid="{57F3598A-8470-4338-BF7E-FEC7F3797B82}"/>
-    <hyperlink ref="L209" r:id="rId562" xr:uid="{77A107A4-A536-44F1-81AF-CECDBA0007F3}"/>
-    <hyperlink ref="M209" r:id="rId563" xr:uid="{94137B3B-9BAE-489E-A68F-0D32E554F8A0}"/>
-    <hyperlink ref="B210" r:id="rId564" xr:uid="{4C604184-2D01-41DA-8D95-D03991108320}"/>
-    <hyperlink ref="L210" r:id="rId565" xr:uid="{F1946E2A-ACE5-4575-8EF2-354B62F25E20}"/>
-    <hyperlink ref="M210" r:id="rId566" xr:uid="{C7FADEDA-3841-4102-A563-F6EF95485863}"/>
-    <hyperlink ref="B211" r:id="rId567" xr:uid="{E772D7F3-7275-4308-98B9-38E4AD176A8A}"/>
-    <hyperlink ref="L211" r:id="rId568" xr:uid="{D3CC3BB0-234C-4C70-8ADF-FF3D42212619}"/>
-    <hyperlink ref="B212" r:id="rId569" xr:uid="{73A69D0A-8BE2-412D-A0CE-CE64C1BB9975}"/>
-    <hyperlink ref="L212" r:id="rId570" xr:uid="{1B374010-AA73-466B-B571-71566D420825}"/>
-    <hyperlink ref="B213" r:id="rId571" xr:uid="{04B83679-6E64-4427-8D2C-9FBA6E409324}"/>
-    <hyperlink ref="H213" r:id="rId572" xr:uid="{A2F67A43-D381-45AE-9548-9314C6CC43E7}"/>
-    <hyperlink ref="L213" r:id="rId573" xr:uid="{9AA9EE3F-09DC-4CE1-B38B-E27D3F359095}"/>
-    <hyperlink ref="M213" r:id="rId574" xr:uid="{E812F4B8-7001-4537-982B-558B5B96B6FF}"/>
-    <hyperlink ref="B214" r:id="rId575" xr:uid="{E7C2004D-A8E2-49D9-8A22-33C0BABD11E3}"/>
-    <hyperlink ref="L214" r:id="rId576" xr:uid="{EB137DD8-5718-4FA8-99FC-4E32F3249787}"/>
-    <hyperlink ref="B215" r:id="rId577" xr:uid="{02078CE1-63FF-45E1-8FA2-A6D397D3DCB8}"/>
-    <hyperlink ref="L215" r:id="rId578" xr:uid="{FC20A19E-BB1D-4ECA-BCC3-E0C48E419F20}"/>
-    <hyperlink ref="B216" r:id="rId579" xr:uid="{02ABA7C3-16B7-4290-8787-3297E22DCA9E}"/>
-    <hyperlink ref="L216" r:id="rId580" xr:uid="{7C8E1754-5DD4-403D-A42D-65E344DDA77C}"/>
-    <hyperlink ref="M216" r:id="rId581" xr:uid="{ECE3019E-F8B5-4F3D-9214-856690550239}"/>
-    <hyperlink ref="B217" r:id="rId582" xr:uid="{A2E20D55-A246-4869-AB21-B01DEF68B377}"/>
-    <hyperlink ref="L217" r:id="rId583" xr:uid="{4679E0A0-5585-4990-8DFC-52F299A4F6AC}"/>
-    <hyperlink ref="M217" r:id="rId584" xr:uid="{7CD589A9-5802-4D28-920D-EB5D353D37E1}"/>
-    <hyperlink ref="B218" r:id="rId585" xr:uid="{E3BC1E74-E0AF-49E7-A00B-9419B43470B8}"/>
-    <hyperlink ref="L218" r:id="rId586" xr:uid="{03566DAA-65FB-4AC9-BEBA-F142FB743631}"/>
-    <hyperlink ref="M218" r:id="rId587" xr:uid="{45B3C2CB-A54F-49A5-9FB0-F512DDB50B95}"/>
-    <hyperlink ref="B219" r:id="rId588" xr:uid="{A3017E25-6377-4455-AF17-548A33C917DE}"/>
-    <hyperlink ref="L219" r:id="rId589" xr:uid="{F2A08BEB-2EAE-4FD1-BDC8-E3FE48011D36}"/>
-    <hyperlink ref="M219" r:id="rId590" xr:uid="{547E12F7-E719-49F2-AC20-DD672B05EA18}"/>
-    <hyperlink ref="B220" r:id="rId591" xr:uid="{B75195B5-FBE0-499B-918E-AA703D1E94ED}"/>
-    <hyperlink ref="L220" r:id="rId592" xr:uid="{63C009AD-A3D7-4C5D-B381-E29E386AA691}"/>
-    <hyperlink ref="B221" r:id="rId593" xr:uid="{C13827DC-CCF8-46BF-91D9-47E3564C3239}"/>
-    <hyperlink ref="L221" r:id="rId594" xr:uid="{F69EB030-97BF-4249-AFCF-2F63306411CA}"/>
-    <hyperlink ref="B222" r:id="rId595" xr:uid="{485D348D-4829-4BBA-BB9A-FC01B84CA7A8}"/>
-    <hyperlink ref="E222" r:id="rId596" xr:uid="{30B299FD-D47C-458B-A89D-0E7E7F240158}"/>
-    <hyperlink ref="L222" r:id="rId597" xr:uid="{0B6AC274-7BF1-48D4-B080-D7EA44E09E74}"/>
-    <hyperlink ref="M222" r:id="rId598" xr:uid="{59E74D00-E637-4867-B631-0C433ADE947C}"/>
-    <hyperlink ref="B223" r:id="rId599" xr:uid="{B5120B85-0D20-42EE-A3A3-B88BB3CF53CD}"/>
-    <hyperlink ref="L223" r:id="rId600" xr:uid="{37ABA84A-A593-429D-9FEE-C40DE477BFEA}"/>
-    <hyperlink ref="B224" r:id="rId601" xr:uid="{53978D0C-6989-41F0-AEF1-5AAD2BDAF653}"/>
-    <hyperlink ref="L224" r:id="rId602" xr:uid="{A0E116F8-2535-42A4-8915-21C9037F1BCC}"/>
-    <hyperlink ref="B225" r:id="rId603" xr:uid="{D0979FE1-D621-4D9D-ADB7-AFC6DB335A34}"/>
-    <hyperlink ref="L225" r:id="rId604" xr:uid="{B7766E56-5826-40EC-8BC0-66283E6C7F8A}"/>
-    <hyperlink ref="B226" r:id="rId605" xr:uid="{6B39E0A5-0214-4B41-B6E0-C4DE1B0DF117}"/>
-    <hyperlink ref="L226" r:id="rId606" xr:uid="{B9E305F8-4CEF-4FE8-B699-A1EE5F111C26}"/>
-    <hyperlink ref="B227" r:id="rId607" xr:uid="{D07FF528-4CE2-4B73-B08E-6E1E8A7776D3}"/>
-    <hyperlink ref="L227" r:id="rId608" xr:uid="{FE343E3D-E5E0-4B99-A6F0-AC58BA9244B0}"/>
-    <hyperlink ref="B228" r:id="rId609" xr:uid="{5A87FAD5-33C9-4D75-ACA5-47CDCFB50786}"/>
-    <hyperlink ref="L228" r:id="rId610" xr:uid="{6DB6C4AA-322E-40FF-B5F6-085B9D008E8D}"/>
-    <hyperlink ref="B229" r:id="rId611" xr:uid="{D3A24742-59B6-4A8D-BCB9-697DFBFB21EA}"/>
-    <hyperlink ref="L229" r:id="rId612" xr:uid="{2026E880-02E2-4FA9-8F25-B30FB4AB0ABA}"/>
-    <hyperlink ref="B230" r:id="rId613" xr:uid="{BFCC0B48-891F-4963-A006-13A19148B8AC}"/>
-    <hyperlink ref="L230" r:id="rId614" xr:uid="{D7181C1F-B2AE-4E64-8947-85075D5C0F36}"/>
-    <hyperlink ref="B231" r:id="rId615" xr:uid="{4D9824C9-8EDF-4D94-BD30-CD852C2713A3}"/>
-    <hyperlink ref="L231" r:id="rId616" xr:uid="{D621499E-9697-4682-AB49-C889C3750DEE}"/>
-    <hyperlink ref="B232" r:id="rId617" xr:uid="{1663BA50-4992-4A4C-A69F-66DBE9E88972}"/>
-    <hyperlink ref="L232" r:id="rId618" xr:uid="{3536DA97-89FB-48B7-920B-43264C6477AE}"/>
-    <hyperlink ref="B233" r:id="rId619" xr:uid="{C7CE4570-68D2-4A7B-A813-685F684735F9}"/>
-    <hyperlink ref="E233" r:id="rId620" xr:uid="{FE7327CA-4734-48B9-828F-32611D54B310}"/>
-    <hyperlink ref="L233" r:id="rId621" xr:uid="{EBAC550F-6FC0-428F-B51C-3C8E940B2A17}"/>
-    <hyperlink ref="M233" r:id="rId622" xr:uid="{1EA0C195-8973-44C0-9592-5C3AFC8713B7}"/>
-    <hyperlink ref="B234" r:id="rId623" xr:uid="{BD7F9288-ADB1-4ED7-83E8-34A4270D9BA9}"/>
-    <hyperlink ref="H234" r:id="rId624" xr:uid="{F5A72F6D-04C2-4DD9-B635-4C1F889C5F25}"/>
-    <hyperlink ref="L234" r:id="rId625" xr:uid="{05E5CF71-F823-4B9B-97D2-14F4385EC1B1}"/>
-    <hyperlink ref="M234" r:id="rId626" xr:uid="{0D1FA251-A22B-4C53-AE07-EE501120F259}"/>
-    <hyperlink ref="B235" r:id="rId627" xr:uid="{2B74FD8C-8FDF-4F5E-9AE4-DAE5587B7541}"/>
-    <hyperlink ref="L235" r:id="rId628" xr:uid="{D8CDF640-6603-4B74-82D1-20FDF3F9AC00}"/>
-    <hyperlink ref="B236" r:id="rId629" xr:uid="{9E06BF0A-5776-4AED-B5AD-D0DD8571DA95}"/>
-    <hyperlink ref="L236" r:id="rId630" xr:uid="{9FBBA2AD-3F2E-4D3D-9595-2D5A2398C794}"/>
-    <hyperlink ref="B237" r:id="rId631" xr:uid="{D1E58C8C-008A-47E1-9708-6873F1B41994}"/>
-    <hyperlink ref="L237" r:id="rId632" xr:uid="{C7FD0456-A895-4A5B-AFF9-1AB9F7FFC544}"/>
-    <hyperlink ref="M237" r:id="rId633" xr:uid="{E84671A7-5128-4BDC-84E3-786EFE4353CF}"/>
-    <hyperlink ref="B238" r:id="rId634" xr:uid="{89ABCE59-9AE5-4670-B0F4-791365EC6C82}"/>
-    <hyperlink ref="L238" r:id="rId635" xr:uid="{53374A9B-872A-4918-B6CD-BAFB09C1F980}"/>
-    <hyperlink ref="B239" r:id="rId636" xr:uid="{27A4DFA2-750C-4B5A-A6D2-8D063F05C8FF}"/>
-    <hyperlink ref="L239" r:id="rId637" xr:uid="{4534EB7A-5AC0-4DFC-A159-135FB366A9B8}"/>
-    <hyperlink ref="B240" r:id="rId638" xr:uid="{8B1C3542-8DFD-4ACC-B934-4960E373317A}"/>
-    <hyperlink ref="L240" r:id="rId639" xr:uid="{1B2BF305-1F32-41A3-B551-3EA3103F65F2}"/>
-    <hyperlink ref="B241" r:id="rId640" xr:uid="{16FBD938-BEA9-4B0C-9B05-14AE44CCF321}"/>
-    <hyperlink ref="L241" r:id="rId641" xr:uid="{76E8E204-DC68-4D7C-BDB9-394F73CCDD75}"/>
-    <hyperlink ref="B242" r:id="rId642" xr:uid="{9D9F72FF-BD2E-438D-8E94-CFF03CBFA290}"/>
-    <hyperlink ref="L242" r:id="rId643" xr:uid="{FC00A34F-F254-4E61-9213-9A3ED8596051}"/>
-    <hyperlink ref="B243" r:id="rId644" xr:uid="{971A923A-4681-4151-B313-B199F0215938}"/>
-    <hyperlink ref="L243" r:id="rId645" xr:uid="{4F9D055D-D07C-4A86-BAD3-C0EBFCBF893E}"/>
-    <hyperlink ref="B244" r:id="rId646" xr:uid="{0C369812-F11E-4A1B-9F00-362E7E4F3652}"/>
-    <hyperlink ref="L244" r:id="rId647" xr:uid="{54DB5B97-9F2A-44AA-94E2-E1502BB99662}"/>
-    <hyperlink ref="B245" r:id="rId648" xr:uid="{79BA4FA4-52DC-4B58-9AF0-B0115B08B45E}"/>
-    <hyperlink ref="L245" r:id="rId649" xr:uid="{1F197288-455F-4B0E-901B-B7ADE48F2AD4}"/>
-    <hyperlink ref="B246" r:id="rId650" xr:uid="{AD484B2E-A0E1-4BE2-99CC-2C41DCDFA84E}"/>
-    <hyperlink ref="L246" r:id="rId651" xr:uid="{0BB713AA-F561-4C46-96B2-11DC0530BFAE}"/>
-    <hyperlink ref="B247" r:id="rId652" xr:uid="{66360BC9-D356-438F-8787-1825D170AC1C}"/>
-    <hyperlink ref="L247" r:id="rId653" xr:uid="{DD4F9BAD-206B-4A4E-86DA-96F9A1D0554C}"/>
-    <hyperlink ref="B248" r:id="rId654" xr:uid="{2FEE503F-F854-4412-B060-C36A31FD403F}"/>
-    <hyperlink ref="L248" r:id="rId655" xr:uid="{4ADA2626-A90C-4A6D-98EE-D528189BD7C9}"/>
-    <hyperlink ref="B249" r:id="rId656" xr:uid="{3A86A5DB-FD62-4307-A64C-342AE53E556E}"/>
-    <hyperlink ref="L249" r:id="rId657" xr:uid="{5E1DA5C9-D144-4CCB-AA6B-2243C23123EF}"/>
-    <hyperlink ref="B250" r:id="rId658" xr:uid="{656B5F9C-DA5B-4AF6-81C8-18E6D9910B63}"/>
-    <hyperlink ref="L250" r:id="rId659" xr:uid="{76C2F806-6B1B-46B4-A339-287A6AD5DB7F}"/>
-    <hyperlink ref="B251" r:id="rId660" xr:uid="{2C6ABAC5-73AC-43BB-ABC1-1DF6A4BD1D1B}"/>
-    <hyperlink ref="L251" r:id="rId661" xr:uid="{C47CF5C2-AA27-4CD8-A41C-233F9D8D7BAA}"/>
-    <hyperlink ref="B252" r:id="rId662" xr:uid="{783DF5CB-C883-400B-9F54-102963181BA9}"/>
-    <hyperlink ref="E252" r:id="rId663" xr:uid="{6A494A39-743C-4874-A4EA-E373956F135A}"/>
-    <hyperlink ref="L252" r:id="rId664" xr:uid="{A6CF9EF9-D8F4-448E-87B9-55D6D4EFAE43}"/>
-    <hyperlink ref="M252" r:id="rId665" xr:uid="{02DC8763-0854-44E8-9CC5-BEC1038953F8}"/>
-    <hyperlink ref="B253" r:id="rId666" xr:uid="{97E8F5CC-578A-4B16-A57A-0CAD7257629F}"/>
-    <hyperlink ref="E253" r:id="rId667" xr:uid="{A738E66C-9970-458D-85B1-FEC9CCA4C0BD}"/>
-    <hyperlink ref="L253" r:id="rId668" xr:uid="{2C132E91-99B6-4D30-AFBB-1411E3959C36}"/>
-    <hyperlink ref="M253" r:id="rId669" xr:uid="{668E8150-6053-4604-914E-D7947EA4FC17}"/>
-    <hyperlink ref="B254" r:id="rId670" xr:uid="{489D941A-4FD1-40D4-9DE5-0E8FE76424E8}"/>
-    <hyperlink ref="E254" r:id="rId671" xr:uid="{BEAF274C-6DAE-4187-93EB-080A7FE8EA1E}"/>
-    <hyperlink ref="L254" r:id="rId672" xr:uid="{9E841D1B-D6EB-406F-8257-E3F0525AB35B}"/>
-    <hyperlink ref="M254" r:id="rId673" xr:uid="{E5BBBAC6-CB40-470C-A42D-99B4A24CC681}"/>
-    <hyperlink ref="B255" r:id="rId674" xr:uid="{256D7C1F-B6A5-4B3A-947F-879F769597C8}"/>
-    <hyperlink ref="L255" r:id="rId675" xr:uid="{053F4811-B932-413E-8736-6E691BE211DD}"/>
-    <hyperlink ref="M255" r:id="rId676" xr:uid="{56F11F1F-7A3A-4329-8E60-EE7DF31CC0D1}"/>
-    <hyperlink ref="B256" r:id="rId677" xr:uid="{504F0142-6144-486D-BDC0-106B354C49C5}"/>
-    <hyperlink ref="L256" r:id="rId678" xr:uid="{C4BF57C3-6259-4A50-B882-205B34D3CA14}"/>
-    <hyperlink ref="B257" r:id="rId679" xr:uid="{61CFC2E0-B5C1-410F-BE01-0F4E611F9381}"/>
-    <hyperlink ref="L257" r:id="rId680" xr:uid="{6361D7EC-693C-4C2D-A6A9-25C1C1840BD7}"/>
-    <hyperlink ref="B258" r:id="rId681" xr:uid="{E203AA78-D29F-4950-9DE2-68228F0F3752}"/>
-    <hyperlink ref="L258" r:id="rId682" xr:uid="{45A20866-3065-46AA-8968-229F50AAA356}"/>
-    <hyperlink ref="B259" r:id="rId683" xr:uid="{E80EC945-BAAA-463C-8922-BABCDBD9E5CC}"/>
-    <hyperlink ref="L259" r:id="rId684" xr:uid="{A8296BA7-97FA-4704-BE54-8FE6A4F4DF2F}"/>
-    <hyperlink ref="B260" r:id="rId685" xr:uid="{32BC2AEA-1FD7-4DBC-8C7D-2CADBC4EE7D5}"/>
-    <hyperlink ref="L260" r:id="rId686" xr:uid="{BC6D78E6-911C-4113-916F-FAF363A0E236}"/>
-    <hyperlink ref="B261" r:id="rId687" xr:uid="{8E3B95B5-1FAB-4702-92B0-38198E728866}"/>
-    <hyperlink ref="L261" r:id="rId688" xr:uid="{F76A4FF9-F4F5-449F-A9ED-6BBF2064FFCC}"/>
-    <hyperlink ref="B262" r:id="rId689" xr:uid="{55AD5103-C5EA-4F90-A279-0BDC53A638F8}"/>
-    <hyperlink ref="L262" r:id="rId690" xr:uid="{D8EC1E8D-4B48-4524-A084-1A8ADA50ADE7}"/>
-    <hyperlink ref="B263" r:id="rId691" xr:uid="{E4977C45-4DAB-4329-86B3-AFFB2B94A509}"/>
-    <hyperlink ref="L263" r:id="rId692" xr:uid="{292BEFEA-7C86-42CD-8157-3811E9AE9825}"/>
-    <hyperlink ref="B264" r:id="rId693" xr:uid="{754967D9-9C2D-4AD0-9AD8-645D6C3C40BC}"/>
-    <hyperlink ref="L264" r:id="rId694" xr:uid="{5D97FF3E-CCD2-4FCD-9560-AE0BA1FFFF8C}"/>
-    <hyperlink ref="B265" r:id="rId695" xr:uid="{B2DE10B1-1408-4547-A049-2072591E737A}"/>
-    <hyperlink ref="L265" r:id="rId696" xr:uid="{B8AD9F2D-6442-4585-A5EE-64673A9B321E}"/>
-    <hyperlink ref="B266" r:id="rId697" xr:uid="{729B772E-AE6B-4A67-B74F-22BC37F5EEAE}"/>
-    <hyperlink ref="L266" r:id="rId698" xr:uid="{407B27AD-8A7D-461D-90CF-2FA4FEF7E518}"/>
-    <hyperlink ref="B267" r:id="rId699" xr:uid="{A36117A0-59D9-4053-ADDD-2AA3E15A3907}"/>
-    <hyperlink ref="L267" r:id="rId700" xr:uid="{301DFCCB-C2C4-4E31-A35C-9F3BF69EE0F7}"/>
-    <hyperlink ref="B268" r:id="rId701" xr:uid="{42477523-948B-4428-BDF8-5ECAC5E6092B}"/>
-    <hyperlink ref="L268" r:id="rId702" xr:uid="{EA5C5F76-6BC9-414C-8718-D620E2A3E72E}"/>
-    <hyperlink ref="B269" r:id="rId703" xr:uid="{7AB10CCC-EEB8-44E8-A6A1-E601D1F0A1D8}"/>
-    <hyperlink ref="L269" r:id="rId704" xr:uid="{6E086B62-3ACB-4185-BB05-4EBB121D09E3}"/>
-    <hyperlink ref="B270" r:id="rId705" xr:uid="{E25552E7-DD6D-4445-BF8D-1EDF36B3F656}"/>
-    <hyperlink ref="L270" r:id="rId706" xr:uid="{16E73EAD-D938-4D00-AA0C-01446D52B636}"/>
-    <hyperlink ref="B271" r:id="rId707" xr:uid="{65E06790-4DDE-4149-8D33-3A1FB65DB52D}"/>
-    <hyperlink ref="E271" r:id="rId708" xr:uid="{8131809B-D209-4A31-BCFC-82221C6E6267}"/>
-    <hyperlink ref="L271" r:id="rId709" xr:uid="{62DA3E6D-794F-472D-AB3E-E98C5633A3E2}"/>
-    <hyperlink ref="M271" r:id="rId710" xr:uid="{11BA7EE6-4528-4F5B-9415-15C3234588B2}"/>
-    <hyperlink ref="B272" r:id="rId711" xr:uid="{6A49FAA1-AE42-43FF-A7E0-F1B7B033714F}"/>
-    <hyperlink ref="L272" r:id="rId712" xr:uid="{AEF2B2A6-FA75-4929-879F-EF5F34A92A60}"/>
-    <hyperlink ref="B273" r:id="rId713" xr:uid="{0718537C-E001-4CAF-BA0E-C18234CC4878}"/>
-    <hyperlink ref="L273" r:id="rId714" xr:uid="{E9559C0B-4A76-42FA-AE36-1667943FAE99}"/>
-    <hyperlink ref="M273" r:id="rId715" xr:uid="{BBF9FA1F-892E-4AF8-8169-45F8453989D2}"/>
-    <hyperlink ref="B274" r:id="rId716" xr:uid="{30FF65B3-60D3-45D1-9395-AE7FF697916D}"/>
-    <hyperlink ref="L274" r:id="rId717" xr:uid="{B9C9A8CB-4752-4293-8308-C68B3838E9AC}"/>
-    <hyperlink ref="B275" r:id="rId718" xr:uid="{DC28E7F3-47DF-451B-9731-C9C5D3083C67}"/>
-    <hyperlink ref="H275" r:id="rId719" xr:uid="{4810006D-A100-4A53-9531-79ECAB4E3145}"/>
-    <hyperlink ref="L275" r:id="rId720" xr:uid="{A27850F4-3753-41F9-B7CC-3E02EF5B5330}"/>
-    <hyperlink ref="M275" r:id="rId721" xr:uid="{F8D989EC-12C7-41AC-B051-8F944564F090}"/>
-    <hyperlink ref="B276" r:id="rId722" xr:uid="{7AE27CF2-53CA-4FBB-9F93-DDF1916D3D6F}"/>
-    <hyperlink ref="L276" r:id="rId723" xr:uid="{4B5057C3-9065-4C30-B22A-FE6E9CEC45FA}"/>
-    <hyperlink ref="M276" r:id="rId724" xr:uid="{ACA4AF61-9873-4A5D-AE9D-C83F7AD721D7}"/>
-    <hyperlink ref="B277" r:id="rId725" xr:uid="{B24C8A38-CE27-4724-95DF-ABFC121FE80B}"/>
-    <hyperlink ref="L277" r:id="rId726" xr:uid="{F9B9CC11-2090-4F74-9206-25B486EDA0D7}"/>
-    <hyperlink ref="M277" r:id="rId727" xr:uid="{ED083070-EFFD-4638-986E-63570A0AD1D7}"/>
-    <hyperlink ref="B278" r:id="rId728" xr:uid="{326606EF-0137-49E9-9987-B5CDC0054597}"/>
-    <hyperlink ref="L278" r:id="rId729" xr:uid="{AD6DA8C1-0FB2-499B-B7E3-4E3AAF0AC2CF}"/>
-    <hyperlink ref="M278" r:id="rId730" xr:uid="{A9CD5DC2-55AD-4528-9A44-ECB21940AC45}"/>
-    <hyperlink ref="B279" r:id="rId731" xr:uid="{DE3A4A87-DBD6-4A44-909D-8D86EA40A6B7}"/>
-    <hyperlink ref="L279" r:id="rId732" xr:uid="{E8FFA4DD-447C-4A01-9BAB-9A286F93BB3D}"/>
-    <hyperlink ref="B280" r:id="rId733" xr:uid="{4F266D74-FFFA-46FE-A6CE-216D993D7257}"/>
-    <hyperlink ref="L280" r:id="rId734" xr:uid="{6446031D-AFD9-46A0-A244-33E716A5A0F4}"/>
-    <hyperlink ref="B281" r:id="rId735" xr:uid="{67BF90F3-9A40-4B37-BC93-4612A16C6F44}"/>
-    <hyperlink ref="L281" r:id="rId736" xr:uid="{0E16EFDB-E675-4DBD-AD01-B290566F7C58}"/>
-    <hyperlink ref="B282" r:id="rId737" xr:uid="{2FAD85E8-4875-4D87-9A56-387BEB4529E9}"/>
-    <hyperlink ref="L282" r:id="rId738" xr:uid="{E2425B99-B04B-4528-92A1-4D66E98FAC1F}"/>
-    <hyperlink ref="B283" r:id="rId739" xr:uid="{B23221AC-DC5B-4DBE-8D4F-7566083BD879}"/>
-    <hyperlink ref="L283" r:id="rId740" xr:uid="{166467E4-4034-4DA0-87A5-BDE2747E8B34}"/>
-    <hyperlink ref="B284" r:id="rId741" xr:uid="{C6D104E0-4929-4C39-96B7-D969D9D5CB67}"/>
-    <hyperlink ref="L284" r:id="rId742" xr:uid="{243325E7-737A-4DFE-978B-9A2A3C659E30}"/>
-    <hyperlink ref="B285" r:id="rId743" xr:uid="{826710E7-58BA-4750-A535-5453AA5D69AB}"/>
-    <hyperlink ref="L285" r:id="rId744" xr:uid="{8A0094AD-B2A9-4711-939C-7CD41E68E9C7}"/>
-    <hyperlink ref="B286" r:id="rId745" xr:uid="{C951C424-217D-4C1E-BDED-E25494D6DE94}"/>
-    <hyperlink ref="L286" r:id="rId746" xr:uid="{4A72BD7A-411D-4D42-8E9A-7259A3C38291}"/>
-    <hyperlink ref="B287" r:id="rId747" xr:uid="{049F8C59-8ED2-4636-A1BA-C5AD3BDE942A}"/>
-    <hyperlink ref="L287" r:id="rId748" xr:uid="{09EE958F-8A2C-4C7E-AA11-40812CE262C4}"/>
-    <hyperlink ref="B288" r:id="rId749" xr:uid="{8EF24461-0656-4591-B82A-1AB580B6D272}"/>
-    <hyperlink ref="L288" r:id="rId750" xr:uid="{50414137-E1E0-4647-889E-8286C25D97A2}"/>
-    <hyperlink ref="B289" r:id="rId751" xr:uid="{DBC91ECB-44BF-4EA2-A8DD-3A252A92039A}"/>
-    <hyperlink ref="L289" r:id="rId752" xr:uid="{B2014C29-AA1F-4F5F-9F4C-BC1CE34771AD}"/>
-    <hyperlink ref="B290" r:id="rId753" xr:uid="{51F2674A-61DD-4C93-A724-65EB8B7F1695}"/>
-    <hyperlink ref="L290" r:id="rId754" xr:uid="{1D9D1A1B-CBE1-41F9-B0F0-C52A1BCFCC97}"/>
-    <hyperlink ref="B291" r:id="rId755" xr:uid="{C71A0068-9628-4F5F-A78A-15C75C832D48}"/>
-    <hyperlink ref="L291" r:id="rId756" xr:uid="{D14AF6D7-08AD-40F0-A836-EEFFE1F552ED}"/>
-    <hyperlink ref="B292" r:id="rId757" xr:uid="{272E3B5E-7049-4C53-9B62-4DB1370CA22E}"/>
-    <hyperlink ref="L292" r:id="rId758" xr:uid="{62DBFEC6-242E-411A-B8A2-3FAB5AB047A4}"/>
-    <hyperlink ref="B293" r:id="rId759" xr:uid="{19E43B4F-B5B9-4175-944E-3344341DD0DD}"/>
-    <hyperlink ref="L293" r:id="rId760" xr:uid="{A6FC6E94-2B4E-4D54-A8D9-DDD5BE4E1D48}"/>
-    <hyperlink ref="B294" r:id="rId761" xr:uid="{E3090863-FEE2-497C-BB53-F8655E307C46}"/>
-    <hyperlink ref="L294" r:id="rId762" xr:uid="{C55B7CCB-605F-440A-A810-34AEBDE0865F}"/>
-    <hyperlink ref="B295" r:id="rId763" xr:uid="{45680AA4-9BF7-424A-A802-FA31299989DC}"/>
-    <hyperlink ref="L295" r:id="rId764" xr:uid="{B4F3EE83-4742-46C9-B1B6-ED1FBB8E5442}"/>
-    <hyperlink ref="M295" r:id="rId765" xr:uid="{B1FB1B27-D637-400A-B979-EE5823E8FA5E}"/>
-    <hyperlink ref="B296" r:id="rId766" xr:uid="{E96482B9-35B3-4F57-B5AC-0F66FA509B21}"/>
-    <hyperlink ref="L296" r:id="rId767" xr:uid="{A00C9E83-F145-4F30-B5C3-A42A2D01A238}"/>
-    <hyperlink ref="B297" r:id="rId768" xr:uid="{D439E693-BDAF-4C06-8B32-E189901BAC94}"/>
-    <hyperlink ref="L297" r:id="rId769" xr:uid="{BCDC65C6-1612-40D5-9534-A258B2C7EFA1}"/>
-    <hyperlink ref="B298" r:id="rId770" xr:uid="{71D7FFB1-485D-4859-9336-93C9C4780EBB}"/>
-    <hyperlink ref="L298" r:id="rId771" xr:uid="{279D2CFD-FF43-4261-8C74-592205401530}"/>
-    <hyperlink ref="B299" r:id="rId772" xr:uid="{A357A92C-156B-4B26-9AFA-ECF073D20D54}"/>
-    <hyperlink ref="L299" r:id="rId773" xr:uid="{CC48CA00-9013-4823-8F8F-7538FEEBFA04}"/>
-    <hyperlink ref="B300" r:id="rId774" xr:uid="{C548B3EB-C0B3-47D5-8580-58D946A278D1}"/>
-    <hyperlink ref="L300" r:id="rId775" xr:uid="{152360BE-78FC-4A37-9AA6-B6C71F661A7C}"/>
-    <hyperlink ref="B301" r:id="rId776" xr:uid="{4BB5F494-A7B6-42A1-B780-F94B086C7E02}"/>
-    <hyperlink ref="L301" r:id="rId777" xr:uid="{90568678-CB1E-4B24-BDFF-1CA2065048FC}"/>
-    <hyperlink ref="B302" r:id="rId778" xr:uid="{1A96C1B7-49A8-46D2-82AB-154189F9E9F2}"/>
-    <hyperlink ref="H302" r:id="rId779" xr:uid="{029A42E1-F7C7-406E-A0B5-EE864E037D38}"/>
-    <hyperlink ref="L302" r:id="rId780" xr:uid="{B752614D-5393-4A60-B74D-345839537D40}"/>
-    <hyperlink ref="M302" r:id="rId781" xr:uid="{2055D406-F226-4294-880C-52A2AF8B5B94}"/>
-    <hyperlink ref="B303" r:id="rId782" xr:uid="{63A73073-5C53-4BD5-AC75-FF100B416E3F}"/>
-    <hyperlink ref="L303" r:id="rId783" xr:uid="{04A22A50-885F-42FD-8A74-9A31605B8D90}"/>
-    <hyperlink ref="B304" r:id="rId784" xr:uid="{B44A91C7-0348-4D3F-91BC-F9A90E45F16D}"/>
-    <hyperlink ref="L304" r:id="rId785" xr:uid="{85DC1A57-24A2-42BF-81F4-14A4D74CA782}"/>
-    <hyperlink ref="B305" r:id="rId786" xr:uid="{6E722D22-19AD-4E63-B691-DCA073188457}"/>
-    <hyperlink ref="L305" r:id="rId787" xr:uid="{381B695D-7CE8-4968-AF55-4175CCE6C783}"/>
-    <hyperlink ref="B306" r:id="rId788" xr:uid="{5833FE5F-EBFA-4BCC-9582-F291F7523DF3}"/>
-    <hyperlink ref="L306" r:id="rId789" xr:uid="{52040664-E133-410C-BEB8-80B6EFB632E8}"/>
-    <hyperlink ref="B307" r:id="rId790" xr:uid="{EB800E5E-3D46-4C16-A416-8824E8DBE4DD}"/>
-    <hyperlink ref="L307" r:id="rId791" xr:uid="{BF55F48F-1F42-4923-A56A-1894227D4EE9}"/>
-    <hyperlink ref="B308" r:id="rId792" xr:uid="{29AEE466-B810-410C-A1A2-C48404D52CCC}"/>
-    <hyperlink ref="L308" r:id="rId793" xr:uid="{3755AE80-5393-41A5-A233-858EAFB6802A}"/>
-    <hyperlink ref="B309" r:id="rId794" xr:uid="{94EEA286-B96E-4E55-9DAF-CCC5B5F6C620}"/>
-    <hyperlink ref="L309" r:id="rId795" xr:uid="{940210F1-3707-44ED-A98A-6C9EA174C789}"/>
-    <hyperlink ref="B310" r:id="rId796" xr:uid="{61BCCF97-20C7-466E-BFBB-295113572489}"/>
-    <hyperlink ref="L310" r:id="rId797" xr:uid="{E965EA06-32F1-4C98-831A-781416F083E7}"/>
-    <hyperlink ref="B311" r:id="rId798" xr:uid="{F57A4F2F-43F8-451C-B6E7-5FFC78C42A4E}"/>
-    <hyperlink ref="L311" r:id="rId799" xr:uid="{2439800C-7A66-44D6-AA8A-BD11C8B94AC5}"/>
-    <hyperlink ref="B312" r:id="rId800" xr:uid="{348576AA-9B6E-4FAA-A69F-04B6758CAA24}"/>
-    <hyperlink ref="L312" r:id="rId801" xr:uid="{0BFAD038-EF74-472B-80C3-F5EF6886EA23}"/>
-    <hyperlink ref="B313" r:id="rId802" xr:uid="{63A5BFA0-46AD-4B68-ACBF-C51D35F3F952}"/>
-    <hyperlink ref="L313" r:id="rId803" xr:uid="{A20BFDE4-8695-4D72-9781-C1A6C2A8EBCA}"/>
-    <hyperlink ref="B314" r:id="rId804" xr:uid="{C7277333-4315-4D1D-95E2-2CD40F6D3BB8}"/>
-    <hyperlink ref="L314" r:id="rId805" xr:uid="{ECD6F71A-339D-4B4A-8142-F1B1F3CC21B3}"/>
-    <hyperlink ref="B315" r:id="rId806" xr:uid="{0C9C22D7-DA73-4167-BF05-5EF2FCA343DB}"/>
-    <hyperlink ref="L315" r:id="rId807" xr:uid="{59CC0917-25B4-42D4-885C-9663FA00B470}"/>
-    <hyperlink ref="B316" r:id="rId808" xr:uid="{A5048730-B54C-47D3-BBA0-B98C393153F3}"/>
-    <hyperlink ref="L316" r:id="rId809" xr:uid="{9CC7CCB9-58F8-4B4F-BD87-0638262CF73F}"/>
-    <hyperlink ref="M316" r:id="rId810" xr:uid="{B721AA78-EFA8-46E9-88FD-92573EEC0E72}"/>
-    <hyperlink ref="B317" r:id="rId811" xr:uid="{E006BC11-A768-400C-B01A-5409BD4F7B6D}"/>
-    <hyperlink ref="L317" r:id="rId812" xr:uid="{C965C958-9A43-4D17-88C6-07A1068795D1}"/>
-    <hyperlink ref="M317" r:id="rId813" xr:uid="{EB7C8B38-A8FE-4A86-AA51-FB2F14251574}"/>
-    <hyperlink ref="B318" r:id="rId814" xr:uid="{6C00FB19-15DC-419D-B142-C394FC324F8B}"/>
-    <hyperlink ref="L318" r:id="rId815" xr:uid="{B3B4FBC0-367A-4E94-9B03-41FCF0C1B983}"/>
-    <hyperlink ref="B319" r:id="rId816" xr:uid="{C36034D8-5C99-4A01-B259-A4238A6E3B22}"/>
-    <hyperlink ref="L319" r:id="rId817" xr:uid="{03DD33AB-AA5E-448F-88EA-55ACBF30BCBA}"/>
-    <hyperlink ref="B320" r:id="rId818" xr:uid="{9A384C42-8DF3-4EF2-B981-B4B25C4EEFFF}"/>
-    <hyperlink ref="E320" r:id="rId819" xr:uid="{6DECA3E2-4F0C-4D77-9AD5-0AB3804399D0}"/>
-    <hyperlink ref="L320" r:id="rId820" xr:uid="{444AAF75-7CBC-4E17-972B-535A1442A621}"/>
-    <hyperlink ref="M320" r:id="rId821" xr:uid="{4041C913-7212-40F0-8312-A32A58F7D58C}"/>
-    <hyperlink ref="B321" r:id="rId822" xr:uid="{35BFF45B-C5CC-4898-9AD5-8A4EA301B2F2}"/>
-    <hyperlink ref="L321" r:id="rId823" xr:uid="{39039707-6D6C-4879-A086-E6C589976C3A}"/>
-    <hyperlink ref="B322" r:id="rId824" xr:uid="{D6DF6545-4EFE-4161-9B72-11B2A30E8BC0}"/>
-    <hyperlink ref="L322" r:id="rId825" xr:uid="{4FEF1688-88C7-4375-9AF1-D31DCFC5D987}"/>
-    <hyperlink ref="B323" r:id="rId826" xr:uid="{CAA1E8CA-F98F-4FF3-BCD9-2BB0505EF6BA}"/>
-    <hyperlink ref="L323" r:id="rId827" xr:uid="{6779B435-B7FF-439C-AE93-43F2F2DCE5B5}"/>
-    <hyperlink ref="B324" r:id="rId828" xr:uid="{A0F1B2AB-CE16-444A-9F68-F0B266A5AB19}"/>
-    <hyperlink ref="L324" r:id="rId829" xr:uid="{7F69849E-1231-4D06-8AF9-7116F8665284}"/>
-    <hyperlink ref="B325" r:id="rId830" xr:uid="{AD007161-9814-4FCE-BF68-575C7B7DC32E}"/>
-    <hyperlink ref="L325" r:id="rId831" xr:uid="{EF7046F1-4A4A-455E-993D-9051351D5FAB}"/>
-    <hyperlink ref="B326" r:id="rId832" xr:uid="{229313DF-5ED9-4AD2-8FF3-C66639E8626D}"/>
-    <hyperlink ref="L326" r:id="rId833" xr:uid="{9710FB42-86B3-4CD4-9239-87F0D691F8D7}"/>
-    <hyperlink ref="B327" r:id="rId834" xr:uid="{A588B2CA-AA85-4979-812D-259F20F3C006}"/>
-    <hyperlink ref="L327" r:id="rId835" xr:uid="{3FD2DFB8-5E5C-4C7C-883B-A88F27D5F417}"/>
-    <hyperlink ref="M327" r:id="rId836" xr:uid="{9CE8DB14-0676-4F19-9DC3-7AF821707B9A}"/>
-    <hyperlink ref="B328" r:id="rId837" xr:uid="{1823A5FE-ED91-4109-A946-EE22C0FC94CA}"/>
-    <hyperlink ref="L328" r:id="rId838" xr:uid="{ADF5D25D-70AB-4147-8404-BA2424882BDA}"/>
-    <hyperlink ref="B329" r:id="rId839" xr:uid="{3E81C955-070D-4995-AC76-878501C6BCF7}"/>
-    <hyperlink ref="L329" r:id="rId840" xr:uid="{1AF13AF2-937E-46E7-B96E-04F6E8ECD48D}"/>
-    <hyperlink ref="B330" r:id="rId841" xr:uid="{2B9812DB-AB2D-4C4E-AB11-D095AB903FA1}"/>
-    <hyperlink ref="L330" r:id="rId842" xr:uid="{680D3188-7189-44B5-AD7D-8F04A630EAE8}"/>
-    <hyperlink ref="B331" r:id="rId843" xr:uid="{8455D1B3-EC15-474B-8ED1-9522FC1F5704}"/>
-    <hyperlink ref="L331" r:id="rId844" xr:uid="{1AF76CD4-892E-46BB-A45F-F7C5DE932994}"/>
-    <hyperlink ref="B332" r:id="rId845" xr:uid="{4E9D52D3-18D8-478B-BC11-EC4ECB3A2671}"/>
-    <hyperlink ref="L332" r:id="rId846" xr:uid="{6440DE23-F3C7-4B84-B269-CEAD6F665D68}"/>
-    <hyperlink ref="B333" r:id="rId847" xr:uid="{EB153C62-EB52-4EAA-8F9D-B36E410091DE}"/>
-    <hyperlink ref="L333" r:id="rId848" xr:uid="{219D50E1-368C-4B51-961E-09C11829172F}"/>
-    <hyperlink ref="B334" r:id="rId849" xr:uid="{A2C65FC6-5EB2-4A7D-88C5-75A6BD0FB309}"/>
-    <hyperlink ref="L334" r:id="rId850" xr:uid="{E732B228-A084-4219-832A-7495921D5DC1}"/>
-    <hyperlink ref="B335" r:id="rId851" xr:uid="{29DB6A2A-B6F4-4CB4-9580-66E68162218F}"/>
-    <hyperlink ref="L335" r:id="rId852" xr:uid="{60F11405-EE36-4174-9471-17F07BE17055}"/>
-    <hyperlink ref="B336" r:id="rId853" xr:uid="{782D562D-CFA2-48F6-8F7D-8897B263EC4B}"/>
-    <hyperlink ref="L336" r:id="rId854" xr:uid="{B59BF701-27C4-447E-8D5A-4A3B498DCACA}"/>
-    <hyperlink ref="B337" r:id="rId855" xr:uid="{131CC98B-F42C-4727-8967-57EF34057BDF}"/>
-    <hyperlink ref="E337" r:id="rId856" xr:uid="{FED94E41-F199-4E8A-BF25-E9871A45E148}"/>
-    <hyperlink ref="L337" r:id="rId857" xr:uid="{95750179-A14B-44BA-898B-FCF9011148F7}"/>
-    <hyperlink ref="M337" r:id="rId858" xr:uid="{5AA5B4A1-7A44-4817-92BB-D267329B24BF}"/>
-    <hyperlink ref="B338" r:id="rId859" xr:uid="{59488B5A-500F-4B7D-B69D-E02FC3F67B52}"/>
-    <hyperlink ref="E338" r:id="rId860" xr:uid="{6D5772D8-58F8-4DE8-A169-622B123213E7}"/>
-    <hyperlink ref="L338" r:id="rId861" xr:uid="{4E6BFDEE-9219-4016-AE94-8B97B191AD92}"/>
-    <hyperlink ref="M338" r:id="rId862" xr:uid="{A95D3CAE-9F05-458A-AC47-0EFA0723E276}"/>
-    <hyperlink ref="B339" r:id="rId863" xr:uid="{813FCC30-CFC2-4FA5-9196-6EB8F3B60BF2}"/>
-    <hyperlink ref="L339" r:id="rId864" xr:uid="{0DD01132-A33E-49C3-9E3A-A5B79B87BEB4}"/>
-    <hyperlink ref="B340" r:id="rId865" xr:uid="{E55F37DE-CE86-4CB1-A730-2A89C81F1C88}"/>
-    <hyperlink ref="L340" r:id="rId866" xr:uid="{5C525523-555D-4B9B-AB8B-D36CCF1739A9}"/>
-    <hyperlink ref="B341" r:id="rId867" xr:uid="{97ED8F57-5258-435A-BC1C-F8574CBA0C61}"/>
-    <hyperlink ref="L341" r:id="rId868" xr:uid="{17B92131-AD77-4C68-AC6A-FAE26F2E0EE2}"/>
-    <hyperlink ref="B342" r:id="rId869" xr:uid="{2AF577C4-7A15-4558-AED1-817173E66859}"/>
-    <hyperlink ref="L342" r:id="rId870" xr:uid="{F6A9E531-7BB0-407D-941D-4305045E5AD7}"/>
-    <hyperlink ref="B343" r:id="rId871" xr:uid="{36E79DEF-D17B-4350-AA3D-1E821F20055D}"/>
-    <hyperlink ref="L343" r:id="rId872" xr:uid="{EBAE61F9-D826-4549-B7ED-6CAF997D1394}"/>
-    <hyperlink ref="M343" r:id="rId873" xr:uid="{49DAAE8E-C5D4-4F0F-9394-0B04ED6A6E80}"/>
-    <hyperlink ref="B344" r:id="rId874" xr:uid="{8DDAF625-92DD-4F06-A368-470ED7AB9F99}"/>
-    <hyperlink ref="L344" r:id="rId875" xr:uid="{D129FB27-2B56-4257-9540-AF10CE5DE9BD}"/>
-    <hyperlink ref="B345" r:id="rId876" xr:uid="{3AC395B2-3CC5-4C45-B7D7-20B6009C15EE}"/>
-    <hyperlink ref="L345" r:id="rId877" xr:uid="{01ECC367-079C-45CD-B36C-CC6A8C03432A}"/>
-    <hyperlink ref="M345" r:id="rId878" xr:uid="{B7A699FC-2C11-44B8-92E6-46A38C75C241}"/>
-    <hyperlink ref="B346" r:id="rId879" xr:uid="{BE6B5648-5096-4640-A8DD-C78CBCFEA970}"/>
-    <hyperlink ref="L346" r:id="rId880" xr:uid="{D88AA394-F934-48A3-A469-45296A33ABAE}"/>
-    <hyperlink ref="M346" r:id="rId881" xr:uid="{32EEE138-1A1F-44AA-87C9-49CFB89F4C03}"/>
-    <hyperlink ref="B347" r:id="rId882" xr:uid="{8C02A91D-7FB1-42D5-B03E-4736577EF33C}"/>
-    <hyperlink ref="L347" r:id="rId883" xr:uid="{2337E378-62AC-4336-BEE3-8E2FE1DBA638}"/>
-    <hyperlink ref="M347" r:id="rId884" xr:uid="{3B43AC28-4D6B-4E88-9DB9-7D69B28E2D9C}"/>
-    <hyperlink ref="B348" r:id="rId885" xr:uid="{E8F250DF-FEFE-4FE8-ACE2-600EE1DC619E}"/>
-    <hyperlink ref="L348" r:id="rId886" xr:uid="{9CFD079D-E4B2-41FE-A646-6C40D080EAC0}"/>
-    <hyperlink ref="M348" r:id="rId887" xr:uid="{6F22AB1F-EEEF-4840-8E51-D8F9A6EE30F8}"/>
-    <hyperlink ref="B349" r:id="rId888" xr:uid="{45611D30-9CC7-40B4-8AB0-3530929FCCB0}"/>
-    <hyperlink ref="L349" r:id="rId889" xr:uid="{4E4C3B28-DA66-4D10-A750-B1E8ADC09483}"/>
-    <hyperlink ref="B350" r:id="rId890" xr:uid="{2CAF6447-3C42-4114-B25B-D21BC34BFBB7}"/>
-    <hyperlink ref="L350" r:id="rId891" xr:uid="{E0F1049C-9982-40B1-A9C6-9FCA2DD9E933}"/>
-    <hyperlink ref="B351" r:id="rId892" xr:uid="{5098FEA9-1074-466C-B5FF-A5519ED92C30}"/>
-    <hyperlink ref="L351" r:id="rId893" xr:uid="{DC02BFB0-005C-4392-8537-42BE7CE9C4BA}"/>
-    <hyperlink ref="B352" r:id="rId894" xr:uid="{3104B8D0-9669-42DD-8243-9198BA1C0E78}"/>
-    <hyperlink ref="L352" r:id="rId895" xr:uid="{8B1DFD7E-4DA6-49E6-B58B-CCC813FDC140}"/>
-    <hyperlink ref="B353" r:id="rId896" xr:uid="{EF17063B-DE8D-4800-B3DC-2C2CE9F70AA0}"/>
-    <hyperlink ref="L353" r:id="rId897" xr:uid="{9A82B52E-735E-45A8-8D32-927023665A5E}"/>
-    <hyperlink ref="B354" r:id="rId898" xr:uid="{6E6CE124-5A49-4AC5-B8EE-CE8C63037674}"/>
-    <hyperlink ref="E354" r:id="rId899" xr:uid="{D55949F4-6244-49C7-9948-5B065E429CD1}"/>
-    <hyperlink ref="H354" r:id="rId900" xr:uid="{2F5FBA9A-84CD-42EF-B84F-778514A6A9CD}"/>
-    <hyperlink ref="L354" r:id="rId901" xr:uid="{AED2C38B-86F0-4EA8-8D16-FFF62809EFF2}"/>
-    <hyperlink ref="M354" r:id="rId902" xr:uid="{EA70C3F5-405D-48D5-9966-087295516E0A}"/>
-    <hyperlink ref="B355" r:id="rId903" xr:uid="{2F9A311B-7ABB-418C-BFF6-CCD804A17998}"/>
-    <hyperlink ref="L355" r:id="rId904" xr:uid="{C16911B0-76D4-413F-876C-C806EA6FCE21}"/>
-    <hyperlink ref="B356" r:id="rId905" xr:uid="{25D4809C-D224-4985-91BD-453ADB529277}"/>
-    <hyperlink ref="L356" r:id="rId906" xr:uid="{41281100-5D25-47E9-81AB-8895B908770E}"/>
-    <hyperlink ref="B357" r:id="rId907" xr:uid="{BBA78CAF-447A-43B2-95AB-60971B71E7CC}"/>
-    <hyperlink ref="L357" r:id="rId908" xr:uid="{0AE87E38-7453-4182-95EA-4C50555C85BE}"/>
-    <hyperlink ref="B358" r:id="rId909" xr:uid="{30E2DB0F-D78D-461D-8321-265FCD8E6E6B}"/>
-    <hyperlink ref="L358" r:id="rId910" xr:uid="{C5871C64-27AE-4D0C-88C7-32FBDDF12BCF}"/>
-    <hyperlink ref="B359" r:id="rId911" xr:uid="{04AF2955-1DCC-4CEF-B601-0CC899842578}"/>
-    <hyperlink ref="L359" r:id="rId912" xr:uid="{4C4CA128-88EB-4328-97C0-8200AF29EBBA}"/>
-    <hyperlink ref="B360" r:id="rId913" xr:uid="{4AD928AF-59F5-4FDB-B918-30156EB60357}"/>
-    <hyperlink ref="L360" r:id="rId914" xr:uid="{A3BD35F8-DAD1-4005-B1DB-1AD2DDB1BCD4}"/>
-    <hyperlink ref="B361" r:id="rId915" xr:uid="{0031D400-B6E1-400B-AD50-12F59EE7F831}"/>
-    <hyperlink ref="L361" r:id="rId916" xr:uid="{3EC34332-1141-4246-8344-8A4772D041AA}"/>
-    <hyperlink ref="B362" r:id="rId917" xr:uid="{3403AA25-E420-4B1D-909D-C649D14DC01B}"/>
-    <hyperlink ref="L362" r:id="rId918" xr:uid="{86900F56-34E9-487E-B0D6-DFA3CA9408B9}"/>
-    <hyperlink ref="B363" r:id="rId919" xr:uid="{A628A918-5521-43A3-8C63-1C48552DD48A}"/>
-    <hyperlink ref="L363" r:id="rId920" xr:uid="{C9D4F579-3FD6-4BBE-BC42-58525C21D8B7}"/>
-    <hyperlink ref="B364" r:id="rId921" xr:uid="{6BA1F5A0-813C-4EDD-B9F0-746266849E9C}"/>
-    <hyperlink ref="L364" r:id="rId922" xr:uid="{BABDC347-E6F5-452D-9869-5C9E7298A96C}"/>
-    <hyperlink ref="B365" r:id="rId923" xr:uid="{CD45DBD5-E235-49AB-ADFE-F2917F393AC7}"/>
-    <hyperlink ref="L365" r:id="rId924" xr:uid="{8064667C-FC51-49D7-AB76-DF72A5BAF98D}"/>
-    <hyperlink ref="B366" r:id="rId925" xr:uid="{817022B0-E937-4632-ADC4-4557B81B70E3}"/>
-    <hyperlink ref="L366" r:id="rId926" xr:uid="{5C557A41-1488-4C30-B690-C426275A09D0}"/>
-    <hyperlink ref="B367" r:id="rId927" xr:uid="{C98BD36C-924C-4231-974D-978767E0ED88}"/>
-    <hyperlink ref="L367" r:id="rId928" xr:uid="{DEC8B68D-FD22-4810-82FF-1D65F2EEA566}"/>
-    <hyperlink ref="B368" r:id="rId929" xr:uid="{5F77E08F-AB12-4A6A-AB70-82255721A4B0}"/>
-    <hyperlink ref="L368" r:id="rId930" xr:uid="{7AB1D353-DB6D-40CB-BD36-64E3D7F6D029}"/>
-    <hyperlink ref="B369" r:id="rId931" xr:uid="{EB5C600A-B763-4FDB-973F-3EA8FA986382}"/>
-    <hyperlink ref="L369" r:id="rId932" xr:uid="{19DD4D94-3758-410E-A0BF-B1AC080C802C}"/>
-    <hyperlink ref="B370" r:id="rId933" xr:uid="{DB177B6C-4D26-4847-9434-A6E387083BD6}"/>
-    <hyperlink ref="L370" r:id="rId934" xr:uid="{3457DAF6-A6A7-4C55-B063-C651AE18D00A}"/>
-    <hyperlink ref="M370" r:id="rId935" xr:uid="{034F2AA5-1B95-4489-B723-DEBF283F728F}"/>
-    <hyperlink ref="B371" r:id="rId936" xr:uid="{2C5A9851-B327-4155-B8F4-17E5D9C25740}"/>
-    <hyperlink ref="L371" r:id="rId937" xr:uid="{0095A0DB-8DE1-40C5-8F39-6276960E596E}"/>
-    <hyperlink ref="B372" r:id="rId938" xr:uid="{16BC92BE-F724-4613-9014-7BF1E8DCFAEA}"/>
-    <hyperlink ref="L372" r:id="rId939" xr:uid="{8A33E25B-2422-4672-B183-B954DED9C524}"/>
-    <hyperlink ref="B373" r:id="rId940" xr:uid="{A2B9F90B-E083-4DEA-934A-29175304F878}"/>
-    <hyperlink ref="L373" r:id="rId941" xr:uid="{826178DA-55A6-4FDA-9915-0F1A4BA26CBB}"/>
-    <hyperlink ref="B374" r:id="rId942" xr:uid="{351C5208-3CC4-455E-98BA-02C8C0A53809}"/>
-    <hyperlink ref="L374" r:id="rId943" xr:uid="{362C2CD9-9107-474D-9202-9C0A1B07FFE7}"/>
-    <hyperlink ref="B375" r:id="rId944" xr:uid="{7AE839E2-BADA-49EF-842F-924D891ABD46}"/>
-    <hyperlink ref="L375" r:id="rId945" xr:uid="{9C561199-709A-4F58-B2D8-38E9C9918C65}"/>
-    <hyperlink ref="B376" r:id="rId946" xr:uid="{EB66E1A0-5338-486D-9179-E4268BCCC256}"/>
-    <hyperlink ref="E376" r:id="rId947" xr:uid="{3E97F082-3542-4EB2-8682-7CD5CB2A649A}"/>
-    <hyperlink ref="L376" r:id="rId948" xr:uid="{702728CF-9F48-41D4-81CA-2A12E11AADED}"/>
-    <hyperlink ref="M376" r:id="rId949" xr:uid="{B6CC4249-DEFB-463A-A557-29B953FB1879}"/>
-    <hyperlink ref="B377" r:id="rId950" xr:uid="{6778221B-5B66-4F9A-9799-021823F246A1}"/>
-    <hyperlink ref="L377" r:id="rId951" xr:uid="{14F67A90-20B9-4A73-B731-31522A05C914}"/>
-    <hyperlink ref="B378" r:id="rId952" xr:uid="{99FA10D3-3713-4D67-8FB6-D46781F75E34}"/>
-    <hyperlink ref="E378" r:id="rId953" xr:uid="{53B7BFDB-1654-42AB-8F5B-B6FAB8D973A4}"/>
-    <hyperlink ref="L378" r:id="rId954" xr:uid="{744FFB7D-1770-431D-A95E-626F8DC6603B}"/>
-    <hyperlink ref="M378" r:id="rId955" xr:uid="{1086EADC-051B-48F4-AE2A-1BC7A87CBB17}"/>
-    <hyperlink ref="B379" r:id="rId956" xr:uid="{F40CF3AC-BC09-43C7-BD79-688C2260E9EA}"/>
-    <hyperlink ref="L379" r:id="rId957" xr:uid="{5179B5EC-5CC5-4632-B411-FEF43E1E9018}"/>
-    <hyperlink ref="B380" r:id="rId958" xr:uid="{290D4C3D-9105-4358-9F46-FD8C285D4B87}"/>
-    <hyperlink ref="E380" r:id="rId959" xr:uid="{8745217D-61F9-47FB-B2D1-6E630ED75303}"/>
-    <hyperlink ref="L380" r:id="rId960" xr:uid="{BC39068B-2F8F-49E5-BF2F-0AFDEFE308F6}"/>
-    <hyperlink ref="M380" r:id="rId961" xr:uid="{F8379860-6C81-4B1D-933A-0D767262DE16}"/>
-    <hyperlink ref="B381" r:id="rId962" xr:uid="{27B29DFF-164C-43BF-947E-91CA05C075B2}"/>
-    <hyperlink ref="E381" r:id="rId963" xr:uid="{C3ABC0F2-7452-47F7-AE57-221608CA9DC9}"/>
-    <hyperlink ref="L381" r:id="rId964" xr:uid="{4B7F1ADB-CB80-42F3-9AB8-C7C27C3AF4BE}"/>
-    <hyperlink ref="M381" r:id="rId965" xr:uid="{5E90A712-D586-4A20-BF49-7834AC72614A}"/>
-    <hyperlink ref="B382" r:id="rId966" xr:uid="{9BD8A54E-56E8-4317-B4F8-EF1885CA1A2D}"/>
-    <hyperlink ref="E382" r:id="rId967" xr:uid="{7FECE92A-F568-4BE1-9087-8E70E35D9339}"/>
-    <hyperlink ref="L382" r:id="rId968" xr:uid="{92779F7C-6629-457C-8D8F-67B9DA250228}"/>
-    <hyperlink ref="M382" r:id="rId969" xr:uid="{E35FCDE9-ABAD-4E95-B199-9B1CC9488475}"/>
-    <hyperlink ref="B383" r:id="rId970" xr:uid="{243634D9-CD6E-46AE-B047-FD895A4D2E76}"/>
-    <hyperlink ref="L383" r:id="rId971" xr:uid="{1C801412-4C92-41D3-9124-BCCFC5402BBA}"/>
-    <hyperlink ref="M383" r:id="rId972" xr:uid="{4AA5BBB6-D21C-4485-BCEC-85D1BE06A4A5}"/>
-    <hyperlink ref="B384" r:id="rId973" xr:uid="{3532AD8B-279B-48F2-B91E-292CB5646683}"/>
-    <hyperlink ref="E384" r:id="rId974" xr:uid="{60DAE1A4-EF23-4CED-86F8-2396A2864F0F}"/>
-    <hyperlink ref="L384" r:id="rId975" xr:uid="{6B912680-42CF-40E4-A85D-CDB14C38170E}"/>
-    <hyperlink ref="M384" r:id="rId976" xr:uid="{00AC411E-3DCF-467A-A30B-939EB1E69095}"/>
-    <hyperlink ref="B385" r:id="rId977" xr:uid="{22ADA246-83EE-4259-8F4D-130A4DD811CA}"/>
-    <hyperlink ref="L385" r:id="rId978" xr:uid="{39F0E8E1-E629-4A90-BFEA-3E14160534FF}"/>
-    <hyperlink ref="B386" r:id="rId979" xr:uid="{F5478327-17F4-449A-82E1-B590E54B2783}"/>
-    <hyperlink ref="L386" r:id="rId980" xr:uid="{956173B2-EBCA-4D22-ABA4-37327AF8E68E}"/>
-    <hyperlink ref="B387" r:id="rId981" xr:uid="{672D5442-9628-41D5-A529-44DCEFC4F757}"/>
-    <hyperlink ref="L387" r:id="rId982" xr:uid="{083A5B99-4268-4AAA-97E4-0488A6AB39A4}"/>
-    <hyperlink ref="B388" r:id="rId983" xr:uid="{F3D8C133-BC2E-479A-A229-52F3FFAA8175}"/>
-    <hyperlink ref="L388" r:id="rId984" xr:uid="{469585C2-FD0B-4D20-AA62-89BB71C7F228}"/>
-    <hyperlink ref="B389" r:id="rId985" xr:uid="{D594604C-4D51-455D-9D5A-8078D68BD143}"/>
-    <hyperlink ref="L389" r:id="rId986" xr:uid="{ADB4E7C6-DFDB-4F58-9B3E-593F5459DF65}"/>
-    <hyperlink ref="B390" r:id="rId987" xr:uid="{CBCD07BC-AD09-45D6-A27D-FDAA49C2D802}"/>
-    <hyperlink ref="L390" r:id="rId988" xr:uid="{532D03B2-BEF1-4E10-9A60-1B826ECD7C49}"/>
-    <hyperlink ref="B391" r:id="rId989" xr:uid="{F40D7BE3-CF59-456B-A43E-650FF4B4FEE2}"/>
-    <hyperlink ref="L391" r:id="rId990" xr:uid="{832DC9E2-A30B-4719-988C-DA0AED4308C0}"/>
-    <hyperlink ref="B392" r:id="rId991" xr:uid="{4611FEF6-B29C-46BB-85D8-BA7D6B794A8B}"/>
-    <hyperlink ref="L392" r:id="rId992" xr:uid="{CB7EDF71-2FB0-4BD4-AA3A-5B40DB207D6F}"/>
-    <hyperlink ref="B393" r:id="rId993" xr:uid="{22AAD2D8-67E3-4B5E-8936-3A5023B55442}"/>
-    <hyperlink ref="L393" r:id="rId994" xr:uid="{489EF7FF-1E13-4FC0-863D-F3EEF5459133}"/>
-    <hyperlink ref="B394" r:id="rId995" xr:uid="{8A9A45C6-F43A-4B14-A648-B27F581FBC2B}"/>
-    <hyperlink ref="E394" r:id="rId996" xr:uid="{CC9EF82E-DDBE-445B-B4C3-73D4F1652A8A}"/>
-    <hyperlink ref="H394" r:id="rId997" xr:uid="{DADF5F12-5B85-4B9F-B04F-09549CEE9FF7}"/>
-    <hyperlink ref="L394" r:id="rId998" xr:uid="{2F0C7539-460B-4A06-BF6E-026FA930F786}"/>
-    <hyperlink ref="M394" r:id="rId999" xr:uid="{0F77CEEB-2180-4ED2-839B-9C8B7A787AB2}"/>
-    <hyperlink ref="B395" r:id="rId1000" xr:uid="{4AC88F30-24CC-4E5B-90C2-3666C24ABA02}"/>
-    <hyperlink ref="E395" r:id="rId1001" xr:uid="{1987F9AA-52C7-40B3-9A96-66D60E798D44}"/>
-    <hyperlink ref="H395" r:id="rId1002" xr:uid="{07C39093-83B7-4473-88BC-01F177F62C53}"/>
-    <hyperlink ref="L395" r:id="rId1003" xr:uid="{0F68ABA5-1618-4D58-8D3C-71247B7E3016}"/>
-    <hyperlink ref="M395" r:id="rId1004" xr:uid="{E1651F0E-715F-41A3-A79D-DDF04A804201}"/>
-    <hyperlink ref="B396" r:id="rId1005" xr:uid="{E73072EF-4787-4EE6-953E-CD67DB49411D}"/>
-    <hyperlink ref="E396" r:id="rId1006" xr:uid="{E458D893-5BA4-49F3-89A8-E16AB89E36E6}"/>
-    <hyperlink ref="H396" r:id="rId1007" xr:uid="{C7AAEF60-2D14-4DDD-9889-346EDCA4FE0C}"/>
-    <hyperlink ref="L396" r:id="rId1008" xr:uid="{D58DC8CC-7785-4D80-92FD-92D5C88541DD}"/>
-    <hyperlink ref="M396" r:id="rId1009" xr:uid="{D0B302C9-21F0-433F-89CD-0EF660864324}"/>
-    <hyperlink ref="B397" r:id="rId1010" xr:uid="{0E6563B5-9CCC-4186-BF03-B0458BC2AD43}"/>
-    <hyperlink ref="L397" r:id="rId1011" xr:uid="{17D665EE-AF7B-48BB-B3C5-70A95D503256}"/>
-    <hyperlink ref="B398" r:id="rId1012" xr:uid="{C2272FF2-BC95-4D0B-AE15-FCDE23542EF6}"/>
-    <hyperlink ref="L398" r:id="rId1013" xr:uid="{260C49C0-F9C0-472D-9168-508519F1B916}"/>
-    <hyperlink ref="B399" r:id="rId1014" xr:uid="{BCC30A6E-5DC9-4BED-918F-F0E7388A8965}"/>
-    <hyperlink ref="L399" r:id="rId1015" xr:uid="{35499119-2650-4B1B-A4E1-3893103D26B5}"/>
-    <hyperlink ref="B400" r:id="rId1016" xr:uid="{B51FF464-8879-4302-85D0-4328DE598BF3}"/>
-    <hyperlink ref="L400" r:id="rId1017" xr:uid="{55067F26-51E0-47C9-BC0D-32C29A967EDE}"/>
-    <hyperlink ref="B401" r:id="rId1018" xr:uid="{B31990F9-59B2-4937-88F4-689F0C762881}"/>
-    <hyperlink ref="L401" r:id="rId1019" xr:uid="{1C484D02-4F94-40E2-94A3-D512E2CBF585}"/>
-    <hyperlink ref="B402" r:id="rId1020" xr:uid="{E6B0C177-780F-48F7-BF2D-C9F2F5730C51}"/>
-    <hyperlink ref="L402" r:id="rId1021" xr:uid="{4FEFD263-F869-432E-89BF-34D7511A67DD}"/>
-    <hyperlink ref="B403" r:id="rId1022" xr:uid="{459A4E21-EB32-4965-B851-36588F837B11}"/>
-    <hyperlink ref="L403" r:id="rId1023" xr:uid="{DBB25638-55BC-4222-9ED6-707D6D4D9CEE}"/>
-    <hyperlink ref="B404" r:id="rId1024" xr:uid="{D9263EF4-1E64-4EF9-88D3-34714A7ADF33}"/>
-    <hyperlink ref="L404" r:id="rId1025" xr:uid="{DFB81E6D-904D-4410-91A9-BAFB216A9C6B}"/>
-    <hyperlink ref="B405" r:id="rId1026" xr:uid="{D7AC571C-FB7A-4E28-9239-02A77986C213}"/>
-    <hyperlink ref="L405" r:id="rId1027" xr:uid="{F6B453EB-707E-48CF-8C69-EE45722B2EDE}"/>
-    <hyperlink ref="B406" r:id="rId1028" xr:uid="{3188B92F-8D8D-4936-9FE0-3CC41A65FFC7}"/>
-    <hyperlink ref="E406" r:id="rId1029" xr:uid="{308A708B-2F2B-429B-BDF3-5D9376FD59A5}"/>
-    <hyperlink ref="L406" r:id="rId1030" xr:uid="{570F0B97-00C4-4085-893B-6BE3492C33EF}"/>
-    <hyperlink ref="M406" r:id="rId1031" xr:uid="{63115446-1851-4E61-A904-AC814505201C}"/>
-    <hyperlink ref="B407" r:id="rId1032" xr:uid="{398ABAEA-06A1-40EA-BDA9-FA2831D28323}"/>
-    <hyperlink ref="H407" r:id="rId1033" xr:uid="{D0E042FA-3940-4436-A9AD-DDB3EB50E3CE}"/>
-    <hyperlink ref="L407" r:id="rId1034" xr:uid="{5617C244-C398-4647-B820-1ADC90DE6B76}"/>
-    <hyperlink ref="M407" r:id="rId1035" xr:uid="{7F8821D0-B65E-478B-A22A-B265F5C545C9}"/>
-    <hyperlink ref="B408" r:id="rId1036" xr:uid="{8D5C614B-A34F-4628-B703-1DCD929BC8CA}"/>
-    <hyperlink ref="L408" r:id="rId1037" xr:uid="{0803681F-108D-48A2-80DE-8780877E574D}"/>
-    <hyperlink ref="B409" r:id="rId1038" xr:uid="{DADE1F3A-7B6D-4962-B4CF-AE115200CAF3}"/>
-    <hyperlink ref="E409" r:id="rId1039" xr:uid="{24E76EDE-FF18-4A32-A1E9-DAA573A2A91E}"/>
-    <hyperlink ref="H409" r:id="rId1040" xr:uid="{98DDE4BF-C3EF-44D2-8495-328DFDB7178E}"/>
-    <hyperlink ref="L409" r:id="rId1041" xr:uid="{0EE7F769-69CC-4F32-B117-BFC4E6B339F3}"/>
-    <hyperlink ref="M409" r:id="rId1042" xr:uid="{3CF51667-9DBE-4302-8DBA-F2AE7BFF0A01}"/>
-    <hyperlink ref="B410" r:id="rId1043" xr:uid="{DF0892B0-6BAE-4A7B-A6A3-34C2F5C19AF7}"/>
-    <hyperlink ref="L410" r:id="rId1044" xr:uid="{209EC956-5D54-4284-B00C-8DB55BED0F04}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{9E406534-5C6A-4C75-BD8F-4B7C41A368D6}"/>
+    <hyperlink ref="E2" r:id="rId2" xr:uid="{0A063659-E295-43A1-AF80-F6E6DE7ED72F}"/>
+    <hyperlink ref="L2" r:id="rId3" xr:uid="{763576C5-B768-4289-BB0B-E439A7562E68}"/>
+    <hyperlink ref="M2" r:id="rId4" xr:uid="{7C5B88EA-D338-4040-9CB5-A5B45B2A1B01}"/>
+    <hyperlink ref="B3" r:id="rId5" xr:uid="{FC74CA89-8418-4189-A345-A6E7E209BEC5}"/>
+    <hyperlink ref="L3" r:id="rId6" xr:uid="{E52AC851-560C-4679-88EA-CE0BD439FDD0}"/>
+    <hyperlink ref="M3" r:id="rId7" xr:uid="{2DFE0162-4A83-40D9-BA6A-BDBE7B968B4F}"/>
+    <hyperlink ref="B4" r:id="rId8" xr:uid="{8D1219C2-EECE-436D-8326-569100C96A9B}"/>
+    <hyperlink ref="L4" r:id="rId9" xr:uid="{BF5E9F73-6763-4438-8E4C-4C94936C5267}"/>
+    <hyperlink ref="B5" r:id="rId10" xr:uid="{206F7AC3-8953-407E-9B96-B9589B57C444}"/>
+    <hyperlink ref="E5" r:id="rId11" xr:uid="{82DC7E70-CA3B-4F46-9D8E-971159655AB9}"/>
+    <hyperlink ref="L5" r:id="rId12" xr:uid="{7EA3451B-DAF0-4BBD-A5B8-093F9B968584}"/>
+    <hyperlink ref="M5" r:id="rId13" xr:uid="{B11D5D13-EEAD-4352-8222-B2290B577317}"/>
+    <hyperlink ref="B6" r:id="rId14" xr:uid="{71F9322B-07F2-40F4-8699-7ED906A88122}"/>
+    <hyperlink ref="E6" r:id="rId15" xr:uid="{71A1A8AA-D7D9-4D33-BD2C-098104B607A3}"/>
+    <hyperlink ref="H6" r:id="rId16" xr:uid="{54E87FFC-8B92-4C85-AA56-ABE9683588EA}"/>
+    <hyperlink ref="L6" r:id="rId17" xr:uid="{A91A1891-8344-45CF-9B5C-0D37CBF19FE8}"/>
+    <hyperlink ref="M6" r:id="rId18" xr:uid="{5CE7A54D-1E97-4F87-82C0-656E371D2357}"/>
+    <hyperlink ref="B7" r:id="rId19" xr:uid="{04AC0497-D5C8-41CC-BF6F-E37B964056F2}"/>
+    <hyperlink ref="E7" r:id="rId20" xr:uid="{F424C30D-D8B8-4BF0-918A-D9A019C5244D}"/>
+    <hyperlink ref="H7" r:id="rId21" xr:uid="{5C28CA83-B1B9-4601-80F8-A8A312BF26FB}"/>
+    <hyperlink ref="L7" r:id="rId22" xr:uid="{F7A3CB2A-45AA-4E6F-B53F-889B81FD8B37}"/>
+    <hyperlink ref="M7" r:id="rId23" xr:uid="{DA7CC4DF-962D-4A34-B089-E5E5383A4948}"/>
+    <hyperlink ref="B8" r:id="rId24" xr:uid="{CC6C858F-FD74-47BA-91F4-C0C0D99B9F32}"/>
+    <hyperlink ref="L8" r:id="rId25" xr:uid="{E2C2A46B-9D71-4D98-982C-A5C1EE5786BB}"/>
+    <hyperlink ref="M8" r:id="rId26" xr:uid="{4D7AECDE-A203-4480-AC80-03355BE1C34F}"/>
+    <hyperlink ref="B9" r:id="rId27" xr:uid="{6EDBCF9A-9EB3-4022-8AA2-828C948D80EA}"/>
+    <hyperlink ref="E9" r:id="rId28" xr:uid="{923856CF-B745-4203-B8C9-C2207E00A4AE}"/>
+    <hyperlink ref="L9" r:id="rId29" xr:uid="{ABDEA780-6671-46DF-95F3-052E7F4A5E22}"/>
+    <hyperlink ref="M9" r:id="rId30" xr:uid="{2159A7BD-8989-4B7C-8B4B-95BBDC364BDB}"/>
+    <hyperlink ref="B10" r:id="rId31" xr:uid="{ED7F32CF-6F5E-40E5-8C7A-9711292DD6A6}"/>
+    <hyperlink ref="L10" r:id="rId32" xr:uid="{C7E6D5CF-7F2B-459A-8C0A-CE5EA22B996C}"/>
+    <hyperlink ref="B11" r:id="rId33" xr:uid="{5F33CBD5-A5AB-42BD-80AA-17FCC6300378}"/>
+    <hyperlink ref="E11" r:id="rId34" xr:uid="{E688DBD7-4DDB-4938-90B5-549E325514A4}"/>
+    <hyperlink ref="L11" r:id="rId35" xr:uid="{C2BD28AD-B12D-482C-8B4C-E86F201F92AF}"/>
+    <hyperlink ref="M11" r:id="rId36" xr:uid="{F691992C-C713-4405-91AA-FAEC85003F0B}"/>
+    <hyperlink ref="B12" r:id="rId37" xr:uid="{0E425A3C-29DA-4AB0-B70B-02DCC2403CED}"/>
+    <hyperlink ref="L12" r:id="rId38" xr:uid="{B29CA2D9-A7F2-4EAB-83CF-B164D8508CC5}"/>
+    <hyperlink ref="B13" r:id="rId39" xr:uid="{4BA5DA26-9425-4E6B-AC6E-C8558885FA67}"/>
+    <hyperlink ref="L13" r:id="rId40" xr:uid="{3DBFBBF5-AB45-4AB5-89E3-1740CA22E546}"/>
+    <hyperlink ref="B14" r:id="rId41" xr:uid="{BB4C8C8F-7214-4C62-97A0-2A44467AB51D}"/>
+    <hyperlink ref="L14" r:id="rId42" xr:uid="{96F602F4-A33B-4BB9-92E7-8A3213E0FE9C}"/>
+    <hyperlink ref="B15" r:id="rId43" xr:uid="{3D182CBB-787F-40BA-BAFC-151DF78BA65F}"/>
+    <hyperlink ref="L15" r:id="rId44" xr:uid="{8BD20B83-C3CE-4EF0-8044-0ED41A9F502C}"/>
+    <hyperlink ref="B16" r:id="rId45" xr:uid="{30B6F6D7-6260-44B0-B648-6B8E72AED096}"/>
+    <hyperlink ref="L16" r:id="rId46" xr:uid="{BDDE7425-5598-4E0C-9E30-165E695E5906}"/>
+    <hyperlink ref="B17" r:id="rId47" xr:uid="{C88B6327-07B3-45C0-9636-9489004252AF}"/>
+    <hyperlink ref="L17" r:id="rId48" xr:uid="{7E1F4568-42EC-4347-A9C4-70EAF7D6307C}"/>
+    <hyperlink ref="B18" r:id="rId49" xr:uid="{BF7E9465-19FC-425F-B19A-E39F083BA14F}"/>
+    <hyperlink ref="L18" r:id="rId50" xr:uid="{3DCD7A77-1993-4244-8E61-B1633A7D602F}"/>
+    <hyperlink ref="B19" r:id="rId51" xr:uid="{ED254229-C22E-4C98-BDC2-FA74ABE50FC5}"/>
+    <hyperlink ref="L19" r:id="rId52" xr:uid="{CC77D7E8-DE6C-4A8A-AE0F-D1724A0AF762}"/>
+    <hyperlink ref="B20" r:id="rId53" xr:uid="{7AF99B21-12E4-402F-AD91-8FB19FA78D2C}"/>
+    <hyperlink ref="L20" r:id="rId54" xr:uid="{7A755C41-9725-4B7D-AFB0-A60E40BDECFC}"/>
+    <hyperlink ref="M20" r:id="rId55" xr:uid="{40F351AB-6CA8-40F7-AD70-9589D5FD6E99}"/>
+    <hyperlink ref="B21" r:id="rId56" xr:uid="{71248D48-DB22-498B-9B1C-B417408635B8}"/>
+    <hyperlink ref="H21" r:id="rId57" xr:uid="{332F4548-E8EB-44E5-8919-91EF53E5FBD3}"/>
+    <hyperlink ref="L21" r:id="rId58" xr:uid="{2B3391FA-6561-4290-9D38-8CC0FF547084}"/>
+    <hyperlink ref="M21" r:id="rId59" xr:uid="{A5340BEE-CF6B-48F3-8FBD-E29953E4F1EE}"/>
+    <hyperlink ref="B22" r:id="rId60" xr:uid="{BAB7BDD0-8D96-470D-902D-8E92D3AB3C84}"/>
+    <hyperlink ref="L22" r:id="rId61" xr:uid="{5967FF9A-E293-4CB8-9F2D-FECA01320FFC}"/>
+    <hyperlink ref="B23" r:id="rId62" xr:uid="{013FAD88-2773-408D-B982-060F5453B7EE}"/>
+    <hyperlink ref="L23" r:id="rId63" xr:uid="{1781F5D9-916B-44DE-BD0D-B5D09C0C6BE0}"/>
+    <hyperlink ref="B24" r:id="rId64" xr:uid="{A1E26B50-B8A0-4BCC-8D87-6929E0388A0D}"/>
+    <hyperlink ref="L24" r:id="rId65" xr:uid="{FDF8F76E-CACB-454B-A209-8B5ED61E7096}"/>
+    <hyperlink ref="B25" r:id="rId66" xr:uid="{1C68C57B-0F91-4097-8D53-61B92544B452}"/>
+    <hyperlink ref="H25" r:id="rId67" xr:uid="{90BAA4DF-EA1E-4D8F-B2A9-D890A298B717}"/>
+    <hyperlink ref="L25" r:id="rId68" xr:uid="{BB02C2E8-9A74-4856-8F09-B547578F93E2}"/>
+    <hyperlink ref="M25" r:id="rId69" xr:uid="{797B32B1-40C2-4786-BCE6-ABD2211047A3}"/>
+    <hyperlink ref="B26" r:id="rId70" xr:uid="{D0ECE350-624A-44A1-9D4C-01025910DDD1}"/>
+    <hyperlink ref="L26" r:id="rId71" xr:uid="{A7B90601-D602-4E02-A5D3-CBCEC028932F}"/>
+    <hyperlink ref="B27" r:id="rId72" xr:uid="{7B3B2ED0-AF30-4326-8614-BF340294CAB1}"/>
+    <hyperlink ref="E27" r:id="rId73" xr:uid="{EE91CDB1-7D57-45A4-B684-FF39D55FF780}"/>
+    <hyperlink ref="L27" r:id="rId74" xr:uid="{377AC54A-BAC6-4DE3-8438-AC54F98C050E}"/>
+    <hyperlink ref="M27" r:id="rId75" xr:uid="{08265B08-5BA2-4A2F-880A-9D34BF0006D7}"/>
+    <hyperlink ref="B28" r:id="rId76" xr:uid="{9A69B06D-FB6A-42A3-8CED-BEA2E0488018}"/>
+    <hyperlink ref="L28" r:id="rId77" xr:uid="{82C65561-C691-4C1B-A054-F13DEF769686}"/>
+    <hyperlink ref="B29" r:id="rId78" xr:uid="{9223390D-8ADB-45C3-9EC2-5AE33204F8D9}"/>
+    <hyperlink ref="E29" r:id="rId79" xr:uid="{4918C2DE-94DE-451E-BE94-CFA395B0B92F}"/>
+    <hyperlink ref="L29" r:id="rId80" xr:uid="{2C94905E-5105-4075-A492-41D7D8A958E7}"/>
+    <hyperlink ref="M29" r:id="rId81" xr:uid="{8B0B3233-6D34-4A99-A0F7-CC40B4FF92FE}"/>
+    <hyperlink ref="B30" r:id="rId82" xr:uid="{FE54EFFD-B238-48E3-8A9E-F4D2AAB39CCC}"/>
+    <hyperlink ref="H30" r:id="rId83" xr:uid="{51BAA7E2-42FA-4061-98F4-03F4FA047D73}"/>
+    <hyperlink ref="L30" r:id="rId84" xr:uid="{F307697E-34B4-4470-84B8-F729EA57F168}"/>
+    <hyperlink ref="M30" r:id="rId85" xr:uid="{C54C68E5-D1C6-4023-87A0-9A922F618958}"/>
+    <hyperlink ref="B31" r:id="rId86" xr:uid="{240187A5-B3D2-48D4-A3FF-B715B76C2A16}"/>
+    <hyperlink ref="L31" r:id="rId87" xr:uid="{86291FD1-E7C7-414C-834A-A00B2AC48F9A}"/>
+    <hyperlink ref="B32" r:id="rId88" xr:uid="{9B590D07-E545-4773-B05E-F5477501E39F}"/>
+    <hyperlink ref="L32" r:id="rId89" xr:uid="{CB61A074-07BE-4940-8520-8446CEAEFFFC}"/>
+    <hyperlink ref="B33" r:id="rId90" xr:uid="{396A74CD-8584-419E-8B54-F40D60CFA842}"/>
+    <hyperlink ref="L33" r:id="rId91" xr:uid="{84A83B55-8857-4BBC-AB00-8085D9D174F4}"/>
+    <hyperlink ref="M33" r:id="rId92" xr:uid="{4A4F90A5-EF55-42D6-8664-4B1B81B05033}"/>
+    <hyperlink ref="B34" r:id="rId93" xr:uid="{1BACC41B-D37F-4524-9A9B-66B0D7C568DF}"/>
+    <hyperlink ref="E34" r:id="rId94" xr:uid="{61CD180A-36C8-49C7-84D6-7C84071CCCED}"/>
+    <hyperlink ref="L34" r:id="rId95" xr:uid="{41F7970D-08DB-4584-BB97-20843F6A7A9F}"/>
+    <hyperlink ref="M34" r:id="rId96" xr:uid="{3C5CF848-6779-4402-BB0D-CD5FD902DCBB}"/>
+    <hyperlink ref="B35" r:id="rId97" xr:uid="{055022B6-7C48-4BCC-92F8-6249A0723732}"/>
+    <hyperlink ref="E35" r:id="rId98" xr:uid="{7DC23EA2-70F2-470A-BFC7-136C59C04E44}"/>
+    <hyperlink ref="H35" r:id="rId99" xr:uid="{E1C8BC70-2817-4672-9F3A-0A5B30C52F33}"/>
+    <hyperlink ref="L35" r:id="rId100" xr:uid="{FEF1ADD8-9772-41F0-A1A9-DA3481345CEE}"/>
+    <hyperlink ref="M35" r:id="rId101" xr:uid="{31F8D451-2ACC-44E6-B2D0-540A10802CA9}"/>
+    <hyperlink ref="B36" r:id="rId102" xr:uid="{DD9977F4-AB8A-4DA9-9D55-925AC15C1D3F}"/>
+    <hyperlink ref="L36" r:id="rId103" xr:uid="{7A88A105-1C33-452E-9A71-BFC4D42AF527}"/>
+    <hyperlink ref="B37" r:id="rId104" xr:uid="{AC5D1D48-17B8-4738-BD7D-1B80C545B402}"/>
+    <hyperlink ref="L37" r:id="rId105" xr:uid="{282C3840-154C-452B-A06D-E99B1E05E4BA}"/>
+    <hyperlink ref="B38" r:id="rId106" xr:uid="{F5FF7C53-3784-4991-9AE5-AD8A4B8C140A}"/>
+    <hyperlink ref="L38" r:id="rId107" xr:uid="{E9930E32-BCA8-41E4-8F60-DC50DC649702}"/>
+    <hyperlink ref="M38" r:id="rId108" xr:uid="{5AC68E35-DD1C-43AB-BE7C-6C0028BEF7F1}"/>
+    <hyperlink ref="B39" r:id="rId109" xr:uid="{DE33B866-72B0-4A9D-AFFF-C35625226CF7}"/>
+    <hyperlink ref="L39" r:id="rId110" xr:uid="{BA0D2781-B1B1-403A-86BF-1616DD8D0AAA}"/>
+    <hyperlink ref="B40" r:id="rId111" xr:uid="{FE3D716B-66A7-44B7-92A7-7DD9558C0207}"/>
+    <hyperlink ref="L40" r:id="rId112" xr:uid="{49F67A40-B67B-47D4-9979-9E2CEC1AB310}"/>
+    <hyperlink ref="M40" r:id="rId113" xr:uid="{6494D02B-A29F-47B4-8416-794BB9F1DD2A}"/>
+    <hyperlink ref="B41" r:id="rId114" xr:uid="{A3125050-33DD-4FEF-96D8-5E202E45B495}"/>
+    <hyperlink ref="L41" r:id="rId115" xr:uid="{A13AAC53-E5A2-4CE5-8FC3-19B102BBD261}"/>
+    <hyperlink ref="B42" r:id="rId116" xr:uid="{962E967A-EE07-4677-A266-BA39AF9835CE}"/>
+    <hyperlink ref="E42" r:id="rId117" xr:uid="{9C9D1C13-3D38-41C2-ABA1-3EDF0F76AD06}"/>
+    <hyperlink ref="L42" r:id="rId118" xr:uid="{649724BC-1224-435B-95E0-8426A10FEB0C}"/>
+    <hyperlink ref="M42" r:id="rId119" xr:uid="{BB14836A-429B-4AA8-9B3B-048444B119EB}"/>
+    <hyperlink ref="B43" r:id="rId120" xr:uid="{1EF6E7D1-3B68-4997-814E-9A0D489AD0FA}"/>
+    <hyperlink ref="L43" r:id="rId121" xr:uid="{8B6FC391-544E-47C4-B36F-40CBBCA4A155}"/>
+    <hyperlink ref="B44" r:id="rId122" xr:uid="{2F10A07E-4CBF-4C84-B65A-76FAA9D7A065}"/>
+    <hyperlink ref="L44" r:id="rId123" xr:uid="{25A7FCAA-8579-4FEF-A827-220CFB4D0232}"/>
+    <hyperlink ref="M44" r:id="rId124" xr:uid="{3133FE4F-11A3-4460-A956-7725FBE91C0C}"/>
+    <hyperlink ref="B45" r:id="rId125" xr:uid="{3CD78345-7229-414C-8EA4-81A06C81199B}"/>
+    <hyperlink ref="L45" r:id="rId126" xr:uid="{1F38DAA9-5B6D-4162-BCC5-972A05D1DE79}"/>
+    <hyperlink ref="M45" r:id="rId127" xr:uid="{0126E413-7806-4F44-A1B1-A7433EF1814B}"/>
+    <hyperlink ref="B46" r:id="rId128" xr:uid="{C5A87C4D-FE17-4E55-98CE-88655BBD3097}"/>
+    <hyperlink ref="L46" r:id="rId129" xr:uid="{7BCC2B12-29BF-4EFB-AE4D-94C05E4D7567}"/>
+    <hyperlink ref="B47" r:id="rId130" xr:uid="{218173E6-6A1B-412E-808B-0B9C640FCE47}"/>
+    <hyperlink ref="L47" r:id="rId131" xr:uid="{A8726822-4181-445C-8E91-8E280AE09253}"/>
+    <hyperlink ref="B48" r:id="rId132" xr:uid="{D98CD911-28FC-447A-81A0-6BC52E303FCE}"/>
+    <hyperlink ref="E48" r:id="rId133" xr:uid="{69226A74-9C90-42E5-845D-960291E3324F}"/>
+    <hyperlink ref="L48" r:id="rId134" xr:uid="{07B48122-FF38-4876-B4D7-B36651CF56AB}"/>
+    <hyperlink ref="M48" r:id="rId135" xr:uid="{BBCBC964-46F6-4B94-99B5-10BF24E98055}"/>
+    <hyperlink ref="B49" r:id="rId136" xr:uid="{7B5B98C9-00C6-449D-868D-46A429162F79}"/>
+    <hyperlink ref="E49" r:id="rId137" xr:uid="{52D92823-071B-4228-B570-C7F420403A3F}"/>
+    <hyperlink ref="L49" r:id="rId138" xr:uid="{5702C887-E445-4383-94C4-87B73EE3F994}"/>
+    <hyperlink ref="M49" r:id="rId139" xr:uid="{0AE28B8D-ADFC-4A88-991B-165E9A7C18E6}"/>
+    <hyperlink ref="B50" r:id="rId140" xr:uid="{5D7F7905-B10D-4868-A203-4D14A1267DA0}"/>
+    <hyperlink ref="L50" r:id="rId141" xr:uid="{CCEC4E75-AEF2-46B1-9CA6-5771AD693060}"/>
+    <hyperlink ref="M50" r:id="rId142" xr:uid="{F08F50BA-D8C3-4EC1-92A4-DF0E51141B33}"/>
+    <hyperlink ref="B51" r:id="rId143" xr:uid="{EBB4351C-8514-4910-BDB7-1B70C1634F73}"/>
+    <hyperlink ref="L51" r:id="rId144" xr:uid="{8E2398F0-BDEC-4DB0-A77C-4CFEB81A3C81}"/>
+    <hyperlink ref="B52" r:id="rId145" xr:uid="{7170C07D-39B1-4CC1-9088-6CD0002D7E37}"/>
+    <hyperlink ref="L52" r:id="rId146" xr:uid="{4D958F1C-0531-4CCC-9FB0-AA56CA7517FC}"/>
+    <hyperlink ref="B53" r:id="rId147" xr:uid="{8D74CE62-FFE3-4DC4-97D9-A4C610663904}"/>
+    <hyperlink ref="L53" r:id="rId148" xr:uid="{E8FFE1B0-3159-4092-8453-E500A5328981}"/>
+    <hyperlink ref="B54" r:id="rId149" xr:uid="{5FF1E6F4-B953-4873-A6F8-2162E00118DC}"/>
+    <hyperlink ref="L54" r:id="rId150" xr:uid="{E8574B6E-3A26-468D-ADD6-3B634C527F9A}"/>
+    <hyperlink ref="B55" r:id="rId151" xr:uid="{1B22A3F5-5E67-434E-B90E-C047A4994787}"/>
+    <hyperlink ref="L55" r:id="rId152" xr:uid="{078A85F5-DA1B-4B40-9207-EBA821FF8F7F}"/>
+    <hyperlink ref="B56" r:id="rId153" xr:uid="{B46D7309-4DBF-47C1-97E6-ADC40CE95C77}"/>
+    <hyperlink ref="L56" r:id="rId154" xr:uid="{A3B1E4E7-E703-46CE-929F-92543F7B32A8}"/>
+    <hyperlink ref="M56" r:id="rId155" xr:uid="{62EC582E-8EA0-4C58-A9A8-C91D7A921A81}"/>
+    <hyperlink ref="B57" r:id="rId156" xr:uid="{D5CEBB34-17A4-4F98-BAD5-BB096BDB73CB}"/>
+    <hyperlink ref="E57" r:id="rId157" xr:uid="{06F1443E-BFEA-4EAD-863A-409856CD1F0D}"/>
+    <hyperlink ref="L57" r:id="rId158" xr:uid="{34DD3DED-E9B5-4077-95C3-369BF6262F77}"/>
+    <hyperlink ref="M57" r:id="rId159" xr:uid="{17381D50-DE8D-4D6E-A547-DB1426CE6862}"/>
+    <hyperlink ref="B58" r:id="rId160" xr:uid="{4DA6901E-9782-4DFF-B848-5861EE3AF3E2}"/>
+    <hyperlink ref="L58" r:id="rId161" xr:uid="{2FD64112-3CB8-4038-AE3B-2B7276714881}"/>
+    <hyperlink ref="M58" r:id="rId162" xr:uid="{2104595E-92E5-4670-874A-C799C87A9585}"/>
+    <hyperlink ref="B59" r:id="rId163" xr:uid="{164721A2-96A7-4E4C-B12B-CD777611D2DE}"/>
+    <hyperlink ref="L59" r:id="rId164" xr:uid="{BC1C48F3-CFA9-4901-9022-D8897134531F}"/>
+    <hyperlink ref="B60" r:id="rId165" xr:uid="{BEC47D67-73F9-4C95-AF4D-D59565D9719A}"/>
+    <hyperlink ref="E60" r:id="rId166" xr:uid="{6AF228E1-47D0-4201-82CC-04E9E90A87CE}"/>
+    <hyperlink ref="L60" r:id="rId167" xr:uid="{A9EBA3A3-5EDB-4032-B666-63D3E5CC3899}"/>
+    <hyperlink ref="M60" r:id="rId168" xr:uid="{7B97CB71-FA33-4AAE-B041-977EE194E514}"/>
+    <hyperlink ref="B61" r:id="rId169" xr:uid="{E7FEFA05-8D5F-4DFD-980C-5F04A9802EA6}"/>
+    <hyperlink ref="E61" r:id="rId170" xr:uid="{CADDED65-E534-4ABB-8BC0-2A3F7FC4F8CE}"/>
+    <hyperlink ref="H61" r:id="rId171" xr:uid="{E880D489-EA72-4222-BC60-093233F4D6DE}"/>
+    <hyperlink ref="L61" r:id="rId172" xr:uid="{5EF4F67B-9272-4CDC-9EB1-1AF35173DCC0}"/>
+    <hyperlink ref="M61" r:id="rId173" xr:uid="{27246677-C906-4A2D-9FC4-6CE448C5D9F0}"/>
+    <hyperlink ref="B62" r:id="rId174" xr:uid="{A7516A55-93A5-4F6E-A5FE-72438F9B0D41}"/>
+    <hyperlink ref="L62" r:id="rId175" xr:uid="{814C3C4E-327C-4B84-8600-887E78F5AA66}"/>
+    <hyperlink ref="B63" r:id="rId176" xr:uid="{E648D704-35C4-4C1C-90F3-8A80F1656AC3}"/>
+    <hyperlink ref="L63" r:id="rId177" xr:uid="{1723F499-D913-48CC-A9C0-26FE381D37C2}"/>
+    <hyperlink ref="B64" r:id="rId178" xr:uid="{C24D9948-5E59-45DC-9ACF-A89126189D84}"/>
+    <hyperlink ref="L64" r:id="rId179" xr:uid="{E71C5843-9F0D-432D-A014-29458B036B61}"/>
+    <hyperlink ref="B65" r:id="rId180" xr:uid="{54614A28-4C47-44FA-A77A-095FB6D0AB37}"/>
+    <hyperlink ref="E65" r:id="rId181" xr:uid="{ED4E3CB5-E4BC-4FAF-8371-57269604C592}"/>
+    <hyperlink ref="L65" r:id="rId182" xr:uid="{96A3CE32-F82C-4587-A3BC-AC62C6F47BD0}"/>
+    <hyperlink ref="M65" r:id="rId183" xr:uid="{8A73B789-3F81-4265-A357-DEDA1A557C32}"/>
+    <hyperlink ref="B66" r:id="rId184" xr:uid="{662D6D08-C3C6-46A0-8D8B-322FEB091F14}"/>
+    <hyperlink ref="L66" r:id="rId185" xr:uid="{25E07F3D-CDA8-4943-88A2-E968CF97767C}"/>
+    <hyperlink ref="B67" r:id="rId186" xr:uid="{02FE7E27-7CF2-4EA1-B77A-281D1BE4AEE9}"/>
+    <hyperlink ref="L67" r:id="rId187" xr:uid="{C0FBF7B5-D6EE-4872-B085-6811E7E5A581}"/>
+    <hyperlink ref="B68" r:id="rId188" xr:uid="{A80A692D-CDE0-4703-ADC0-F817EB4909D8}"/>
+    <hyperlink ref="L68" r:id="rId189" xr:uid="{6F919C11-2961-4E54-B0B9-B4D3F054C085}"/>
+    <hyperlink ref="B69" r:id="rId190" xr:uid="{CBF5F9D1-B388-48FC-BD9B-37F7CA8E191A}"/>
+    <hyperlink ref="L69" r:id="rId191" xr:uid="{30CE6CBC-6590-4CC6-B5A5-27C030059D7B}"/>
+    <hyperlink ref="B70" r:id="rId192" xr:uid="{B44B995A-934F-4520-AE85-8FE5B87CC35D}"/>
+    <hyperlink ref="L70" r:id="rId193" xr:uid="{B7165F9C-B7C9-4E9C-8A27-FA38D708B310}"/>
+    <hyperlink ref="B71" r:id="rId194" xr:uid="{30DF0C84-974A-4478-A712-1A6207E7C033}"/>
+    <hyperlink ref="L71" r:id="rId195" xr:uid="{AA3BD05B-8AAD-4FD0-BE20-F16EAD3267D4}"/>
+    <hyperlink ref="B72" r:id="rId196" xr:uid="{0A3F9502-A84B-4020-B668-20457B543C94}"/>
+    <hyperlink ref="L72" r:id="rId197" xr:uid="{A6A1EC1B-A7EC-477E-AEA4-9C16D113048C}"/>
+    <hyperlink ref="B73" r:id="rId198" xr:uid="{EA527177-BB64-41D2-88A6-C8930CF43529}"/>
+    <hyperlink ref="L73" r:id="rId199" xr:uid="{BA342355-C6D2-4382-8BC0-23514E81E861}"/>
+    <hyperlink ref="B74" r:id="rId200" xr:uid="{BE95DCD2-11D3-4D58-85DB-1F0C59EF8DAC}"/>
+    <hyperlink ref="L74" r:id="rId201" xr:uid="{3177546C-3182-435D-B952-6C8B87F92D7E}"/>
+    <hyperlink ref="B75" r:id="rId202" xr:uid="{0437185B-DF94-4C8B-B021-A4222765128A}"/>
+    <hyperlink ref="L75" r:id="rId203" xr:uid="{BFEF6E67-A99E-4B8C-98E4-1497BA50CF86}"/>
+    <hyperlink ref="B76" r:id="rId204" xr:uid="{19AF3DDB-2B75-4252-85D2-718EA8FDDF0D}"/>
+    <hyperlink ref="L76" r:id="rId205" xr:uid="{0FCDF16D-3E35-4B88-8470-EB49A4B6122D}"/>
+    <hyperlink ref="B77" r:id="rId206" xr:uid="{CE54B50E-DC97-4B9A-A645-BD1141D974C6}"/>
+    <hyperlink ref="L77" r:id="rId207" xr:uid="{57B183D7-EF20-47CD-9F1A-4ADF3966D457}"/>
+    <hyperlink ref="M77" r:id="rId208" xr:uid="{9CC3C677-54E9-4AA1-ABF4-69C4F6EB4108}"/>
+    <hyperlink ref="B78" r:id="rId209" xr:uid="{D8AD5709-46C3-4102-84CC-B85D8269FC0A}"/>
+    <hyperlink ref="L78" r:id="rId210" xr:uid="{78B721A4-C150-4F38-A16A-2B6A3B1D4E03}"/>
+    <hyperlink ref="B79" r:id="rId211" xr:uid="{54024431-0936-4C68-8BC4-6181FA66EED5}"/>
+    <hyperlink ref="L79" r:id="rId212" xr:uid="{91763AD2-B3A7-4D9D-ABEC-EC8F37957A02}"/>
+    <hyperlink ref="B80" r:id="rId213" xr:uid="{9E3D2300-E7EF-4CB4-B42B-0C025F49EC1C}"/>
+    <hyperlink ref="L80" r:id="rId214" xr:uid="{AB91536C-8BD2-4AC4-AF09-195A8CC94DCF}"/>
+    <hyperlink ref="B81" r:id="rId215" xr:uid="{92AA4345-4EFC-42CF-B332-6C743FB47515}"/>
+    <hyperlink ref="L81" r:id="rId216" xr:uid="{96796F42-6186-4C68-8CAB-19F276B8AE4B}"/>
+    <hyperlink ref="B82" r:id="rId217" xr:uid="{F076F69D-80DF-4D27-822E-A47E2BB69E17}"/>
+    <hyperlink ref="L82" r:id="rId218" xr:uid="{0CD8D744-2E73-4BEF-8C7F-0DEDBECBD9B1}"/>
+    <hyperlink ref="B83" r:id="rId219" xr:uid="{8AB7F24F-ABFE-4E9D-BB80-CE45871A3378}"/>
+    <hyperlink ref="E83" r:id="rId220" xr:uid="{C543846B-5032-4E2B-B395-0A194318BB42}"/>
+    <hyperlink ref="L83" r:id="rId221" xr:uid="{5A201157-4A3B-4F09-B085-4B7126A01716}"/>
+    <hyperlink ref="M83" r:id="rId222" xr:uid="{A389CA03-B714-44C0-9B0F-6CCB3D491A11}"/>
+    <hyperlink ref="B84" r:id="rId223" xr:uid="{9B051646-BAA3-49C2-92FB-B68016E338AD}"/>
+    <hyperlink ref="E84" r:id="rId224" xr:uid="{81F7C422-982F-454F-BB5F-27D20F83FF3D}"/>
+    <hyperlink ref="L84" r:id="rId225" xr:uid="{FDA4AEB2-808B-4E9A-9BA6-87BEE44F8656}"/>
+    <hyperlink ref="M84" r:id="rId226" xr:uid="{F02AC4C4-CA43-4DAC-BB09-369B6F5BEDDC}"/>
+    <hyperlink ref="B85" r:id="rId227" xr:uid="{0652EAB5-FD19-467C-BA6E-088A436815C9}"/>
+    <hyperlink ref="L85" r:id="rId228" xr:uid="{9274D0B4-E52D-4388-8BA8-98C0B0A8206E}"/>
+    <hyperlink ref="B86" r:id="rId229" xr:uid="{DE5963CB-FA01-4CFC-9E35-30A2D6CF1178}"/>
+    <hyperlink ref="L86" r:id="rId230" xr:uid="{715C3AD1-B2A0-4329-9B39-54B1496C944A}"/>
+    <hyperlink ref="B87" r:id="rId231" xr:uid="{B5671F09-F4D5-4F93-9A83-F4177DA94BC5}"/>
+    <hyperlink ref="L87" r:id="rId232" xr:uid="{7BB53861-9E38-4215-BC34-95FB1C16CEBA}"/>
+    <hyperlink ref="B88" r:id="rId233" xr:uid="{35AA0484-E1CE-42B2-95B2-B562161F8780}"/>
+    <hyperlink ref="L88" r:id="rId234" xr:uid="{5E43DAB8-CD90-4791-8953-54B505C56420}"/>
+    <hyperlink ref="B89" r:id="rId235" xr:uid="{D003C917-74C1-4B36-88FC-CAF2A839C5DB}"/>
+    <hyperlink ref="L89" r:id="rId236" xr:uid="{09E8236E-2CDE-4F5C-9630-63838C989D8B}"/>
+    <hyperlink ref="B90" r:id="rId237" xr:uid="{44363D30-A074-407B-A753-52FECFE298A3}"/>
+    <hyperlink ref="L90" r:id="rId238" xr:uid="{E94309EA-1906-4B48-8720-A50CB16D4B6E}"/>
+    <hyperlink ref="M90" r:id="rId239" xr:uid="{A92BA091-68EC-456F-A19D-42B8EA3FB3E0}"/>
+    <hyperlink ref="B91" r:id="rId240" xr:uid="{C3972285-5128-426A-9AA7-DF6B02CED9F2}"/>
+    <hyperlink ref="L91" r:id="rId241" xr:uid="{6D26D21B-801D-451E-B83E-ABC1368B397B}"/>
+    <hyperlink ref="M91" r:id="rId242" xr:uid="{49804460-A7F0-4649-8F8A-10CCBBB607AA}"/>
+    <hyperlink ref="B92" r:id="rId243" xr:uid="{FB565557-C3E6-46E5-B691-757D8D096F0E}"/>
+    <hyperlink ref="H92" r:id="rId244" xr:uid="{F0BB6689-C1AD-4DF1-87C2-264F5690919B}"/>
+    <hyperlink ref="L92" r:id="rId245" xr:uid="{894931C8-7AB8-4DB8-9D6A-0318618CA9D2}"/>
+    <hyperlink ref="M92" r:id="rId246" xr:uid="{12E08C47-BEA7-494F-AA1D-6B8327855F72}"/>
+    <hyperlink ref="B93" r:id="rId247" xr:uid="{0A80DEBB-B0BB-4AF0-898B-B7B078D0309A}"/>
+    <hyperlink ref="L93" r:id="rId248" xr:uid="{1E7C3465-8DF8-411C-8DAC-0806D3C5C566}"/>
+    <hyperlink ref="B94" r:id="rId249" xr:uid="{06A5AA2A-9F2F-48AA-9A6B-E8EDF02A5CEC}"/>
+    <hyperlink ref="H94" r:id="rId250" xr:uid="{ECAABECA-A677-40B8-AEF6-729E3BFFB514}"/>
+    <hyperlink ref="L94" r:id="rId251" xr:uid="{9174507B-82F9-49F0-9935-E5E10A76D2C0}"/>
+    <hyperlink ref="M94" r:id="rId252" xr:uid="{34F7DF51-C957-457B-9533-C295F8D654FA}"/>
+    <hyperlink ref="B95" r:id="rId253" xr:uid="{34B5038D-7C04-4209-8086-069F18A2BB4A}"/>
+    <hyperlink ref="E95" r:id="rId254" xr:uid="{624DE9EF-4946-4364-9034-ACDF5570B545}"/>
+    <hyperlink ref="L95" r:id="rId255" xr:uid="{26F74C9C-93FF-44BF-B325-E4BAA8741C5C}"/>
+    <hyperlink ref="M95" r:id="rId256" xr:uid="{19C0CE68-917B-42AB-8C34-0BB2D9DDBEE7}"/>
+    <hyperlink ref="B96" r:id="rId257" xr:uid="{B80445BD-47C8-4DA9-A0CD-64AB93DEB328}"/>
+    <hyperlink ref="L96" r:id="rId258" xr:uid="{C44A2EB8-42D6-4173-B2AE-33A82487461E}"/>
+    <hyperlink ref="B97" r:id="rId259" xr:uid="{85FB937A-8DC6-4AB0-85F9-767B09B30A5E}"/>
+    <hyperlink ref="L97" r:id="rId260" xr:uid="{FCEEC153-21C5-4394-890B-7868C3DB66DB}"/>
+    <hyperlink ref="B98" r:id="rId261" xr:uid="{1128E228-C487-4BA0-AC09-8DA3F7796952}"/>
+    <hyperlink ref="L98" r:id="rId262" xr:uid="{A46AF389-8FE1-4D65-9B8C-B4D628E10BAD}"/>
+    <hyperlink ref="B99" r:id="rId263" xr:uid="{269CC351-D051-482E-AFD9-1B2B8423AF7D}"/>
+    <hyperlink ref="E99" r:id="rId264" xr:uid="{8410433D-9B8B-4719-ACBE-8B4560F8107A}"/>
+    <hyperlink ref="L99" r:id="rId265" xr:uid="{766CB748-FA93-4D35-8DF3-E6BE0DDED0B9}"/>
+    <hyperlink ref="M99" r:id="rId266" xr:uid="{5BA1FDBD-09FE-47C1-BDBA-CA622EA532EA}"/>
+    <hyperlink ref="B100" r:id="rId267" xr:uid="{11A49F89-C0AF-4D1E-9BC8-5888B32A9C15}"/>
+    <hyperlink ref="L100" r:id="rId268" xr:uid="{AA010884-642C-4B68-80C0-4AB3AF2C465F}"/>
+    <hyperlink ref="B101" r:id="rId269" xr:uid="{F5A317F1-A7CD-4F3A-843D-CF8AC7B0C8DC}"/>
+    <hyperlink ref="L101" r:id="rId270" xr:uid="{7E5CABD4-2929-4556-80CD-F792F5B8A19D}"/>
+    <hyperlink ref="B102" r:id="rId271" xr:uid="{7DEDDB63-850C-41FB-ADE5-79EB74C95D37}"/>
+    <hyperlink ref="E102" r:id="rId272" xr:uid="{F447C5AE-0C4D-4C90-92F3-8F2F91B75E9B}"/>
+    <hyperlink ref="L102" r:id="rId273" xr:uid="{E71DD945-3C38-48C7-975C-CD8CD0DD5E54}"/>
+    <hyperlink ref="M102" r:id="rId274" xr:uid="{798CE5CB-3591-4989-A546-835AA085D1D2}"/>
+    <hyperlink ref="B103" r:id="rId275" xr:uid="{A22113A4-7D54-4BD4-819A-54497C6FE4D8}"/>
+    <hyperlink ref="L103" r:id="rId276" xr:uid="{F1545569-7BE1-4EDD-96FA-3788605F35D9}"/>
+    <hyperlink ref="M103" r:id="rId277" xr:uid="{432AC817-BB0A-45C9-83EA-1907124DD303}"/>
+    <hyperlink ref="B104" r:id="rId278" xr:uid="{308AD99A-F179-46C0-96CF-0A6DC795A0C1}"/>
+    <hyperlink ref="L104" r:id="rId279" xr:uid="{742B2B5B-B602-4433-8868-A087F271FD45}"/>
+    <hyperlink ref="B105" r:id="rId280" xr:uid="{7C84741F-CB8D-4B9B-BA49-39895F94B62D}"/>
+    <hyperlink ref="L105" r:id="rId281" xr:uid="{CA4A5F75-DB1B-460E-A4E0-A8C04C467D8F}"/>
+    <hyperlink ref="B106" r:id="rId282" xr:uid="{03044963-4A67-4335-B57C-08089508A2D9}"/>
+    <hyperlink ref="L106" r:id="rId283" xr:uid="{D7FE2E4F-0B42-4D9E-8C78-EA2DE3080142}"/>
+    <hyperlink ref="B107" r:id="rId284" xr:uid="{2A917957-D4FC-413A-98A3-967F5092F6A7}"/>
+    <hyperlink ref="L107" r:id="rId285" xr:uid="{73B1D3C4-50FF-463B-866C-E1354221E361}"/>
+    <hyperlink ref="M107" r:id="rId286" xr:uid="{FC2A4CF2-9DC1-448F-846A-5E9EACB812CF}"/>
+    <hyperlink ref="B108" r:id="rId287" xr:uid="{04DD23CD-9F6A-4EFF-83A2-2F37EBF4EC6C}"/>
+    <hyperlink ref="E108" r:id="rId288" xr:uid="{68D8E565-E272-4903-97C2-2190ACD8579F}"/>
+    <hyperlink ref="L108" r:id="rId289" xr:uid="{5AA7E8B8-2A57-480C-849D-978CEE6E1ADA}"/>
+    <hyperlink ref="M108" r:id="rId290" xr:uid="{5DC19380-B62C-4AAE-8EF9-5DB8A3D1B3AC}"/>
+    <hyperlink ref="B109" r:id="rId291" xr:uid="{604A305F-63B1-4898-80E1-311BFFCA5503}"/>
+    <hyperlink ref="H109" r:id="rId292" xr:uid="{9821BF9F-0184-4027-876D-415E1D8C5590}"/>
+    <hyperlink ref="L109" r:id="rId293" xr:uid="{7AAFC5F9-32BE-44BD-80C2-CB4824F074FB}"/>
+    <hyperlink ref="M109" r:id="rId294" xr:uid="{CE16C1FF-712B-42B9-8F60-686BF7E5919D}"/>
+    <hyperlink ref="B110" r:id="rId295" xr:uid="{6734C34F-28A3-40CC-8B7B-59B36E897CB7}"/>
+    <hyperlink ref="E110" r:id="rId296" xr:uid="{8484EAFB-C94D-4DE6-8CA8-0279A29C3E95}"/>
+    <hyperlink ref="L110" r:id="rId297" xr:uid="{4DFCE129-A22F-422C-BA39-C30BA6675AB6}"/>
+    <hyperlink ref="M110" r:id="rId298" xr:uid="{85FE4CD1-EAA6-4F10-8D31-9BBA3F4DF5F8}"/>
+    <hyperlink ref="B111" r:id="rId299" xr:uid="{790AB01C-FBFE-433C-962C-39250B4177CF}"/>
+    <hyperlink ref="L111" r:id="rId300" xr:uid="{9D3CFEBB-8465-4512-B714-20445C054B1A}"/>
+    <hyperlink ref="B112" r:id="rId301" xr:uid="{9B4FE3A7-E904-448F-A044-39F3F2FAC336}"/>
+    <hyperlink ref="L112" r:id="rId302" xr:uid="{17115DEC-2161-4302-B51F-40740B7B7886}"/>
+    <hyperlink ref="M112" r:id="rId303" xr:uid="{90B8DBBF-504C-4453-99E5-F1EC8AA71EBD}"/>
+    <hyperlink ref="B113" r:id="rId304" xr:uid="{F1FEC920-C46B-47F2-8959-C901E090ABFC}"/>
+    <hyperlink ref="L113" r:id="rId305" xr:uid="{3207284D-9543-4F1F-9F3D-03AB48005DB7}"/>
+    <hyperlink ref="B114" r:id="rId306" xr:uid="{1778CB9E-AF7A-492C-8B57-79DBD1B798F7}"/>
+    <hyperlink ref="L114" r:id="rId307" xr:uid="{7227BF0F-610A-4C98-A395-3E1D1E22C713}"/>
+    <hyperlink ref="M114" r:id="rId308" xr:uid="{90EC85F3-365C-4DF7-B924-81FFECB173C5}"/>
+    <hyperlink ref="B115" r:id="rId309" xr:uid="{FD37C651-529F-4155-B1CB-4CB4527FD0E9}"/>
+    <hyperlink ref="L115" r:id="rId310" xr:uid="{7A49B15D-9E83-4E86-BD71-E94FA69702F4}"/>
+    <hyperlink ref="B116" r:id="rId311" xr:uid="{9A25E9F2-E95D-4E41-90EE-AA13350D62C6}"/>
+    <hyperlink ref="L116" r:id="rId312" xr:uid="{3AC68BD8-E6DF-49DF-9CE7-B6A682A12950}"/>
+    <hyperlink ref="B117" r:id="rId313" xr:uid="{C38CA6D0-3858-46A9-8A71-980E742CC3A1}"/>
+    <hyperlink ref="L117" r:id="rId314" xr:uid="{8123D3E8-51E2-4335-A38D-EAF572E9996C}"/>
+    <hyperlink ref="B118" r:id="rId315" xr:uid="{CD7205BA-9678-4D0C-835D-09474F6DBEAE}"/>
+    <hyperlink ref="L118" r:id="rId316" xr:uid="{87DBC7B8-C042-4275-876A-0F3D535C1EF6}"/>
+    <hyperlink ref="M118" r:id="rId317" xr:uid="{1C6BCDA2-5E27-425B-868B-26650B7A0FB1}"/>
+    <hyperlink ref="B119" r:id="rId318" xr:uid="{D6A9995A-6C0A-4B75-AB80-27AE4EC06438}"/>
+    <hyperlink ref="L119" r:id="rId319" xr:uid="{1FCC2E87-ECBC-43D0-B922-3251B3CD8F24}"/>
+    <hyperlink ref="B120" r:id="rId320" xr:uid="{55BAB299-3BAB-43E3-B6F9-D1223A38410C}"/>
+    <hyperlink ref="H120" r:id="rId321" xr:uid="{8B65E204-024E-4449-BC0A-B766A122D5A5}"/>
+    <hyperlink ref="L120" r:id="rId322" xr:uid="{0FC21D94-A5D1-43D8-AA4A-DFF5858919DA}"/>
+    <hyperlink ref="M120" r:id="rId323" xr:uid="{76B89B00-10E6-44F2-8590-805C52C958DF}"/>
+    <hyperlink ref="B121" r:id="rId324" xr:uid="{DA478955-F48C-4A50-BB7D-EA27CAEA5715}"/>
+    <hyperlink ref="L121" r:id="rId325" xr:uid="{E3AAA419-77F3-411E-B7B4-4486DDC5640B}"/>
+    <hyperlink ref="B122" r:id="rId326" xr:uid="{2B4E4CAA-3F86-41C0-9E6B-B305412F4E1C}"/>
+    <hyperlink ref="E122" r:id="rId327" xr:uid="{9BCB4840-151C-497B-9AEE-E97B7D3D9FB0}"/>
+    <hyperlink ref="L122" r:id="rId328" xr:uid="{E2635B40-B144-45A4-9BFE-6167DF00548F}"/>
+    <hyperlink ref="M122" r:id="rId329" xr:uid="{E65B2842-9200-445E-99DA-52FA3B2C9C87}"/>
+    <hyperlink ref="B123" r:id="rId330" xr:uid="{0A16676D-02D8-4AE2-B043-7B4C456C88C6}"/>
+    <hyperlink ref="L123" r:id="rId331" xr:uid="{33DAF1C1-629D-49F0-8CC2-2967F9F2309C}"/>
+    <hyperlink ref="B124" r:id="rId332" xr:uid="{8B76DAE7-386B-4851-A707-5B1849D729EE}"/>
+    <hyperlink ref="L124" r:id="rId333" xr:uid="{6D43F41D-FA13-48C4-AC8B-49000E29B93C}"/>
+    <hyperlink ref="B125" r:id="rId334" xr:uid="{BED34F41-9503-4907-A111-65ED2665DBA5}"/>
+    <hyperlink ref="L125" r:id="rId335" xr:uid="{6E0D2C2F-FD9A-46D6-824E-DB21AC42853C}"/>
+    <hyperlink ref="B126" r:id="rId336" xr:uid="{A3B923A0-7C3B-4907-83B7-C0BDFE538645}"/>
+    <hyperlink ref="L126" r:id="rId337" xr:uid="{E0FC6040-1A86-4BBC-B2D2-817A3CB1D895}"/>
+    <hyperlink ref="B127" r:id="rId338" xr:uid="{F88BEDE1-88EA-4B53-96C6-381C6F99687A}"/>
+    <hyperlink ref="L127" r:id="rId339" xr:uid="{47FAA09E-0C53-4880-8F46-828AC124E356}"/>
+    <hyperlink ref="B128" r:id="rId340" xr:uid="{691A6D1E-1C3B-4C60-9B9D-E4BB6231A768}"/>
+    <hyperlink ref="L128" r:id="rId341" xr:uid="{29D2ADF8-CAD2-441F-A87F-805E41170E98}"/>
+    <hyperlink ref="B129" r:id="rId342" xr:uid="{8D82E149-D64D-4ADB-A377-E24F12E33B91}"/>
+    <hyperlink ref="E129" r:id="rId343" xr:uid="{CB35CD37-1914-4810-AEDD-E5DC6C2F8B49}"/>
+    <hyperlink ref="L129" r:id="rId344" xr:uid="{BA5DABF8-AC53-409E-8B2B-0FDF3C72C9A9}"/>
+    <hyperlink ref="M129" r:id="rId345" xr:uid="{D8092C27-9DCE-4425-9810-C72108BE81BC}"/>
+    <hyperlink ref="B130" r:id="rId346" xr:uid="{44097194-F6A0-434C-826C-41E72EB780FE}"/>
+    <hyperlink ref="L130" r:id="rId347" xr:uid="{EB632BFB-45DB-49CC-9A5E-F0A01528F6DA}"/>
+    <hyperlink ref="M130" r:id="rId348" xr:uid="{BE131254-DFD7-47D3-9F4D-2B5DD7B44F3E}"/>
+    <hyperlink ref="B131" r:id="rId349" xr:uid="{E8191F3F-0B97-4F3F-B7CD-5DFCEB143F98}"/>
+    <hyperlink ref="L131" r:id="rId350" xr:uid="{0DF2E7BB-6848-4515-B5D4-F5CB29668840}"/>
+    <hyperlink ref="M131" r:id="rId351" xr:uid="{F253F7D6-9E2F-44E3-807A-15202B84B6F3}"/>
+    <hyperlink ref="B132" r:id="rId352" xr:uid="{781AFC50-6747-45FA-90C6-4A8C9B7DF82B}"/>
+    <hyperlink ref="E132" r:id="rId353" xr:uid="{84233DA7-DD54-434D-BF79-30BDF57C4708}"/>
+    <hyperlink ref="L132" r:id="rId354" xr:uid="{A426A0E1-5DAD-48BF-920A-3622C5F7E289}"/>
+    <hyperlink ref="M132" r:id="rId355" xr:uid="{573DFFE1-6E31-452E-8303-E5F92DD5FE9E}"/>
+    <hyperlink ref="B133" r:id="rId356" xr:uid="{209FD39A-7CF1-4B24-8127-21479A6A04D4}"/>
+    <hyperlink ref="E133" r:id="rId357" xr:uid="{C10229BC-7EE1-43B2-AD3E-F09D2D21500C}"/>
+    <hyperlink ref="L133" r:id="rId358" xr:uid="{9183DF4F-7699-42C9-924A-62CC3AAA39C5}"/>
+    <hyperlink ref="M133" r:id="rId359" xr:uid="{26CBDFB7-AC6C-40DB-A257-5A2566D3B37A}"/>
+    <hyperlink ref="B134" r:id="rId360" xr:uid="{334EA26F-D75E-451A-922E-4E746A3789AF}"/>
+    <hyperlink ref="L134" r:id="rId361" xr:uid="{5A74EED8-3C3D-430D-BEA2-D2867E873BAE}"/>
+    <hyperlink ref="B135" r:id="rId362" xr:uid="{9F63F09B-BA32-4F43-9A20-1682F4E49501}"/>
+    <hyperlink ref="E135" r:id="rId363" xr:uid="{74B6B14D-16B4-4B0E-B858-E6BEAECBCBF6}"/>
+    <hyperlink ref="L135" r:id="rId364" xr:uid="{43EEE320-7C53-448D-8941-1BE567433668}"/>
+    <hyperlink ref="M135" r:id="rId365" xr:uid="{5758D511-52AE-4724-9A26-FDDBFD66E922}"/>
+    <hyperlink ref="B136" r:id="rId366" xr:uid="{0A7E2E38-06C6-4CD9-BF8B-46883ADD0E5E}"/>
+    <hyperlink ref="H136" r:id="rId367" xr:uid="{90EF23E2-C25C-4D3B-B5A1-07ACAD5BADC5}"/>
+    <hyperlink ref="L136" r:id="rId368" xr:uid="{166ACBBB-133D-4672-B015-5738F7691871}"/>
+    <hyperlink ref="M136" r:id="rId369" xr:uid="{DBF93BED-78F5-4293-A3EE-A83CD454BBE0}"/>
+    <hyperlink ref="B137" r:id="rId370" xr:uid="{8BCDC0B2-0FB8-4328-8931-1F08910214F3}"/>
+    <hyperlink ref="L137" r:id="rId371" xr:uid="{B26EC1A8-0AAB-4B23-A5F9-3E1DEFA691E2}"/>
+    <hyperlink ref="B138" r:id="rId372" xr:uid="{976B664E-9423-4D24-8CFC-69049A49AEBD}"/>
+    <hyperlink ref="L138" r:id="rId373" xr:uid="{D5D1591D-41D3-46B7-9C31-9142A2A6DD29}"/>
+    <hyperlink ref="B139" r:id="rId374" xr:uid="{EC6F3DF4-8E6F-4FDF-8CE0-0B8E6AB1EF74}"/>
+    <hyperlink ref="L139" r:id="rId375" xr:uid="{E9A1F47B-70CF-4538-82A2-22225A7E745A}"/>
+    <hyperlink ref="B140" r:id="rId376" xr:uid="{5BACC985-4728-4949-A7F9-721C763F49D9}"/>
+    <hyperlink ref="L140" r:id="rId377" xr:uid="{137C4AA0-7298-49CE-819C-02F6241B0C74}"/>
+    <hyperlink ref="B141" r:id="rId378" xr:uid="{19979693-648D-4779-A769-D1ED578A8AA6}"/>
+    <hyperlink ref="L141" r:id="rId379" xr:uid="{D580FF5F-BB93-4BDB-98AA-063CC01688F7}"/>
+    <hyperlink ref="B142" r:id="rId380" xr:uid="{8177367B-C5A7-4859-92C0-FA248930E8FC}"/>
+    <hyperlink ref="L142" r:id="rId381" xr:uid="{37676528-A534-4BB8-8FF5-7DA1C02F6DDC}"/>
+    <hyperlink ref="B143" r:id="rId382" xr:uid="{B6EE9A6C-AF54-4E37-BA49-9F448FE6DAF0}"/>
+    <hyperlink ref="L143" r:id="rId383" xr:uid="{BE720CFB-2B71-4559-8EA2-56D585858AC2}"/>
+    <hyperlink ref="B144" r:id="rId384" xr:uid="{180A7FB0-5FFF-4DB8-9ACE-243D4BE48D19}"/>
+    <hyperlink ref="L144" r:id="rId385" xr:uid="{6435734E-8813-4162-893A-EA230C1C300A}"/>
+    <hyperlink ref="B145" r:id="rId386" xr:uid="{2FF80965-EBA3-4087-9593-9299BF51BD98}"/>
+    <hyperlink ref="L145" r:id="rId387" xr:uid="{B197ED09-037A-4B53-8C1E-C0A9FBB754A4}"/>
+    <hyperlink ref="B146" r:id="rId388" xr:uid="{9FFE4E42-319D-41A5-BC20-83B871D60BBD}"/>
+    <hyperlink ref="L146" r:id="rId389" xr:uid="{1341FA50-A8AF-4434-9A46-1A049E2D38D5}"/>
+    <hyperlink ref="B147" r:id="rId390" xr:uid="{F5C57325-00F3-4FC7-A72A-5CC42B5FE02E}"/>
+    <hyperlink ref="L147" r:id="rId391" xr:uid="{16664CFF-9113-4DE2-84C2-9B983A13C154}"/>
+    <hyperlink ref="B148" r:id="rId392" xr:uid="{B6FBD92F-09E2-4BCD-9C22-D4F32DF46DF5}"/>
+    <hyperlink ref="L148" r:id="rId393" xr:uid="{9759C224-A819-4E38-8C44-512C8486F947}"/>
+    <hyperlink ref="B149" r:id="rId394" xr:uid="{5BDA7187-69AF-4DEF-9712-A526A5B61514}"/>
+    <hyperlink ref="L149" r:id="rId395" xr:uid="{EE6D38D4-1727-4196-A413-784E20FBEDDE}"/>
+    <hyperlink ref="B150" r:id="rId396" xr:uid="{FF34CD12-918F-4025-9D6A-26229262FBB0}"/>
+    <hyperlink ref="E150" r:id="rId397" xr:uid="{3249E8FC-367F-452A-B7A1-A3338A79D58C}"/>
+    <hyperlink ref="L150" r:id="rId398" xr:uid="{D0DB5826-9565-49F6-BEF0-4E56B780C398}"/>
+    <hyperlink ref="M150" r:id="rId399" xr:uid="{B8F5C709-048D-44FA-AC00-F1E512BA818F}"/>
+    <hyperlink ref="B151" r:id="rId400" xr:uid="{0246C020-D924-44A6-838C-9A753BE786EF}"/>
+    <hyperlink ref="L151" r:id="rId401" xr:uid="{E4402315-131C-4C72-B3B2-ECD0CE0B61CB}"/>
+    <hyperlink ref="B152" r:id="rId402" xr:uid="{64AA7270-DD87-46E8-8B3D-7EB7F6D54977}"/>
+    <hyperlink ref="L152" r:id="rId403" xr:uid="{131BB1CA-9933-41EC-83D8-F39F2FD9E2D5}"/>
+    <hyperlink ref="B153" r:id="rId404" xr:uid="{AC5303D3-710B-4697-A433-8101ECFB28BC}"/>
+    <hyperlink ref="L153" r:id="rId405" xr:uid="{82B128A8-77F6-4991-B35D-A62632D6930C}"/>
+    <hyperlink ref="B154" r:id="rId406" xr:uid="{4A6561DB-EE9E-480A-9214-D6736EA79168}"/>
+    <hyperlink ref="L154" r:id="rId407" xr:uid="{B67675D6-7C76-4FDA-90B3-D90B83CC89E5}"/>
+    <hyperlink ref="B155" r:id="rId408" xr:uid="{D8FDAFB9-0D80-43CA-B8B6-79F87328BAC3}"/>
+    <hyperlink ref="E155" r:id="rId409" xr:uid="{3CE0C2CF-B6D4-44CB-99AF-095B2B840121}"/>
+    <hyperlink ref="L155" r:id="rId410" xr:uid="{33D283E7-0324-4324-809D-F7B8C13F680D}"/>
+    <hyperlink ref="M155" r:id="rId411" xr:uid="{B17D94DE-CA84-4138-9938-201A109794B2}"/>
+    <hyperlink ref="B156" r:id="rId412" xr:uid="{2F09671B-A4C9-4173-A9EB-51785C567371}"/>
+    <hyperlink ref="L156" r:id="rId413" xr:uid="{E26FCCBC-94DC-4850-823F-EE7477DDAFB7}"/>
+    <hyperlink ref="B157" r:id="rId414" xr:uid="{4012317D-1392-490C-96AA-7292578D50DE}"/>
+    <hyperlink ref="L157" r:id="rId415" xr:uid="{BD3AD8CA-C8E3-453C-BBD3-9E753673B603}"/>
+    <hyperlink ref="M157" r:id="rId416" xr:uid="{DD984BD5-2DD2-4DAF-808F-8E9136139114}"/>
+    <hyperlink ref="B158" r:id="rId417" xr:uid="{DDF5AD87-08BD-4824-AC9D-7F1A1A081D5B}"/>
+    <hyperlink ref="L158" r:id="rId418" xr:uid="{E49AF3ED-E8C5-4DDF-9667-32F4D05175DA}"/>
+    <hyperlink ref="B159" r:id="rId419" xr:uid="{51530AA9-0FF4-431A-8904-91C888D0A560}"/>
+    <hyperlink ref="H159" r:id="rId420" xr:uid="{FDFDF3BB-3604-406F-896E-F56801D1A4BF}"/>
+    <hyperlink ref="L159" r:id="rId421" xr:uid="{DF8506BF-414E-4E2A-974B-4873A327A2C1}"/>
+    <hyperlink ref="M159" r:id="rId422" xr:uid="{508EAFAF-7D07-4B05-B239-88C4E68E2650}"/>
+    <hyperlink ref="B160" r:id="rId423" xr:uid="{B5E036CC-23C8-4CA0-8885-35A5A833018D}"/>
+    <hyperlink ref="L160" r:id="rId424" xr:uid="{043A8F42-5B55-4A08-923B-03BBEB45592F}"/>
+    <hyperlink ref="B161" r:id="rId425" xr:uid="{AEDB6E6F-4912-431F-8F87-6FB416ACEA88}"/>
+    <hyperlink ref="L161" r:id="rId426" xr:uid="{5E594E27-BD99-4689-9065-15BD603D6F59}"/>
+    <hyperlink ref="B162" r:id="rId427" xr:uid="{D1A62A6B-8BC9-49D9-8B21-D2366EF7AD97}"/>
+    <hyperlink ref="L162" r:id="rId428" xr:uid="{A35775B7-D283-477E-A86B-E2D2ECEFEF85}"/>
+    <hyperlink ref="B163" r:id="rId429" xr:uid="{A8167B6D-396A-413A-B8D7-261CB873D6B7}"/>
+    <hyperlink ref="E163" r:id="rId430" xr:uid="{9F6BD7D5-1626-482B-9DD9-398B032D8258}"/>
+    <hyperlink ref="L163" r:id="rId431" xr:uid="{3F79BA84-5F64-41EE-BA2F-7515219147E4}"/>
+    <hyperlink ref="M163" r:id="rId432" xr:uid="{7175EDED-0C3E-4388-B238-45C48BF2AD14}"/>
+    <hyperlink ref="B164" r:id="rId433" xr:uid="{A08F2156-7C99-4572-BCDA-E18D76CC638C}"/>
+    <hyperlink ref="L164" r:id="rId434" xr:uid="{786D928A-BB29-4741-9CD1-261FC0DDBFD8}"/>
+    <hyperlink ref="M164" r:id="rId435" xr:uid="{0AF30E1D-0B25-494A-A4AA-CCDE0DAEEA90}"/>
+    <hyperlink ref="B165" r:id="rId436" xr:uid="{6A8670DE-34BF-4917-8204-006AA3EFE12E}"/>
+    <hyperlink ref="L165" r:id="rId437" xr:uid="{7853DA1F-7779-4006-85D0-570E28D3B42C}"/>
+    <hyperlink ref="B166" r:id="rId438" xr:uid="{3B843F50-5B06-40E4-A1C5-16FC03694C7F}"/>
+    <hyperlink ref="L166" r:id="rId439" xr:uid="{3FFB8682-B454-4742-BDF9-6C960904DB3B}"/>
+    <hyperlink ref="B167" r:id="rId440" xr:uid="{535239C1-BF86-4256-ADAC-A4D91DEDD80F}"/>
+    <hyperlink ref="L167" r:id="rId441" xr:uid="{CE8D930F-761D-45EF-80DF-9C36B4F3744C}"/>
+    <hyperlink ref="M167" r:id="rId442" xr:uid="{A3AC04A7-6CF8-4DB9-9A60-DFF2E9C7CD16}"/>
+    <hyperlink ref="B168" r:id="rId443" xr:uid="{AA8190A8-242A-4518-B9E9-AAAF3942A191}"/>
+    <hyperlink ref="L168" r:id="rId444" xr:uid="{3E50A816-172A-4F7E-ACD1-F107DE3DE0ED}"/>
+    <hyperlink ref="B169" r:id="rId445" xr:uid="{8C47B137-FF80-4AEC-9F61-7A72382213C6}"/>
+    <hyperlink ref="E169" r:id="rId446" xr:uid="{CD218DB8-79A9-4913-9A4A-95E72782BC0C}"/>
+    <hyperlink ref="L169" r:id="rId447" xr:uid="{DCEC2DFB-E8FB-4D96-958D-51039299A19E}"/>
+    <hyperlink ref="M169" r:id="rId448" xr:uid="{A152DEAF-8C4C-4A61-8337-9E0F1C4B4B42}"/>
+    <hyperlink ref="B170" r:id="rId449" xr:uid="{36458AA8-C5DE-400A-97B7-E4F4B9F2D479}"/>
+    <hyperlink ref="L170" r:id="rId450" xr:uid="{920562C7-88E3-460E-A78C-F1B4D60C6697}"/>
+    <hyperlink ref="B171" r:id="rId451" xr:uid="{77D510FA-BE69-454E-8D9A-5BEBB6879CDD}"/>
+    <hyperlink ref="L171" r:id="rId452" xr:uid="{DFD6E319-9B44-458F-A9FE-435943B4C938}"/>
+    <hyperlink ref="B172" r:id="rId453" xr:uid="{5B3ABDBD-EAF2-4873-A753-83FF30ECBB46}"/>
+    <hyperlink ref="L172" r:id="rId454" xr:uid="{13024876-5E3C-4F4C-9837-F2D387C107AE}"/>
+    <hyperlink ref="B173" r:id="rId455" xr:uid="{5F2DF95C-EF02-4AC1-99DA-F260B808DCF8}"/>
+    <hyperlink ref="E173" r:id="rId456" xr:uid="{B7981DF3-FD75-4FBB-84F8-B312205732BB}"/>
+    <hyperlink ref="L173" r:id="rId457" xr:uid="{D8C293EA-4A6C-48F8-ABDE-CDC6A563E41B}"/>
+    <hyperlink ref="M173" r:id="rId458" xr:uid="{F4160B13-61F5-4F16-B6B9-5D569F75ADA5}"/>
+    <hyperlink ref="B174" r:id="rId459" xr:uid="{3FCC55C1-9DED-4100-984E-2B6060EECF63}"/>
+    <hyperlink ref="L174" r:id="rId460" xr:uid="{3F450402-B744-460B-86A5-DA1473300017}"/>
+    <hyperlink ref="B175" r:id="rId461" xr:uid="{64443F1B-8990-4E18-B336-0D97FECC188A}"/>
+    <hyperlink ref="L175" r:id="rId462" xr:uid="{B027F4C1-F544-4EE7-B6D1-AB5192AEFE1F}"/>
+    <hyperlink ref="B176" r:id="rId463" xr:uid="{499CBDD5-97FA-49AC-B731-BB94526A26BB}"/>
+    <hyperlink ref="L176" r:id="rId464" xr:uid="{3790D0E4-1101-497C-A8B7-5B8014913C30}"/>
+    <hyperlink ref="B177" r:id="rId465" xr:uid="{B980398D-E38B-4479-A20C-54A5EEFB3441}"/>
+    <hyperlink ref="E177" r:id="rId466" xr:uid="{346CE815-0709-47C3-B0BA-8B7DA0597755}"/>
+    <hyperlink ref="L177" r:id="rId467" xr:uid="{76DF5085-4ACD-4E99-9D4A-1561C15C957C}"/>
+    <hyperlink ref="M177" r:id="rId468" xr:uid="{049B83A2-7639-493D-842C-4385B1DA1A83}"/>
+    <hyperlink ref="B178" r:id="rId469" xr:uid="{949C0E89-EDE5-4C81-BD79-902328EC7D81}"/>
+    <hyperlink ref="E178" r:id="rId470" xr:uid="{D3FA2CED-91B4-4446-BBF5-3668C199A0C2}"/>
+    <hyperlink ref="L178" r:id="rId471" xr:uid="{D39857F6-0B2D-4514-BCB3-9C1F5A9FD6DB}"/>
+    <hyperlink ref="M178" r:id="rId472" xr:uid="{581BDCAF-DC78-44E6-A3D4-B6CFCB687136}"/>
+    <hyperlink ref="B179" r:id="rId473" xr:uid="{45728CAD-6F1A-4A6F-9AFF-AF93F8525FC6}"/>
+    <hyperlink ref="L179" r:id="rId474" xr:uid="{1F95FC3E-7AA5-4C6E-B276-E484D151E6F8}"/>
+    <hyperlink ref="B180" r:id="rId475" xr:uid="{820CF8B4-5F43-40AB-928D-494769E5B83A}"/>
+    <hyperlink ref="E180" r:id="rId476" xr:uid="{8526A066-D11F-49EB-9AA1-915ED9B22E23}"/>
+    <hyperlink ref="L180" r:id="rId477" xr:uid="{261237D0-9D37-4EB9-AE96-AB73609C8C07}"/>
+    <hyperlink ref="M180" r:id="rId478" xr:uid="{087D5613-D9AC-46DF-9AD3-C49CAFC55B41}"/>
+    <hyperlink ref="B181" r:id="rId479" xr:uid="{CCE695E0-4F97-459F-9A70-C0A42B924813}"/>
+    <hyperlink ref="L181" r:id="rId480" xr:uid="{F824350A-7994-4282-A06F-1558BEAB3910}"/>
+    <hyperlink ref="B182" r:id="rId481" xr:uid="{4656A668-A30C-4A99-9204-D166A9429090}"/>
+    <hyperlink ref="E182" r:id="rId482" xr:uid="{F4390EB1-27AE-4370-9C2E-BB75C8D74CF7}"/>
+    <hyperlink ref="L182" r:id="rId483" xr:uid="{6C70B1F1-22D3-446A-9CAA-9115FDE553B5}"/>
+    <hyperlink ref="M182" r:id="rId484" xr:uid="{66590329-689D-496B-82C1-75F9765423C6}"/>
+    <hyperlink ref="B183" r:id="rId485" xr:uid="{5E9CC006-0480-41B7-9B1E-F34AF75F1F62}"/>
+    <hyperlink ref="L183" r:id="rId486" xr:uid="{C939E009-E125-487B-99C9-96CC54A33314}"/>
+    <hyperlink ref="B184" r:id="rId487" xr:uid="{8E47C2A4-C4DB-4FAB-92B3-341843C063A8}"/>
+    <hyperlink ref="L184" r:id="rId488" xr:uid="{3F718029-501D-40AF-9024-6FAA8B8DDABB}"/>
+    <hyperlink ref="B185" r:id="rId489" xr:uid="{A2DEA92F-68FC-41AF-ABA1-E550025C9F9B}"/>
+    <hyperlink ref="H185" r:id="rId490" xr:uid="{A4111DC1-3CB8-4D22-98D9-431878F32BD9}"/>
+    <hyperlink ref="L185" r:id="rId491" xr:uid="{CAA3F67C-EA93-460E-A93E-2DA27623BFE5}"/>
+    <hyperlink ref="M185" r:id="rId492" xr:uid="{6D9CF0B8-197F-4117-9B73-CD865794C2D2}"/>
+    <hyperlink ref="B186" r:id="rId493" xr:uid="{0CA86837-72FE-451A-9BC8-C3F21C241A4B}"/>
+    <hyperlink ref="H186" r:id="rId494" xr:uid="{38025CD6-D255-42C0-8ADF-7427D6B815E8}"/>
+    <hyperlink ref="L186" r:id="rId495" xr:uid="{47D42D45-B7DC-4BC9-9A7A-1AEB4D28C50D}"/>
+    <hyperlink ref="M186" r:id="rId496" xr:uid="{FC03D824-5A80-45ED-A704-A6C517F2931A}"/>
+    <hyperlink ref="B187" r:id="rId497" xr:uid="{5A75C93F-882E-4BC2-8D44-9880A7D1ACDD}"/>
+    <hyperlink ref="L187" r:id="rId498" xr:uid="{1CCBADB6-6C1D-4E2A-9087-06E722294DE5}"/>
+    <hyperlink ref="B188" r:id="rId499" xr:uid="{D678D924-9ED1-42BB-9F7B-57811DEEB0B1}"/>
+    <hyperlink ref="E188" r:id="rId500" xr:uid="{A5883D8C-9714-4C24-9100-6CEDE69ED20D}"/>
+    <hyperlink ref="L188" r:id="rId501" xr:uid="{C7C7438D-AE0F-40C6-9A83-1A882E65FACC}"/>
+    <hyperlink ref="M188" r:id="rId502" xr:uid="{0DE21998-C14D-4ED7-BE7B-3D8CF8FE0244}"/>
+    <hyperlink ref="B189" r:id="rId503" xr:uid="{EB8E6E8B-0E12-42CB-AD77-B43289DC8D60}"/>
+    <hyperlink ref="L189" r:id="rId504" xr:uid="{937F86A6-86C9-4560-994C-4E96DC48FA38}"/>
+    <hyperlink ref="B190" r:id="rId505" xr:uid="{F688077A-191F-4C89-BFF2-73D33AF5A040}"/>
+    <hyperlink ref="E190" r:id="rId506" xr:uid="{1CF7DF42-7A24-4231-A870-48247AC44A34}"/>
+    <hyperlink ref="L190" r:id="rId507" xr:uid="{D306DD36-B07A-4565-8870-E7AD219EB5F5}"/>
+    <hyperlink ref="M190" r:id="rId508" xr:uid="{767228F9-062C-46A8-B44D-048A79930469}"/>
+    <hyperlink ref="B191" r:id="rId509" xr:uid="{C319DA59-F4AB-4912-928F-E3794AE735F6}"/>
+    <hyperlink ref="L191" r:id="rId510" xr:uid="{225DDB20-A187-40AB-9919-D47DC944CBDB}"/>
+    <hyperlink ref="B192" r:id="rId511" xr:uid="{5628EA51-BD64-421F-9896-27AF04FFF24F}"/>
+    <hyperlink ref="E192" r:id="rId512" xr:uid="{47EA5C8E-D3B5-4286-B392-C510C5CCE69C}"/>
+    <hyperlink ref="H192" r:id="rId513" xr:uid="{F52A56D3-0B8C-4A15-B8B1-F4794F4ED0B4}"/>
+    <hyperlink ref="L192" r:id="rId514" xr:uid="{6A367B76-429B-40E0-8A04-583C29E1C6C9}"/>
+    <hyperlink ref="M192" r:id="rId515" xr:uid="{3548D8E0-3AFF-49D8-803F-7D4FCC32F6E4}"/>
+    <hyperlink ref="B193" r:id="rId516" xr:uid="{F5605E38-7A88-412E-B090-78A7EBD04B58}"/>
+    <hyperlink ref="L193" r:id="rId517" xr:uid="{3CF23391-4B34-479F-B4F8-93F56C2786CD}"/>
+    <hyperlink ref="B194" r:id="rId518" xr:uid="{4C48DDAE-0509-48A4-BCFC-43019488C983}"/>
+    <hyperlink ref="L194" r:id="rId519" xr:uid="{AC83EB3E-8836-46F4-9C84-EB5C3FA5F810}"/>
+    <hyperlink ref="M194" r:id="rId520" xr:uid="{DB5BBDDB-3ADE-4B8E-820D-FDA88D13C85B}"/>
+    <hyperlink ref="B195" r:id="rId521" xr:uid="{886AAF11-9AE7-4D54-AD8E-9B2F668C6FCC}"/>
+    <hyperlink ref="L195" r:id="rId522" xr:uid="{A78C3983-E98F-43DE-95DA-6F744D119519}"/>
+    <hyperlink ref="B196" r:id="rId523" xr:uid="{CA7BBF0D-61E5-41E8-AD66-A43C77BA6891}"/>
+    <hyperlink ref="E196" r:id="rId524" xr:uid="{F35574D4-5502-4504-A0D5-753D01992C48}"/>
+    <hyperlink ref="L196" r:id="rId525" xr:uid="{82398A9D-CDAD-49EF-88F3-E3A6F03ADBC4}"/>
+    <hyperlink ref="M196" r:id="rId526" xr:uid="{A6911EA6-18FA-4275-83E6-30BA0A633383}"/>
+    <hyperlink ref="B197" r:id="rId527" xr:uid="{F8DEAE0D-E015-4ECA-85E3-4A76036C3231}"/>
+    <hyperlink ref="E197" r:id="rId528" xr:uid="{0DB63BA6-8306-4026-8A11-AAD0A5C4A01B}"/>
+    <hyperlink ref="L197" r:id="rId529" xr:uid="{E2FB5DD6-FF65-4ACB-B63A-90CD63DF6D9D}"/>
+    <hyperlink ref="M197" r:id="rId530" xr:uid="{BC2CDD2E-7E20-4EB7-8E5F-32ECC7EB1705}"/>
+    <hyperlink ref="B198" r:id="rId531" xr:uid="{7352E0D6-A299-41D2-8180-A869A19DF5D8}"/>
+    <hyperlink ref="L198" r:id="rId532" xr:uid="{46FBB4E4-9383-4E0C-95C2-42AD3BCD3FDA}"/>
+    <hyperlink ref="B199" r:id="rId533" xr:uid="{0CE5B0FE-2941-4E61-BB60-777E1FFF1BF3}"/>
+    <hyperlink ref="L199" r:id="rId534" xr:uid="{6FE3B76F-2A1F-45FC-906D-1D2D5C493B5A}"/>
+    <hyperlink ref="B200" r:id="rId535" xr:uid="{1DB3E804-450F-493D-AF70-C5D68576CE6D}"/>
+    <hyperlink ref="L200" r:id="rId536" xr:uid="{EB8A13D7-8819-4F65-889A-98EC58E0F86C}"/>
+    <hyperlink ref="B201" r:id="rId537" xr:uid="{4BC06911-5E99-47DC-967B-C3FDD81ABD06}"/>
+    <hyperlink ref="L201" r:id="rId538" xr:uid="{E5FDD14D-76E9-41D2-BF87-A9EF71BC9471}"/>
+    <hyperlink ref="M201" r:id="rId539" xr:uid="{C56BC396-6EA5-4A9C-AAF5-9A1083B692C7}"/>
+    <hyperlink ref="B202" r:id="rId540" xr:uid="{F8F04232-6FD8-4D3F-A5F4-545F7FC6470B}"/>
+    <hyperlink ref="L202" r:id="rId541" xr:uid="{4F215694-3414-4DDF-BCDC-B6D784E956E6}"/>
+    <hyperlink ref="B203" r:id="rId542" xr:uid="{FA7FD6BA-6F5A-462C-ADDE-6A149FB0BB43}"/>
+    <hyperlink ref="E203" r:id="rId543" xr:uid="{39D98D44-AEE2-45DF-97BC-41284830AB1F}"/>
+    <hyperlink ref="L203" r:id="rId544" xr:uid="{7A5F1952-EF93-4D27-A282-28FB4F4E3B49}"/>
+    <hyperlink ref="M203" r:id="rId545" xr:uid="{2AD0A3CD-60EC-4B88-811A-6935F1157B1B}"/>
+    <hyperlink ref="B204" r:id="rId546" xr:uid="{DB018303-AB73-446E-A105-CD91CCFD16AF}"/>
+    <hyperlink ref="L204" r:id="rId547" xr:uid="{5DBC8B10-F35E-4288-9BDD-211B25659F6C}"/>
+    <hyperlink ref="B205" r:id="rId548" xr:uid="{D273D77E-2049-4635-B470-50F20ED0D1B7}"/>
+    <hyperlink ref="L205" r:id="rId549" xr:uid="{D12AC4B4-53EC-4EEF-BCEC-3AD395395B4E}"/>
+    <hyperlink ref="B206" r:id="rId550" xr:uid="{619ED0C2-363F-4EB3-A172-011C37845BE9}"/>
+    <hyperlink ref="L206" r:id="rId551" xr:uid="{25C59271-8602-4A77-B3FD-65658B41DB05}"/>
+    <hyperlink ref="B207" r:id="rId552" xr:uid="{FAD0007A-5163-4DCB-9902-7B6AD7022F24}"/>
+    <hyperlink ref="L207" r:id="rId553" xr:uid="{051F8532-4534-42C1-8B09-FF25C0F82476}"/>
+    <hyperlink ref="B208" r:id="rId554" xr:uid="{4D83980F-0942-44E4-BA2C-58F5879B16D2}"/>
+    <hyperlink ref="L208" r:id="rId555" xr:uid="{21CA3503-1F5F-4066-BDB2-759BF0E73691}"/>
+    <hyperlink ref="M208" r:id="rId556" xr:uid="{3F9FA0CC-3D3E-48A6-8DDC-6AE21B0931CF}"/>
+    <hyperlink ref="B209" r:id="rId557" xr:uid="{4BE4ED40-F10A-48D2-B77F-B9131F83F875}"/>
+    <hyperlink ref="E209" r:id="rId558" xr:uid="{FE4817AE-6855-41AF-97DF-56CB38A4952C}"/>
+    <hyperlink ref="L209" r:id="rId559" xr:uid="{5728A906-54B5-4FE9-88C9-B5F6C5B45DA1}"/>
+    <hyperlink ref="M209" r:id="rId560" xr:uid="{7366833C-2276-47A0-85DF-00D3ABE4D8E3}"/>
+    <hyperlink ref="B210" r:id="rId561" xr:uid="{05AA6DB9-B8EF-42A2-8673-21B086AF27FB}"/>
+    <hyperlink ref="L210" r:id="rId562" xr:uid="{723EC9DD-136A-48FC-81EF-8C8789F049E3}"/>
+    <hyperlink ref="M210" r:id="rId563" xr:uid="{EED0A03E-8234-4065-87DC-16A45CC9E534}"/>
+    <hyperlink ref="B211" r:id="rId564" xr:uid="{37792762-15A3-4DF4-93BE-2F60C76E42ED}"/>
+    <hyperlink ref="L211" r:id="rId565" xr:uid="{B062C568-2F07-42BF-A809-94551A9A56E2}"/>
+    <hyperlink ref="M211" r:id="rId566" xr:uid="{3AFD1EF1-3357-428F-870C-103845838347}"/>
+    <hyperlink ref="B212" r:id="rId567" xr:uid="{A4C548AE-E531-4647-8843-EC03C023E2A9}"/>
+    <hyperlink ref="L212" r:id="rId568" xr:uid="{14323B4A-6DB6-497F-A187-D1E8DFAF17F1}"/>
+    <hyperlink ref="B213" r:id="rId569" xr:uid="{D0AA2B0B-2DEF-4D8B-9131-852CB02C0094}"/>
+    <hyperlink ref="L213" r:id="rId570" xr:uid="{93A21493-172B-4281-B99F-5EF2D2E22605}"/>
+    <hyperlink ref="B214" r:id="rId571" xr:uid="{EB0DA12A-0F7D-4C40-9FDA-68B4B78DC60E}"/>
+    <hyperlink ref="H214" r:id="rId572" xr:uid="{C44B6755-27EE-4324-A268-561E389517B7}"/>
+    <hyperlink ref="L214" r:id="rId573" xr:uid="{61E8E769-3334-49B4-9D67-C62462C92539}"/>
+    <hyperlink ref="M214" r:id="rId574" xr:uid="{40FF8705-5781-40AA-9229-3E9E2B8C66C4}"/>
+    <hyperlink ref="B215" r:id="rId575" xr:uid="{33D95E51-E0F7-41CA-A0E7-B25E87C406E5}"/>
+    <hyperlink ref="L215" r:id="rId576" xr:uid="{1B3BA363-E99F-442B-BAA4-6CFB18EDE192}"/>
+    <hyperlink ref="B216" r:id="rId577" xr:uid="{9A213E79-43C5-4F31-B6FA-6E95082EA9FC}"/>
+    <hyperlink ref="L216" r:id="rId578" xr:uid="{EB77F959-6C26-49DA-9353-518EEB6FA316}"/>
+    <hyperlink ref="B217" r:id="rId579" xr:uid="{7BDF9153-500B-4117-B0A2-DE8088C6C030}"/>
+    <hyperlink ref="L217" r:id="rId580" xr:uid="{A76BCA8C-8913-4326-B07B-F5675D755F4A}"/>
+    <hyperlink ref="M217" r:id="rId581" xr:uid="{00E8AF58-8C6E-4B54-8838-AD1DA01E6BDC}"/>
+    <hyperlink ref="B218" r:id="rId582" xr:uid="{3D6CE5CF-5A90-4A13-AE0F-AFB990A07A80}"/>
+    <hyperlink ref="L218" r:id="rId583" xr:uid="{2212F3EB-CBD3-4784-8425-790D358CAD6A}"/>
+    <hyperlink ref="M218" r:id="rId584" xr:uid="{812CFC49-0A50-42B8-8662-0BFE60594B27}"/>
+    <hyperlink ref="B219" r:id="rId585" xr:uid="{5092AEE5-6A80-4B10-A47D-C7540530A538}"/>
+    <hyperlink ref="L219" r:id="rId586" xr:uid="{C466206F-342C-4DD2-96DD-65654E692D76}"/>
+    <hyperlink ref="M219" r:id="rId587" xr:uid="{BA9E8222-AC52-40B1-A8FC-0BAE8A756949}"/>
+    <hyperlink ref="B220" r:id="rId588" xr:uid="{9D1F6AB0-3CE3-4639-A794-EBD7EFDC8474}"/>
+    <hyperlink ref="L220" r:id="rId589" xr:uid="{AE2CB813-8DE1-4CA7-A7F9-6DB13CC1D34C}"/>
+    <hyperlink ref="M220" r:id="rId590" xr:uid="{135292BD-CFE0-473A-83A0-34480765BCAB}"/>
+    <hyperlink ref="B221" r:id="rId591" xr:uid="{EAD3CF00-71F5-4EC5-8622-D4FE139D8B34}"/>
+    <hyperlink ref="L221" r:id="rId592" xr:uid="{3218021D-1E46-4C8E-B67E-95A43A7FBA8E}"/>
+    <hyperlink ref="B222" r:id="rId593" xr:uid="{ED7F3E52-4D89-457A-9F1F-197B0168A426}"/>
+    <hyperlink ref="L222" r:id="rId594" xr:uid="{3E439D8D-A68B-4588-A0B4-3AED19A2FD23}"/>
+    <hyperlink ref="B223" r:id="rId595" xr:uid="{5BA796E9-8FEB-4A0D-B38D-05D26CBEBEAD}"/>
+    <hyperlink ref="E223" r:id="rId596" xr:uid="{71942CF2-7FC0-452A-8D63-83D5B86DFD27}"/>
+    <hyperlink ref="L223" r:id="rId597" xr:uid="{CB938387-A7D8-4520-BB2E-F52D431682D2}"/>
+    <hyperlink ref="M223" r:id="rId598" xr:uid="{E77A84E5-2D6D-4AA5-B809-0F80C8CDC1B9}"/>
+    <hyperlink ref="B224" r:id="rId599" xr:uid="{AD1620EF-C417-4803-B10A-C1F83640FE87}"/>
+    <hyperlink ref="L224" r:id="rId600" xr:uid="{DEFC3366-6520-44E1-A671-76C182CE9DCF}"/>
+    <hyperlink ref="B225" r:id="rId601" xr:uid="{7115D6CE-D5F4-4E6A-8337-BAACD38C8579}"/>
+    <hyperlink ref="L225" r:id="rId602" xr:uid="{ED1CBD1D-9B1C-4900-B4BE-10BB6F1B9779}"/>
+    <hyperlink ref="B226" r:id="rId603" xr:uid="{1CABF8B7-6375-48AF-8EF1-6EDAE9760238}"/>
+    <hyperlink ref="L226" r:id="rId604" xr:uid="{FB0B38AD-A58C-404A-A11D-B87065349E0B}"/>
+    <hyperlink ref="B227" r:id="rId605" xr:uid="{7ABEE3E3-C5A5-4D46-8D51-E0909203BA54}"/>
+    <hyperlink ref="L227" r:id="rId606" xr:uid="{D27EB115-39A6-4AFC-B13C-4BDAA79D8BBF}"/>
+    <hyperlink ref="B228" r:id="rId607" xr:uid="{73168768-A7AD-4996-AAAD-2F6D9E3522C8}"/>
+    <hyperlink ref="L228" r:id="rId608" xr:uid="{B53240ED-A313-4600-AD5C-CFB38AE627CD}"/>
+    <hyperlink ref="B229" r:id="rId609" xr:uid="{97EAAB2B-E7F2-44D9-8881-B912E1B959B3}"/>
+    <hyperlink ref="L229" r:id="rId610" xr:uid="{A776897B-83CE-46A9-8A04-0E17C0348A56}"/>
+    <hyperlink ref="B230" r:id="rId611" xr:uid="{FBB91FC3-A3BF-4606-A149-B24F0A409F73}"/>
+    <hyperlink ref="L230" r:id="rId612" xr:uid="{B09BF52F-3053-4941-98C4-20FEEB46CA9C}"/>
+    <hyperlink ref="B231" r:id="rId613" xr:uid="{6031E21A-A2EE-4E01-BBBB-83453361800F}"/>
+    <hyperlink ref="L231" r:id="rId614" xr:uid="{FE0DE943-B2DA-4103-8567-429986C961AE}"/>
+    <hyperlink ref="B232" r:id="rId615" xr:uid="{E5DF4647-9626-483E-BEEF-9223E5E2BA66}"/>
+    <hyperlink ref="L232" r:id="rId616" xr:uid="{28400EBA-3DE7-4679-9165-636D832C54F6}"/>
+    <hyperlink ref="B233" r:id="rId617" xr:uid="{E10CE151-93A9-4F8B-89A2-9115EBE440D2}"/>
+    <hyperlink ref="L233" r:id="rId618" xr:uid="{341AA69C-778A-4DAF-A0D2-EC72F625CC18}"/>
+    <hyperlink ref="B234" r:id="rId619" xr:uid="{82CB8061-D39D-47BB-BA19-490E124B1F0C}"/>
+    <hyperlink ref="E234" r:id="rId620" xr:uid="{7998C4E6-6565-491F-BE12-15011928AE8E}"/>
+    <hyperlink ref="L234" r:id="rId621" xr:uid="{25C813D6-DDCE-462C-881E-1D850A32BAE3}"/>
+    <hyperlink ref="M234" r:id="rId622" xr:uid="{70C2766D-53B9-4C19-927A-F2729EA7F650}"/>
+    <hyperlink ref="B235" r:id="rId623" xr:uid="{4F609874-D3CE-4023-97F2-9C048DE107A3}"/>
+    <hyperlink ref="H235" r:id="rId624" xr:uid="{5106BAB7-839F-4200-863A-DE4ACB8F95C0}"/>
+    <hyperlink ref="L235" r:id="rId625" xr:uid="{14B34FA7-E078-4EB3-A036-B626470EAFDC}"/>
+    <hyperlink ref="M235" r:id="rId626" xr:uid="{8AD3589B-C780-47F5-80A6-19E2C1FDF678}"/>
+    <hyperlink ref="B236" r:id="rId627" xr:uid="{170BE2C2-F3FF-4DAA-BCE9-C4A7B7AD4CFE}"/>
+    <hyperlink ref="L236" r:id="rId628" xr:uid="{EAE4F122-CB40-426A-9311-FAB201AF88A4}"/>
+    <hyperlink ref="B237" r:id="rId629" xr:uid="{AFF12051-11C5-4B94-B57A-786D1C2CD108}"/>
+    <hyperlink ref="L237" r:id="rId630" xr:uid="{E2F538FA-7BF2-4C56-860E-F0DA7619CF35}"/>
+    <hyperlink ref="B238" r:id="rId631" xr:uid="{CA9FDDAB-D7C8-4557-AE10-E1DEB470E1A6}"/>
+    <hyperlink ref="L238" r:id="rId632" xr:uid="{EED6BEFD-845A-4728-85C7-1B9BD5062961}"/>
+    <hyperlink ref="M238" r:id="rId633" xr:uid="{E18C06F8-86FB-4697-A07F-36D16194B029}"/>
+    <hyperlink ref="B239" r:id="rId634" xr:uid="{F0B672B4-73FA-40ED-BC8C-A99A0091B97C}"/>
+    <hyperlink ref="L239" r:id="rId635" xr:uid="{134948DE-86DD-41FC-8645-C0596D29BF56}"/>
+    <hyperlink ref="B240" r:id="rId636" xr:uid="{33B9724B-6562-4BB6-AE8F-63DB44583E65}"/>
+    <hyperlink ref="L240" r:id="rId637" xr:uid="{C66C79DE-66DE-43C1-B316-EE1A1B23A26B}"/>
+    <hyperlink ref="B241" r:id="rId638" xr:uid="{FB5C0E60-CC19-44C3-96D4-76452025A289}"/>
+    <hyperlink ref="L241" r:id="rId639" xr:uid="{22FD4C52-9865-43AE-88DD-F1D3A21899B0}"/>
+    <hyperlink ref="B242" r:id="rId640" xr:uid="{A63F78F9-A705-48EA-8544-72B926C99F95}"/>
+    <hyperlink ref="L242" r:id="rId641" xr:uid="{54AF416A-C9AC-4299-BCE6-7968B69989DC}"/>
+    <hyperlink ref="B243" r:id="rId642" xr:uid="{AF7DB771-983F-4A5F-AC35-D556B6B8A730}"/>
+    <hyperlink ref="L243" r:id="rId643" xr:uid="{6128AE6A-4299-4438-A805-31C5B9896AF7}"/>
+    <hyperlink ref="B244" r:id="rId644" xr:uid="{32656CBC-CFAC-4855-B26B-65AB3E8B860E}"/>
+    <hyperlink ref="L244" r:id="rId645" xr:uid="{5AA15A16-139C-4D6F-B3F9-1E2AB67ADFF2}"/>
+    <hyperlink ref="B245" r:id="rId646" xr:uid="{6EE9B912-DDF7-42AC-943C-694EAEBF6291}"/>
+    <hyperlink ref="L245" r:id="rId647" xr:uid="{8AA31FF6-0B3B-4D21-8F24-7D921B9BD37C}"/>
+    <hyperlink ref="B246" r:id="rId648" xr:uid="{745B3B92-16B2-4674-8DB9-0F4A6D8EBA4F}"/>
+    <hyperlink ref="L246" r:id="rId649" xr:uid="{BE26BF5E-605D-4513-B824-4107ECACB445}"/>
+    <hyperlink ref="B247" r:id="rId650" xr:uid="{1BA4E768-417A-47DB-B4F2-CEF35762891C}"/>
+    <hyperlink ref="L247" r:id="rId651" xr:uid="{AD9527E4-0C5B-4CB7-9F8C-3A02F3B24238}"/>
+    <hyperlink ref="B248" r:id="rId652" xr:uid="{D105B9B9-1751-4AA0-AAF3-2E7BD73AC825}"/>
+    <hyperlink ref="L248" r:id="rId653" xr:uid="{DC5164DA-03F3-4887-A402-797C68B9ACE7}"/>
+    <hyperlink ref="B249" r:id="rId654" xr:uid="{9F58C6DD-3C81-4E5D-AA54-FF76783250F4}"/>
+    <hyperlink ref="L249" r:id="rId655" xr:uid="{CABF4327-9D60-4ABA-95D5-8A002C2EA3F8}"/>
+    <hyperlink ref="B250" r:id="rId656" xr:uid="{F91B9417-395D-4C7D-B8F8-2C228A6660AA}"/>
+    <hyperlink ref="L250" r:id="rId657" xr:uid="{EE2B1A72-AB00-4954-A203-6E818EDE314B}"/>
+    <hyperlink ref="B251" r:id="rId658" xr:uid="{F8E2DE40-3A4E-4FE1-AD8C-0F2B053FB3EE}"/>
+    <hyperlink ref="L251" r:id="rId659" xr:uid="{323AAD6D-8B69-4EF5-87B0-839BF5B5C4DA}"/>
+    <hyperlink ref="B252" r:id="rId660" xr:uid="{DD3F0FFA-187B-48D2-AC64-5D57FB97B2FD}"/>
+    <hyperlink ref="L252" r:id="rId661" xr:uid="{E474565E-C026-499C-8353-A157B2027D89}"/>
+    <hyperlink ref="B253" r:id="rId662" xr:uid="{32D01E81-F9B8-4D25-912A-91E69C953A9C}"/>
+    <hyperlink ref="E253" r:id="rId663" xr:uid="{F60ECD56-CA00-492D-8365-F1E8EA28A620}"/>
+    <hyperlink ref="L253" r:id="rId664" xr:uid="{7AF7C0CB-E09A-4E7E-ABE1-171EF839508D}"/>
+    <hyperlink ref="M253" r:id="rId665" xr:uid="{A0B688F2-45CF-4AA7-838A-5502AC6259B4}"/>
+    <hyperlink ref="B254" r:id="rId666" xr:uid="{003B51FA-D75D-42C9-A4B2-C3B70E65FFBC}"/>
+    <hyperlink ref="E254" r:id="rId667" xr:uid="{2B5BBA69-DDF2-41F1-8189-41EB1BC9AF5A}"/>
+    <hyperlink ref="L254" r:id="rId668" xr:uid="{FD8FE63D-6BD8-4ECB-A1CD-200EA0669BC1}"/>
+    <hyperlink ref="M254" r:id="rId669" xr:uid="{D61083EB-2F89-4C3E-81BD-BE00926702BB}"/>
+    <hyperlink ref="B255" r:id="rId670" xr:uid="{D42C0930-6BD9-494C-9D33-21F04692A857}"/>
+    <hyperlink ref="E255" r:id="rId671" xr:uid="{19A5BD4D-1222-45C3-97C2-72DAFEE0ABA8}"/>
+    <hyperlink ref="L255" r:id="rId672" xr:uid="{C7F05FF5-4339-4D51-9F74-97EE06DCE1A6}"/>
+    <hyperlink ref="M255" r:id="rId673" xr:uid="{1A30A4FC-C3F5-47AF-8E32-6802211EABB6}"/>
+    <hyperlink ref="B256" r:id="rId674" xr:uid="{7F8C2E23-1876-4E80-84D2-C75542A223C5}"/>
+    <hyperlink ref="L256" r:id="rId675" xr:uid="{BC0BDCA5-88B5-474E-A849-070DD424E9C9}"/>
+    <hyperlink ref="M256" r:id="rId676" xr:uid="{79725720-E55E-4BFE-BD79-FD3AD9B30789}"/>
+    <hyperlink ref="B257" r:id="rId677" xr:uid="{0C4B533E-8DB7-4E5F-8C0B-5F2D019718D9}"/>
+    <hyperlink ref="L257" r:id="rId678" xr:uid="{8357927D-04F0-4347-ABA8-4EF27F206146}"/>
+    <hyperlink ref="B258" r:id="rId679" xr:uid="{AF0B7348-1792-4174-B0B8-DB1DF7B9B81D}"/>
+    <hyperlink ref="L258" r:id="rId680" xr:uid="{9F74BBAC-8703-40B9-912E-4ACDBE88E488}"/>
+    <hyperlink ref="B259" r:id="rId681" xr:uid="{34F20CA5-1710-4999-BE97-6632148705EF}"/>
+    <hyperlink ref="L259" r:id="rId682" xr:uid="{11884C78-3EBD-4C89-829D-7EA99A9BB1DB}"/>
+    <hyperlink ref="B260" r:id="rId683" xr:uid="{407D2D5B-C6DB-4C13-B471-DC39DB286436}"/>
+    <hyperlink ref="L260" r:id="rId684" xr:uid="{3719041E-13EA-4B45-9A95-33FEE99A605A}"/>
+    <hyperlink ref="B261" r:id="rId685" xr:uid="{E812585D-6C80-4111-B96A-03DE49CE84D4}"/>
+    <hyperlink ref="L261" r:id="rId686" xr:uid="{9ABBABC0-38BD-4C15-AD8A-6976B04CB02A}"/>
+    <hyperlink ref="B262" r:id="rId687" xr:uid="{03E4AD78-7425-4AA0-AD28-6B3822F7D97C}"/>
+    <hyperlink ref="L262" r:id="rId688" xr:uid="{07221E75-1E3B-4AAB-B0A9-A0B4C8157744}"/>
+    <hyperlink ref="B263" r:id="rId689" xr:uid="{3D25AF38-DB15-4D31-8168-2885D8C066E1}"/>
+    <hyperlink ref="L263" r:id="rId690" xr:uid="{05836E64-FACC-488A-AB9E-78E1820D0C36}"/>
+    <hyperlink ref="B264" r:id="rId691" xr:uid="{6AE95820-611D-44C9-8584-FD59F75C91E8}"/>
+    <hyperlink ref="L264" r:id="rId692" xr:uid="{9E5281DA-73EA-4F69-89F5-B5A6ACAC7D69}"/>
+    <hyperlink ref="B265" r:id="rId693" xr:uid="{4A130044-D23D-4B01-A8B5-582B09FA345E}"/>
+    <hyperlink ref="L265" r:id="rId694" xr:uid="{A6C738E8-08AA-4808-9364-3E9A7206A4CC}"/>
+    <hyperlink ref="B266" r:id="rId695" xr:uid="{B47860B4-99E6-4C84-AD35-11D48844CA05}"/>
+    <hyperlink ref="L266" r:id="rId696" xr:uid="{968467CC-C998-4806-8D30-A43587E55503}"/>
+    <hyperlink ref="B267" r:id="rId697" xr:uid="{E2D9FD60-D750-4745-AAB3-7FA9E04838D3}"/>
+    <hyperlink ref="L267" r:id="rId698" xr:uid="{0625A0BE-6D64-42A0-8F18-5488ED595D7C}"/>
+    <hyperlink ref="B268" r:id="rId699" xr:uid="{16CE9B76-30C1-4222-A882-D52368EBFC50}"/>
+    <hyperlink ref="L268" r:id="rId700" xr:uid="{7BAB7020-ADF0-4580-9D4F-3CF0C558F481}"/>
+    <hyperlink ref="B269" r:id="rId701" xr:uid="{179209A5-C741-4AC6-85A2-8530D2947CBE}"/>
+    <hyperlink ref="L269" r:id="rId702" xr:uid="{858622C0-6DAE-44A2-9B6D-890599C9239F}"/>
+    <hyperlink ref="B270" r:id="rId703" xr:uid="{E0291DB5-408D-4C13-B85E-9F713732CDCF}"/>
+    <hyperlink ref="L270" r:id="rId704" xr:uid="{10CC2B0E-E58A-47C8-BC77-211CC45434DB}"/>
+    <hyperlink ref="B271" r:id="rId705" xr:uid="{9030D530-898A-49FB-99FC-83A2350436B1}"/>
+    <hyperlink ref="L271" r:id="rId706" xr:uid="{D7CB0EA1-D695-4649-BCC7-A6DC1472B98B}"/>
+    <hyperlink ref="B272" r:id="rId707" xr:uid="{88A2E56A-0C40-4964-A9C5-5CD54A8AA878}"/>
+    <hyperlink ref="E272" r:id="rId708" xr:uid="{6FF828FE-683D-4DFF-B68C-4E0818631062}"/>
+    <hyperlink ref="L272" r:id="rId709" xr:uid="{5C341122-3AF5-4B55-8858-2E91321FC158}"/>
+    <hyperlink ref="M272" r:id="rId710" xr:uid="{9128C637-DD7F-463F-9894-4D82D170E747}"/>
+    <hyperlink ref="B273" r:id="rId711" xr:uid="{C50B0C00-92E7-4865-8090-DE7E8F89B19D}"/>
+    <hyperlink ref="L273" r:id="rId712" xr:uid="{B9F75C08-11AA-4033-960A-BF98953B4EEC}"/>
+    <hyperlink ref="B274" r:id="rId713" xr:uid="{B8438BF9-EEFC-49F6-9C57-0C4C892E4B7C}"/>
+    <hyperlink ref="L274" r:id="rId714" xr:uid="{B7D589CD-0EE6-4F96-BD43-772E63FA5961}"/>
+    <hyperlink ref="M274" r:id="rId715" xr:uid="{64EF4862-F7BB-4DE8-9B3D-FF129FB8329A}"/>
+    <hyperlink ref="B275" r:id="rId716" xr:uid="{4ABB4AFC-4607-4860-9362-53F54E314C9B}"/>
+    <hyperlink ref="L275" r:id="rId717" xr:uid="{DB964837-E176-4171-8E79-B4BD1091C551}"/>
+    <hyperlink ref="B276" r:id="rId718" xr:uid="{282CE3E6-DF5D-40CE-BC2D-A33809504518}"/>
+    <hyperlink ref="H276" r:id="rId719" xr:uid="{4C23463B-D312-40E5-AF9B-1018DA7706CA}"/>
+    <hyperlink ref="L276" r:id="rId720" xr:uid="{54374BA5-BC77-49EF-AD30-2A0B1AF6052D}"/>
+    <hyperlink ref="M276" r:id="rId721" xr:uid="{2119FECD-3429-47BC-8D47-87F1A93700C8}"/>
+    <hyperlink ref="B277" r:id="rId722" xr:uid="{4111B163-2D8E-4147-953F-3E2ED2A8E52E}"/>
+    <hyperlink ref="L277" r:id="rId723" xr:uid="{3F382D0B-1AD1-4B07-8CCC-8CD01C515D0D}"/>
+    <hyperlink ref="M277" r:id="rId724" xr:uid="{B23DD3D1-3805-48D0-A4FE-A4E1405EB0D9}"/>
+    <hyperlink ref="B278" r:id="rId725" xr:uid="{FCD59304-559E-4367-983E-05E42FB57820}"/>
+    <hyperlink ref="L278" r:id="rId726" xr:uid="{FDB638B0-CD99-4D3E-B992-F3C640EA5C2C}"/>
+    <hyperlink ref="M278" r:id="rId727" xr:uid="{2A84E16F-E652-45B4-978C-F9EA639640B0}"/>
+    <hyperlink ref="B279" r:id="rId728" xr:uid="{6AA7ED3A-6288-47D0-9F21-A46607103C8B}"/>
+    <hyperlink ref="L279" r:id="rId729" xr:uid="{D2105D23-8EAF-4089-B863-76C6259514AF}"/>
+    <hyperlink ref="M279" r:id="rId730" xr:uid="{56ECEF4B-E24E-45E2-9228-61A3FCE6BF22}"/>
+    <hyperlink ref="B280" r:id="rId731" xr:uid="{B24BA187-0E1B-4AE5-9AE4-0402AC3ED035}"/>
+    <hyperlink ref="L280" r:id="rId732" xr:uid="{1A60FB3E-A452-464F-A019-F3B823BDC684}"/>
+    <hyperlink ref="B281" r:id="rId733" xr:uid="{E8229F79-C1C3-48F4-B58C-F63A5E7CAF39}"/>
+    <hyperlink ref="L281" r:id="rId734" xr:uid="{FE30426D-7383-4167-84A7-1CBFB885868E}"/>
+    <hyperlink ref="B282" r:id="rId735" xr:uid="{FA71D09F-A6D3-4530-BB31-5490275EBCD8}"/>
+    <hyperlink ref="L282" r:id="rId736" xr:uid="{D5251FFE-3A8E-4EC0-B178-FF0B064B86F1}"/>
+    <hyperlink ref="B283" r:id="rId737" xr:uid="{05C33DB9-DA7A-49D7-B9DC-F6D6068A80F2}"/>
+    <hyperlink ref="L283" r:id="rId738" xr:uid="{3036B47D-175F-43D6-812A-C9F1DBA717C4}"/>
+    <hyperlink ref="B284" r:id="rId739" xr:uid="{77FDCCCB-78FD-4746-82C4-B6870FE02B90}"/>
+    <hyperlink ref="L284" r:id="rId740" xr:uid="{53CC48DF-CF46-4137-BBEB-EDA097626F32}"/>
+    <hyperlink ref="B285" r:id="rId741" xr:uid="{E25D0327-62B9-499D-8F77-07D91CC2BD61}"/>
+    <hyperlink ref="L285" r:id="rId742" xr:uid="{9599B9B0-EF42-4A4C-B502-88C537C7DE91}"/>
+    <hyperlink ref="B286" r:id="rId743" xr:uid="{E5540B2A-2B67-42FB-AB79-6A1A097C87C9}"/>
+    <hyperlink ref="L286" r:id="rId744" xr:uid="{B8A9361F-776E-4F5A-A57A-1F59B2A6FB08}"/>
+    <hyperlink ref="B287" r:id="rId745" xr:uid="{A82C56A8-9082-4765-86C7-EC0DDEDFC35D}"/>
+    <hyperlink ref="L287" r:id="rId746" xr:uid="{BC5324CE-7063-4C4F-8CF0-05106F48F894}"/>
+    <hyperlink ref="B288" r:id="rId747" xr:uid="{A3E92A2B-4BED-490B-831C-D98CF8A5D7CD}"/>
+    <hyperlink ref="L288" r:id="rId748" xr:uid="{2CCFA966-2253-4B2A-9486-002A271D0C3B}"/>
+    <hyperlink ref="B289" r:id="rId749" xr:uid="{334FB46B-4FA2-4748-9EAA-30357F87CF7A}"/>
+    <hyperlink ref="L289" r:id="rId750" xr:uid="{CF1D3A92-99B7-463A-8B10-44D36D19FAE6}"/>
+    <hyperlink ref="B290" r:id="rId751" xr:uid="{B0FADED0-26A3-477C-B6C8-805DEB4F4E2E}"/>
+    <hyperlink ref="L290" r:id="rId752" xr:uid="{D46D9D32-D9C4-4CFD-8028-9E5E70247BE8}"/>
+    <hyperlink ref="B291" r:id="rId753" xr:uid="{B5B0CEAF-6AF8-4F1D-85F1-0C97D18690A5}"/>
+    <hyperlink ref="L291" r:id="rId754" xr:uid="{363E8E96-8830-490A-AB32-37AE7A741C16}"/>
+    <hyperlink ref="B292" r:id="rId755" xr:uid="{2B776EA9-EF0E-4522-BE36-6AC3CB7CFCBA}"/>
+    <hyperlink ref="L292" r:id="rId756" xr:uid="{C2BBACF0-4825-47CD-97AA-733138863477}"/>
+    <hyperlink ref="B293" r:id="rId757" xr:uid="{B29C202F-CF2C-496D-807E-8212F2327963}"/>
+    <hyperlink ref="L293" r:id="rId758" xr:uid="{4D650C14-93D5-4F74-AB2F-786DDDB5EACB}"/>
+    <hyperlink ref="B294" r:id="rId759" xr:uid="{DAC26848-B24A-4689-9B6A-0B1661B1917A}"/>
+    <hyperlink ref="L294" r:id="rId760" xr:uid="{12BEED96-A082-4CA2-8511-86192EBDC7A3}"/>
+    <hyperlink ref="B295" r:id="rId761" xr:uid="{1F0EA9E3-66F5-4649-96D5-E29B981866D8}"/>
+    <hyperlink ref="L295" r:id="rId762" xr:uid="{454D3ED0-805E-48C5-A836-B2B61B50B562}"/>
+    <hyperlink ref="B296" r:id="rId763" xr:uid="{6C66C144-88DC-4B9D-B865-42BA601D8015}"/>
+    <hyperlink ref="L296" r:id="rId764" xr:uid="{26435335-9E07-49B5-A807-6DCFEEEB549D}"/>
+    <hyperlink ref="M296" r:id="rId765" xr:uid="{B45F5C5C-E53A-4C10-939D-2B70EBED347F}"/>
+    <hyperlink ref="B297" r:id="rId766" xr:uid="{E5F56CC1-6BB1-4772-B2EF-C3DBD9445E16}"/>
+    <hyperlink ref="L297" r:id="rId767" xr:uid="{3EA46306-6B4F-4A03-9B18-667724785064}"/>
+    <hyperlink ref="B298" r:id="rId768" xr:uid="{CC76F991-AC3D-4B04-9550-D1825EEADEDC}"/>
+    <hyperlink ref="L298" r:id="rId769" xr:uid="{79A70D13-BFEA-4C41-A94D-451272120627}"/>
+    <hyperlink ref="B299" r:id="rId770" xr:uid="{B36CC80C-6EF9-4BF0-A0C3-ECA28041AE48}"/>
+    <hyperlink ref="L299" r:id="rId771" xr:uid="{5218980C-9587-422E-BEA5-A3C0F0CEE2BD}"/>
+    <hyperlink ref="B300" r:id="rId772" xr:uid="{5922FF9C-9237-4A62-9753-8ED67923516E}"/>
+    <hyperlink ref="L300" r:id="rId773" xr:uid="{C70BC366-0380-4C09-B835-EFA367D752E0}"/>
+    <hyperlink ref="B301" r:id="rId774" xr:uid="{8DEE334D-A4C9-484C-A349-27D81D0FD551}"/>
+    <hyperlink ref="L301" r:id="rId775" xr:uid="{557D54BC-8A2A-458F-A6B5-C8735FA94A6D}"/>
+    <hyperlink ref="B302" r:id="rId776" xr:uid="{6AFEAAD8-40D9-422A-8761-A326E004ECB7}"/>
+    <hyperlink ref="L302" r:id="rId777" xr:uid="{2ECFC1D6-7624-4F5F-8A98-B3DD15D27B31}"/>
+    <hyperlink ref="B303" r:id="rId778" xr:uid="{F6B3F4F5-DB60-44AA-BFD6-C59C603E4ED3}"/>
+    <hyperlink ref="H303" r:id="rId779" xr:uid="{91764401-A6B1-4B60-A87E-C92EC9272DF3}"/>
+    <hyperlink ref="L303" r:id="rId780" xr:uid="{E63005A7-4108-4DE0-BB49-FC3E78E5F342}"/>
+    <hyperlink ref="M303" r:id="rId781" xr:uid="{516CBAF6-2E9D-4936-B09E-E481D6F0E694}"/>
+    <hyperlink ref="B304" r:id="rId782" xr:uid="{B348A943-6B4A-407B-B783-0FE64D9356C6}"/>
+    <hyperlink ref="L304" r:id="rId783" xr:uid="{35367E9E-80F8-45E5-A198-E2C73E1A8F04}"/>
+    <hyperlink ref="B305" r:id="rId784" xr:uid="{6BF7B903-A4E7-4CDC-84FE-62A20A1829B9}"/>
+    <hyperlink ref="L305" r:id="rId785" xr:uid="{C3947D8A-C5AA-48BF-92DF-E6ECFA63A5D0}"/>
+    <hyperlink ref="B306" r:id="rId786" xr:uid="{BE51CA94-5952-4646-B7D3-211F18772165}"/>
+    <hyperlink ref="L306" r:id="rId787" xr:uid="{E5BD6091-8BEA-4EB1-962A-DB29CED8D248}"/>
+    <hyperlink ref="B307" r:id="rId788" xr:uid="{082A599F-EC4D-40D7-8880-E4C3F8B1D5AC}"/>
+    <hyperlink ref="L307" r:id="rId789" xr:uid="{7B5331BE-8175-4B8E-A031-6273A42AA96F}"/>
+    <hyperlink ref="B308" r:id="rId790" xr:uid="{9ED15528-039E-40D5-973D-77522DF0FB4F}"/>
+    <hyperlink ref="L308" r:id="rId791" xr:uid="{0F489C83-87FE-4CD0-8A08-0FC9DDF95386}"/>
+    <hyperlink ref="B309" r:id="rId792" xr:uid="{9EEAA2FC-7572-4028-8BB0-6A4F415CF305}"/>
+    <hyperlink ref="L309" r:id="rId793" xr:uid="{B8FC00A6-FE89-42B4-8DFC-D27AAA810DE8}"/>
+    <hyperlink ref="B310" r:id="rId794" xr:uid="{EB46B8CA-1F7C-48D2-8977-88C057A415DF}"/>
+    <hyperlink ref="L310" r:id="rId795" xr:uid="{A238B155-A5C4-42B6-9EAF-C82DD9B97D5D}"/>
+    <hyperlink ref="B311" r:id="rId796" xr:uid="{E4670C6D-FC11-4BEA-951D-E6012E311732}"/>
+    <hyperlink ref="L311" r:id="rId797" xr:uid="{B883E5B4-EEFE-40F1-A01F-00C4110E7A75}"/>
+    <hyperlink ref="B312" r:id="rId798" xr:uid="{72B490A4-B113-4759-92FB-7A655FD7ED63}"/>
+    <hyperlink ref="L312" r:id="rId799" xr:uid="{882DCCCB-8423-45BC-9FD5-ECBA57085BAA}"/>
+    <hyperlink ref="B313" r:id="rId800" xr:uid="{1420768B-C9A1-452D-BB52-9A0C3A1C1EF5}"/>
+    <hyperlink ref="L313" r:id="rId801" xr:uid="{51198438-DEDF-43B0-9F51-CCA256CD0516}"/>
+    <hyperlink ref="B314" r:id="rId802" xr:uid="{2B016F00-387E-4F86-9AE0-F29F2C8CFE59}"/>
+    <hyperlink ref="L314" r:id="rId803" xr:uid="{408FDDCF-84FE-457B-9E19-71738216927E}"/>
+    <hyperlink ref="B315" r:id="rId804" xr:uid="{0C801164-008C-4ECA-91E7-3B8786CC007D}"/>
+    <hyperlink ref="L315" r:id="rId805" xr:uid="{67E54216-71EF-4FBC-8DE4-6B26C6483D18}"/>
+    <hyperlink ref="B316" r:id="rId806" xr:uid="{310E6A5D-6A7B-4F37-A5FC-C437034E7296}"/>
+    <hyperlink ref="L316" r:id="rId807" xr:uid="{DA377536-3938-4D0F-9F1E-71C0AED0476F}"/>
+    <hyperlink ref="B317" r:id="rId808" xr:uid="{FF447BB9-02DA-4D63-B019-4A8A98456048}"/>
+    <hyperlink ref="L317" r:id="rId809" xr:uid="{7F3CC623-9CDB-4DD1-951C-1C04443EA04F}"/>
+    <hyperlink ref="M317" r:id="rId810" xr:uid="{EECE6F46-F905-4952-AE3E-7F0DD8A5385B}"/>
+    <hyperlink ref="B318" r:id="rId811" xr:uid="{9AE205FE-5CB3-4B03-88C8-ED5D34349F16}"/>
+    <hyperlink ref="L318" r:id="rId812" xr:uid="{177D6DA7-4742-4AAA-A34B-D269161F035A}"/>
+    <hyperlink ref="M318" r:id="rId813" xr:uid="{2CEB8E15-A208-4156-847E-43446DA06DEA}"/>
+    <hyperlink ref="B319" r:id="rId814" xr:uid="{42B6A6FF-44D3-49DF-AECA-D25698F51394}"/>
+    <hyperlink ref="L319" r:id="rId815" xr:uid="{D6AB7053-3B62-4259-89E1-DCFA492F4E6C}"/>
+    <hyperlink ref="B320" r:id="rId816" xr:uid="{67C997A4-0A9F-4C04-B0A8-A32B63552D83}"/>
+    <hyperlink ref="L320" r:id="rId817" xr:uid="{1848C576-A1AA-4AED-98E1-FCBBEB0346AB}"/>
+    <hyperlink ref="B321" r:id="rId818" xr:uid="{4ED79D50-3191-4CEC-9EE0-D2111D736C09}"/>
+    <hyperlink ref="E321" r:id="rId819" xr:uid="{682FFA39-502B-4A7E-AEF3-4EB7F651F06E}"/>
+    <hyperlink ref="L321" r:id="rId820" xr:uid="{7327DB31-93EF-41CC-9A7F-07ABA63424CE}"/>
+    <hyperlink ref="M321" r:id="rId821" xr:uid="{4CA21FD7-B3AD-4863-86E9-32003F85BEDD}"/>
+    <hyperlink ref="B322" r:id="rId822" xr:uid="{635380B4-9565-49B7-8979-ED5506F949C8}"/>
+    <hyperlink ref="L322" r:id="rId823" xr:uid="{552286F3-2420-41D2-91A3-9CB585E6CFC8}"/>
+    <hyperlink ref="B323" r:id="rId824" xr:uid="{490809AF-E87A-4A07-A30B-ABE818F7E730}"/>
+    <hyperlink ref="L323" r:id="rId825" xr:uid="{AF87C7F3-B156-43F8-9D1E-F6A9D05FBB4D}"/>
+    <hyperlink ref="B324" r:id="rId826" xr:uid="{D1977664-575F-4F29-BBBF-C389056272C6}"/>
+    <hyperlink ref="L324" r:id="rId827" xr:uid="{8BB85103-50B5-4046-A13A-52EE65ECF23D}"/>
+    <hyperlink ref="B325" r:id="rId828" xr:uid="{A7531745-FBC2-4C89-B9F9-54C1906D73E9}"/>
+    <hyperlink ref="L325" r:id="rId829" xr:uid="{DDB677A6-E2D2-4B80-95BA-A1B49981390A}"/>
+    <hyperlink ref="B326" r:id="rId830" xr:uid="{F76A02F3-6AE2-420A-B3BE-3316CEF36351}"/>
+    <hyperlink ref="L326" r:id="rId831" xr:uid="{0492D4B7-6205-46F0-B9DE-57131FF855BB}"/>
+    <hyperlink ref="B327" r:id="rId832" xr:uid="{AF40A6AD-56D8-411F-B150-3ABAA477FE06}"/>
+    <hyperlink ref="L327" r:id="rId833" xr:uid="{4FE2257C-9C02-430C-B115-D39DBFF14E6D}"/>
+    <hyperlink ref="B328" r:id="rId834" xr:uid="{F76DE430-13B9-457C-A7E8-A113A722D70F}"/>
+    <hyperlink ref="L328" r:id="rId835" xr:uid="{18217F56-AC5A-4251-BA1E-5D608582D0EB}"/>
+    <hyperlink ref="M328" r:id="rId836" xr:uid="{063F434B-6905-48DA-A447-82FF74CD7AC7}"/>
+    <hyperlink ref="B329" r:id="rId837" xr:uid="{11673439-F250-4AB1-BB77-A229589A6FB9}"/>
+    <hyperlink ref="L329" r:id="rId838" xr:uid="{7C75C72C-1E24-4082-A48C-8683A5A97DFB}"/>
+    <hyperlink ref="B330" r:id="rId839" xr:uid="{38CE4853-6E7D-4424-BA10-73319657F13F}"/>
+    <hyperlink ref="L330" r:id="rId840" xr:uid="{6974F84C-B12C-412F-BEBA-D4CB5D971318}"/>
+    <hyperlink ref="B331" r:id="rId841" xr:uid="{4BF170FE-0D97-49A1-A2E0-0B387389D842}"/>
+    <hyperlink ref="L331" r:id="rId842" xr:uid="{9588A883-B2CF-468A-871F-57554D74140E}"/>
+    <hyperlink ref="B332" r:id="rId843" xr:uid="{264467F3-7250-4CD1-8A14-848F60B737B3}"/>
+    <hyperlink ref="L332" r:id="rId844" xr:uid="{F689051C-FB72-4E4A-B464-890BB6436EDC}"/>
+    <hyperlink ref="B333" r:id="rId845" xr:uid="{E0EB3E1E-9B6B-41C9-85DC-EB1E73FE42DC}"/>
+    <hyperlink ref="L333" r:id="rId846" xr:uid="{C47CE44B-7375-4031-8320-391397F1F771}"/>
+    <hyperlink ref="B334" r:id="rId847" xr:uid="{42738D0B-06F8-4082-B22C-E1320067AA8A}"/>
+    <hyperlink ref="L334" r:id="rId848" xr:uid="{0C6D2367-511A-47D9-8411-1832C81886B0}"/>
+    <hyperlink ref="B335" r:id="rId849" xr:uid="{780969C1-F86A-4C31-B3D0-42DF2DBD1749}"/>
+    <hyperlink ref="L335" r:id="rId850" xr:uid="{BA46BEDF-106E-4C2C-97D0-9950416AE801}"/>
+    <hyperlink ref="B336" r:id="rId851" xr:uid="{2BF6C636-9FE6-4327-A67E-AAAB05992C16}"/>
+    <hyperlink ref="L336" r:id="rId852" xr:uid="{9546FCEF-9871-4103-AC87-74A465708AF5}"/>
+    <hyperlink ref="B337" r:id="rId853" xr:uid="{DE5138D4-280D-4167-8FEE-2558C42275D4}"/>
+    <hyperlink ref="L337" r:id="rId854" xr:uid="{9D313A09-4C47-407D-90AF-5758D1B26963}"/>
+    <hyperlink ref="B338" r:id="rId855" xr:uid="{F60232E6-0D35-4B04-ADE0-A5E12B83F2BD}"/>
+    <hyperlink ref="E338" r:id="rId856" xr:uid="{81883B9D-5191-4DF5-A261-6018675EEB8A}"/>
+    <hyperlink ref="L338" r:id="rId857" xr:uid="{BD50509D-0EF0-438F-AF66-99427B24CA85}"/>
+    <hyperlink ref="M338" r:id="rId858" xr:uid="{0186CFDF-6FFB-4F06-9918-15562DBB81D9}"/>
+    <hyperlink ref="B339" r:id="rId859" xr:uid="{CA9FE326-B603-4445-A3DB-2C04D1A46BF4}"/>
+    <hyperlink ref="E339" r:id="rId860" xr:uid="{0D425F2D-48F1-47EB-9D51-D3E76B6A7425}"/>
+    <hyperlink ref="L339" r:id="rId861" xr:uid="{C3E4D37F-990C-40DB-8979-2E531A84F78F}"/>
+    <hyperlink ref="M339" r:id="rId862" xr:uid="{7BD168FB-DA4D-42F0-A07A-BF6ECC010549}"/>
+    <hyperlink ref="B340" r:id="rId863" xr:uid="{1B203CF6-45F5-4F5F-A358-F2E49BAB4275}"/>
+    <hyperlink ref="L340" r:id="rId864" xr:uid="{BD9D4DCD-FE83-4709-9036-00C294CABB68}"/>
+    <hyperlink ref="B341" r:id="rId865" xr:uid="{8E761B14-D81A-4BE5-B08F-CF7973B09C49}"/>
+    <hyperlink ref="L341" r:id="rId866" xr:uid="{E79378AA-7239-43F0-9645-467C5A32D62E}"/>
+    <hyperlink ref="B342" r:id="rId867" xr:uid="{29556F7E-90D4-4362-B1F4-639E6DE526C4}"/>
+    <hyperlink ref="L342" r:id="rId868" xr:uid="{FB0EFDC1-394D-4A55-AF80-1FFAF5050EC7}"/>
+    <hyperlink ref="B343" r:id="rId869" xr:uid="{4C3E9932-E0B2-454F-88B2-5CCA82B491B5}"/>
+    <hyperlink ref="L343" r:id="rId870" xr:uid="{00CFF698-2E82-4762-8DE9-2D0D74F1B9A7}"/>
+    <hyperlink ref="B344" r:id="rId871" xr:uid="{1B053D71-FB5C-461B-9BFE-331E20445A5D}"/>
+    <hyperlink ref="L344" r:id="rId872" xr:uid="{109B05E3-B2F6-4EE3-9E53-7D93E0A84D69}"/>
+    <hyperlink ref="M344" r:id="rId873" xr:uid="{026FE2F3-1967-4987-9545-057A2C7C8CD9}"/>
+    <hyperlink ref="B345" r:id="rId874" xr:uid="{573898A6-D77A-4688-8497-489DDC9D3E4B}"/>
+    <hyperlink ref="L345" r:id="rId875" xr:uid="{DA4F8FE4-94B0-482B-BFA4-CB9D7CC85917}"/>
+    <hyperlink ref="B346" r:id="rId876" xr:uid="{BAF59F1E-A199-4E35-BF6A-B37E4E0F8680}"/>
+    <hyperlink ref="L346" r:id="rId877" xr:uid="{42C59A0D-9B4E-4EE6-B5CF-05B8DD9E3184}"/>
+    <hyperlink ref="M346" r:id="rId878" xr:uid="{F37819BF-153B-4FAE-9D05-37EDE95F1D5C}"/>
+    <hyperlink ref="B347" r:id="rId879" xr:uid="{AC33A3FB-8CD5-48B0-9E60-467A41C84868}"/>
+    <hyperlink ref="L347" r:id="rId880" xr:uid="{5CC01199-1B5F-4E2A-9E39-92498900AF3F}"/>
+    <hyperlink ref="M347" r:id="rId881" xr:uid="{06DAA897-FF75-4EA9-BA7E-08F1BC00E50B}"/>
+    <hyperlink ref="B348" r:id="rId882" xr:uid="{8ABBDC9F-2DA5-47F1-9B40-A4752A95D357}"/>
+    <hyperlink ref="L348" r:id="rId883" xr:uid="{42BB1AB3-76A1-4694-8EBB-FF678FA53D24}"/>
+    <hyperlink ref="M348" r:id="rId884" xr:uid="{55FD4A77-6D5F-444C-B56A-AFC7F65F511C}"/>
+    <hyperlink ref="B349" r:id="rId885" xr:uid="{3640D47E-8BEC-4068-B994-3EF88131903A}"/>
+    <hyperlink ref="L349" r:id="rId886" xr:uid="{06608F3B-7FF5-42EA-9454-1C4C3EDD37A8}"/>
+    <hyperlink ref="M349" r:id="rId887" xr:uid="{A76A3EF5-B4AD-44A3-BDB5-31BA4E1352BC}"/>
+    <hyperlink ref="B350" r:id="rId888" xr:uid="{92B49AFA-13F1-4CC2-869D-88D1764ACB9B}"/>
+    <hyperlink ref="L350" r:id="rId889" xr:uid="{4BD76C80-FBCD-474F-A9F6-B1874083684A}"/>
+    <hyperlink ref="B351" r:id="rId890" xr:uid="{287A847C-89E6-41F8-8824-405D6777A7E0}"/>
+    <hyperlink ref="L351" r:id="rId891" xr:uid="{0D98047B-CC9D-4DFF-98A4-F78F35824558}"/>
+    <hyperlink ref="B352" r:id="rId892" xr:uid="{4EBFF6CD-91B6-4996-BFAD-D707D202855E}"/>
+    <hyperlink ref="L352" r:id="rId893" xr:uid="{9A0EECE3-C807-4B36-AA7C-13393244766E}"/>
+    <hyperlink ref="B353" r:id="rId894" xr:uid="{FDBBCE02-CBCC-4B47-B25B-226F239F162D}"/>
+    <hyperlink ref="L353" r:id="rId895" xr:uid="{C4BE665A-C153-402B-A0C6-CF085EAF4D0D}"/>
+    <hyperlink ref="B354" r:id="rId896" xr:uid="{9026E9C4-71AA-4E93-AFA1-1D1426445DB5}"/>
+    <hyperlink ref="L354" r:id="rId897" xr:uid="{3662C0A1-319A-48E0-87B9-D1DCA014EA1C}"/>
+    <hyperlink ref="B355" r:id="rId898" xr:uid="{33A46EC2-9DFF-4D8C-BCA3-0BD51E81679F}"/>
+    <hyperlink ref="E355" r:id="rId899" xr:uid="{4E9AA8AA-FC3A-46E8-ACE2-70AB7FD6A8A5}"/>
+    <hyperlink ref="H355" r:id="rId900" xr:uid="{0DAADEB4-00E9-49A0-9D12-983C16FB2408}"/>
+    <hyperlink ref="L355" r:id="rId901" xr:uid="{7CAFD3C2-0811-4DF1-B59A-E3C07C8C8083}"/>
+    <hyperlink ref="M355" r:id="rId902" xr:uid="{F77D500F-EABE-4685-9C5D-308CF17A695B}"/>
+    <hyperlink ref="B356" r:id="rId903" xr:uid="{CF4C6776-FF95-4568-8BE9-4D5942265515}"/>
+    <hyperlink ref="L356" r:id="rId904" xr:uid="{45565E7F-4B61-4CB0-98A8-F386D7C938BE}"/>
+    <hyperlink ref="B357" r:id="rId905" xr:uid="{AF862B7C-2BCA-4DA1-A1B3-45D6D8023AE3}"/>
+    <hyperlink ref="L357" r:id="rId906" xr:uid="{1EF9D50C-139A-43F9-AB16-09A932464FC7}"/>
+    <hyperlink ref="B358" r:id="rId907" xr:uid="{A70D5E0D-FD9A-48A3-859D-48340CF530ED}"/>
+    <hyperlink ref="L358" r:id="rId908" xr:uid="{1BB70139-5D74-4BEF-A4A9-A2A5CDF23A88}"/>
+    <hyperlink ref="B359" r:id="rId909" xr:uid="{11D25DDF-B9C4-4027-8A0F-70513B29C837}"/>
+    <hyperlink ref="L359" r:id="rId910" xr:uid="{DEF9F3BF-AA8D-4169-AD00-E195D2199DA3}"/>
+    <hyperlink ref="B360" r:id="rId911" xr:uid="{B67A8749-761E-4BD1-AB83-7892AE6568D0}"/>
+    <hyperlink ref="L360" r:id="rId912" xr:uid="{89E54B12-0CB6-4D7E-BC23-D88F37494C17}"/>
+    <hyperlink ref="B361" r:id="rId913" xr:uid="{2B47AA65-061F-49C0-9EFB-2DAB86A1A618}"/>
+    <hyperlink ref="L361" r:id="rId914" xr:uid="{0E19A256-A7B2-4791-8918-C934A42DA8D6}"/>
+    <hyperlink ref="B362" r:id="rId915" xr:uid="{EE729189-667E-4B27-9F65-35449181322A}"/>
+    <hyperlink ref="L362" r:id="rId916" xr:uid="{13B47383-0CDA-4B56-BD00-748E70108F05}"/>
+    <hyperlink ref="B363" r:id="rId917" xr:uid="{47FA56EC-A1D7-4900-86D2-0FFE0FDE1AB6}"/>
+    <hyperlink ref="L363" r:id="rId918" xr:uid="{A480ACAD-24D9-4524-8545-260F5ADCCC5D}"/>
+    <hyperlink ref="B364" r:id="rId919" xr:uid="{E37A3039-4C03-4C61-81C7-8AC896C971DD}"/>
+    <hyperlink ref="L364" r:id="rId920" xr:uid="{A2457D1B-2EED-4005-99E4-E1D8EDBA38BB}"/>
+    <hyperlink ref="B365" r:id="rId921" xr:uid="{174C8A48-BD26-43B3-9CA7-1446EE0C31DB}"/>
+    <hyperlink ref="L365" r:id="rId922" xr:uid="{AC16B4E6-BDC7-465F-A5D1-3587084BC793}"/>
+    <hyperlink ref="B366" r:id="rId923" xr:uid="{597B6A03-0A83-4701-A1D6-7881FB2E19B6}"/>
+    <hyperlink ref="L366" r:id="rId924" xr:uid="{8D83748E-40FD-4CDA-9091-EBB2B166026A}"/>
+    <hyperlink ref="B367" r:id="rId925" xr:uid="{AEFAC0CC-3D79-441D-AC83-61E7E4E875FD}"/>
+    <hyperlink ref="L367" r:id="rId926" xr:uid="{48977D59-3064-4ED3-A0CB-87C3EAFFEADB}"/>
+    <hyperlink ref="B368" r:id="rId927" xr:uid="{68086E33-36AA-4CDF-BB7A-3CD9AE934F75}"/>
+    <hyperlink ref="L368" r:id="rId928" xr:uid="{E8E77ADB-EE9C-4051-8A33-F37389ED4013}"/>
+    <hyperlink ref="B369" r:id="rId929" xr:uid="{D661BE69-A2A7-4352-9E1A-8647B4785DD3}"/>
+    <hyperlink ref="L369" r:id="rId930" xr:uid="{4AFAEED0-79F2-4166-8616-A2920B598E10}"/>
+    <hyperlink ref="B370" r:id="rId931" xr:uid="{C03C7BC4-C567-460E-B258-C16D170E130B}"/>
+    <hyperlink ref="L370" r:id="rId932" xr:uid="{431A58C7-AD29-4FFD-B961-90FE902DECBE}"/>
+    <hyperlink ref="B371" r:id="rId933" xr:uid="{FEF83608-3026-4CCD-B5EA-3F989C333E2B}"/>
+    <hyperlink ref="L371" r:id="rId934" xr:uid="{68613369-F3BE-4F15-8672-1972BC61BC94}"/>
+    <hyperlink ref="M371" r:id="rId935" xr:uid="{A150508E-168B-4CB5-ABFA-B7CA3F734C78}"/>
+    <hyperlink ref="B372" r:id="rId936" xr:uid="{3216DE7A-484E-4A41-B6FD-D6B15C5EBE3F}"/>
+    <hyperlink ref="L372" r:id="rId937" xr:uid="{91FCA9B6-CE5F-4BAD-9C77-E6FADB173EC1}"/>
+    <hyperlink ref="B373" r:id="rId938" xr:uid="{EBF727C4-16E5-4C38-8FD7-7A6B908EB30A}"/>
+    <hyperlink ref="L373" r:id="rId939" xr:uid="{64F3A3CE-5ADA-4AD8-815D-43F55F169F31}"/>
+    <hyperlink ref="B374" r:id="rId940" xr:uid="{83B5BE74-095D-457A-BA95-93990B4614EE}"/>
+    <hyperlink ref="L374" r:id="rId941" xr:uid="{F9462463-8510-42B7-8315-320CE3F05722}"/>
+    <hyperlink ref="B375" r:id="rId942" xr:uid="{867D6D6B-5531-46CC-A3B0-0CE3DBF8F4F5}"/>
+    <hyperlink ref="L375" r:id="rId943" xr:uid="{C672FBEF-9BB3-4D4B-8646-18467ED8C09E}"/>
+    <hyperlink ref="B376" r:id="rId944" xr:uid="{463056BB-EB2D-4ADF-871D-FBA1412681C4}"/>
+    <hyperlink ref="L376" r:id="rId945" xr:uid="{EAD7C76B-A7DE-4523-AD2E-7A7C1924B855}"/>
+    <hyperlink ref="B377" r:id="rId946" xr:uid="{B849381A-0B3E-4629-B3DB-5A74178E65AD}"/>
+    <hyperlink ref="E377" r:id="rId947" xr:uid="{9C8E9BB1-A0AF-43F8-8B91-1E1B175BDFAC}"/>
+    <hyperlink ref="L377" r:id="rId948" xr:uid="{BE800076-DD97-4850-A5C4-2FAFB1CB9DF2}"/>
+    <hyperlink ref="M377" r:id="rId949" xr:uid="{5B239AF6-5BE1-40B3-9F9D-D45312ADBC1E}"/>
+    <hyperlink ref="B378" r:id="rId950" xr:uid="{FA469E39-42FF-4B94-B825-12EF2D81D91F}"/>
+    <hyperlink ref="L378" r:id="rId951" xr:uid="{E585D031-08ED-4DF9-81D4-0DFA0CE30883}"/>
+    <hyperlink ref="B379" r:id="rId952" xr:uid="{0CE83767-1207-4A66-9CE8-EB082667B41A}"/>
+    <hyperlink ref="E379" r:id="rId953" xr:uid="{4992718B-5890-497C-8B04-9393DEEBD2BD}"/>
+    <hyperlink ref="L379" r:id="rId954" xr:uid="{4239094C-712C-4DBC-9AF4-2B2BB8C819AD}"/>
+    <hyperlink ref="M379" r:id="rId955" xr:uid="{840CD2C2-00AF-40E6-8A4C-3A05571E6D2E}"/>
+    <hyperlink ref="B380" r:id="rId956" xr:uid="{87361EC7-D93B-4E84-8E24-3D332AA8B287}"/>
+    <hyperlink ref="L380" r:id="rId957" xr:uid="{3693E6F1-CA79-45C7-B4C4-E7A3C9C2CD38}"/>
+    <hyperlink ref="B381" r:id="rId958" xr:uid="{331DC7D7-9C1C-4F00-A72C-A327D01D6BE8}"/>
+    <hyperlink ref="E381" r:id="rId959" xr:uid="{22A00CFF-7207-49EC-A74D-2C5780F9ACE5}"/>
+    <hyperlink ref="L381" r:id="rId960" xr:uid="{E599AD6B-5859-4434-9846-3F28DE6BB9D2}"/>
+    <hyperlink ref="M381" r:id="rId961" xr:uid="{9B173F5A-6645-4575-9C6E-23CA10D02F07}"/>
+    <hyperlink ref="B382" r:id="rId962" xr:uid="{09340EDB-30BD-4F59-B9E6-45EEED14DEDC}"/>
+    <hyperlink ref="E382" r:id="rId963" xr:uid="{74818830-46B7-47EB-9E50-1A190B7ECB1A}"/>
+    <hyperlink ref="L382" r:id="rId964" xr:uid="{93D0E2B0-8E98-4862-A741-3D44111D7376}"/>
+    <hyperlink ref="M382" r:id="rId965" xr:uid="{0F214CC3-69A3-46A4-8162-D71000EA287F}"/>
+    <hyperlink ref="B383" r:id="rId966" xr:uid="{6FC71DEE-864F-44CD-B235-7838A1E5C55F}"/>
+    <hyperlink ref="E383" r:id="rId967" xr:uid="{D9E81F59-8D1B-4E72-85F2-179828D454E5}"/>
+    <hyperlink ref="L383" r:id="rId968" xr:uid="{BD20B3BD-ABB4-48BE-8842-5F4C5489E63A}"/>
+    <hyperlink ref="M383" r:id="rId969" xr:uid="{8FF16A23-2371-47C5-B881-C3F1CD760E4A}"/>
+    <hyperlink ref="B384" r:id="rId970" xr:uid="{996C8CEA-A8B7-4C17-B23B-C16F4509A6CB}"/>
+    <hyperlink ref="L384" r:id="rId971" xr:uid="{C04646E6-D180-4914-BD6E-37FA4AC55343}"/>
+    <hyperlink ref="M384" r:id="rId972" xr:uid="{C2009D8A-DE9D-4DF0-8C9F-FB1CFBA643DA}"/>
+    <hyperlink ref="B385" r:id="rId973" xr:uid="{A09A12D0-D62C-45B9-B02F-64A12AAC3D78}"/>
+    <hyperlink ref="E385" r:id="rId974" xr:uid="{1BFD2D37-AE07-46BE-80C5-F08CD2663BE7}"/>
+    <hyperlink ref="L385" r:id="rId975" xr:uid="{92355D8D-D198-4365-8C46-188ADF773779}"/>
+    <hyperlink ref="M385" r:id="rId976" xr:uid="{EE461818-F2E2-479E-A641-B857CC3EE05D}"/>
+    <hyperlink ref="B386" r:id="rId977" xr:uid="{4FDFF20E-775A-40B6-9F04-6AD6920B639F}"/>
+    <hyperlink ref="L386" r:id="rId978" xr:uid="{2ACCC96E-1DB8-40A0-8E95-346068135572}"/>
+    <hyperlink ref="B387" r:id="rId979" xr:uid="{BD8C6AA0-B35B-42DE-A833-FC7E370F0E16}"/>
+    <hyperlink ref="L387" r:id="rId980" xr:uid="{5A97BFCE-8B8B-4181-9226-FEA63018AFBA}"/>
+    <hyperlink ref="B388" r:id="rId981" xr:uid="{3F3D81F8-33EE-4C53-848D-8FA315C0178A}"/>
+    <hyperlink ref="L388" r:id="rId982" xr:uid="{EBE9EE7C-8BA2-4C38-BCAC-6407A61BB186}"/>
+    <hyperlink ref="B389" r:id="rId983" xr:uid="{74F65253-16BA-401A-8315-F518EB15099D}"/>
+    <hyperlink ref="L389" r:id="rId984" xr:uid="{1A152F16-EE51-4985-BE83-3D141ADB3596}"/>
+    <hyperlink ref="B390" r:id="rId985" xr:uid="{12714CEE-8714-4BFB-ADEA-FA8B6C9FA1F0}"/>
+    <hyperlink ref="L390" r:id="rId986" xr:uid="{E61D9B5C-61D3-44E0-8A76-ED7B7DAD3C1C}"/>
+    <hyperlink ref="B391" r:id="rId987" xr:uid="{FF9B30EF-CE5A-4B12-AC2F-6F4665C3E6BD}"/>
+    <hyperlink ref="L391" r:id="rId988" xr:uid="{F729DC88-A03C-4A09-8D01-25079026F9B0}"/>
+    <hyperlink ref="B392" r:id="rId989" xr:uid="{DA6D1784-B5E6-414D-B64B-40126B520C4E}"/>
+    <hyperlink ref="L392" r:id="rId990" xr:uid="{51FA8C96-9C12-4D77-95EB-6283B127D87B}"/>
+    <hyperlink ref="B393" r:id="rId991" xr:uid="{CA29DBD0-B019-4FB2-AF12-5EFE5B5C49B0}"/>
+    <hyperlink ref="L393" r:id="rId992" xr:uid="{874F52C8-0295-4964-B19D-78D99EDB8336}"/>
+    <hyperlink ref="B394" r:id="rId993" xr:uid="{A44C00E7-FEA4-4E53-AFAE-028E0E5FEFB7}"/>
+    <hyperlink ref="L394" r:id="rId994" xr:uid="{5B99DEA2-BCE6-49EC-B417-77797E562AD4}"/>
+    <hyperlink ref="B395" r:id="rId995" xr:uid="{2C123C10-3841-476B-A078-4BBE157E76D1}"/>
+    <hyperlink ref="E395" r:id="rId996" xr:uid="{4EC5E290-CE87-43E8-8145-5BCBF28A7E35}"/>
+    <hyperlink ref="H395" r:id="rId997" xr:uid="{4C94E246-9E4C-4349-8459-5DC104FE0039}"/>
+    <hyperlink ref="L395" r:id="rId998" xr:uid="{20289652-91C0-4F84-BED5-AA0CEBAD8F76}"/>
+    <hyperlink ref="M395" r:id="rId999" xr:uid="{C6F49EF9-36A8-4279-82F3-3C233A59F789}"/>
+    <hyperlink ref="B396" r:id="rId1000" xr:uid="{6CA128F3-6743-4665-9C98-C98B8DA7E101}"/>
+    <hyperlink ref="E396" r:id="rId1001" xr:uid="{290F016E-F131-45F7-94D6-2AE0A30AAA2A}"/>
+    <hyperlink ref="H396" r:id="rId1002" xr:uid="{9C2B44CA-A3E9-43EA-90C2-B0FF74D952C8}"/>
+    <hyperlink ref="L396" r:id="rId1003" xr:uid="{50A1CCB8-0D16-401F-A72B-1C56A34A07BA}"/>
+    <hyperlink ref="M396" r:id="rId1004" xr:uid="{E24F28BF-6CA4-4DAA-954D-505904929B4B}"/>
+    <hyperlink ref="B397" r:id="rId1005" xr:uid="{11CE0D8A-DB8A-438D-BF2F-03086E8E65C8}"/>
+    <hyperlink ref="E397" r:id="rId1006" xr:uid="{7B24330B-40E2-494F-AC68-B6F8F05FF546}"/>
+    <hyperlink ref="H397" r:id="rId1007" xr:uid="{C0214436-0250-4AA5-B619-A2FA34752B9E}"/>
+    <hyperlink ref="L397" r:id="rId1008" xr:uid="{54AC3DFC-40FD-4C33-8FAC-EA17B7E6C71C}"/>
+    <hyperlink ref="M397" r:id="rId1009" xr:uid="{00EC0596-3FA4-4537-89E7-B478336E5B65}"/>
+    <hyperlink ref="B398" r:id="rId1010" xr:uid="{AD3D3AE9-EAE7-4936-AD9A-B97ACC5D0EDF}"/>
+    <hyperlink ref="L398" r:id="rId1011" xr:uid="{345DFB34-FEC2-4B72-9575-9AFAD003BC71}"/>
+    <hyperlink ref="B399" r:id="rId1012" xr:uid="{73E2C807-9B4E-4C5C-9043-2C18D911B1B1}"/>
+    <hyperlink ref="L399" r:id="rId1013" xr:uid="{A15E2915-1446-403D-9A10-7441E387928A}"/>
+    <hyperlink ref="B400" r:id="rId1014" xr:uid="{442F49A1-CDA3-461D-A485-D64217173628}"/>
+    <hyperlink ref="L400" r:id="rId1015" xr:uid="{C7499EE7-3DCB-4285-9C54-2DE06666DA83}"/>
+    <hyperlink ref="B401" r:id="rId1016" xr:uid="{220A7190-59CF-4569-B9FD-55A36FDCFF9C}"/>
+    <hyperlink ref="L401" r:id="rId1017" xr:uid="{7A895455-0E6E-47AE-A9C8-855256D07D20}"/>
+    <hyperlink ref="B402" r:id="rId1018" xr:uid="{F41E9094-1639-4903-8E9E-B7DB72B580FD}"/>
+    <hyperlink ref="L402" r:id="rId1019" xr:uid="{8566ECD8-497C-4F6D-AEA9-62F61000B9C2}"/>
+    <hyperlink ref="B403" r:id="rId1020" xr:uid="{304E0292-01BF-4867-A361-658626C48C3A}"/>
+    <hyperlink ref="L403" r:id="rId1021" xr:uid="{923AB061-177B-4E95-92C7-16C7FB083DEA}"/>
+    <hyperlink ref="B404" r:id="rId1022" xr:uid="{B437A625-B82B-4DE7-9F64-CBAE6D0F1FDF}"/>
+    <hyperlink ref="L404" r:id="rId1023" xr:uid="{80008E87-35B0-454A-8DEB-E6A3844C2934}"/>
+    <hyperlink ref="B405" r:id="rId1024" xr:uid="{0EB65B14-2DDF-4DA8-965B-657FD6627720}"/>
+    <hyperlink ref="L405" r:id="rId1025" xr:uid="{516921F8-FE85-4E59-B05E-3C08ADA6104F}"/>
+    <hyperlink ref="B406" r:id="rId1026" xr:uid="{E5EBD5F2-E0C2-4765-B449-7E9E13636667}"/>
+    <hyperlink ref="L406" r:id="rId1027" xr:uid="{96976492-24CB-42DC-8C8A-088F231D814A}"/>
+    <hyperlink ref="B407" r:id="rId1028" xr:uid="{35283EDD-582C-44A6-8FDD-1DA531E816AF}"/>
+    <hyperlink ref="E407" r:id="rId1029" xr:uid="{8E10DF19-67EE-4867-A1AF-920059CC96EB}"/>
+    <hyperlink ref="L407" r:id="rId1030" xr:uid="{E3ECFB0C-6244-4193-A53C-C8124D93E015}"/>
+    <hyperlink ref="M407" r:id="rId1031" xr:uid="{A5152444-F21B-4D14-B5F6-8A8DB9F59A81}"/>
+    <hyperlink ref="B408" r:id="rId1032" xr:uid="{748BDA96-C5BD-4C0C-BD89-DAF501DA3FDE}"/>
+    <hyperlink ref="H408" r:id="rId1033" xr:uid="{1E8ECD30-51B8-4AA2-B8CC-6CAA790AF2D8}"/>
+    <hyperlink ref="L408" r:id="rId1034" xr:uid="{BF3E0921-9EF3-4EB2-984F-CCAC3316A172}"/>
+    <hyperlink ref="M408" r:id="rId1035" xr:uid="{4BCD1D27-7F07-4A4B-AC41-8FEFE75BFE94}"/>
+    <hyperlink ref="B409" r:id="rId1036" xr:uid="{D776FBD5-F716-4385-AC42-127C5F17D8BC}"/>
+    <hyperlink ref="L409" r:id="rId1037" xr:uid="{2B1A6CFC-91BC-4664-95BB-8F87AEECD788}"/>
+    <hyperlink ref="B410" r:id="rId1038" xr:uid="{B2F045DE-C98B-42CB-980F-217C22440A0D}"/>
+    <hyperlink ref="E410" r:id="rId1039" xr:uid="{9AB6A80E-2699-47E8-92F3-5E47FE34A370}"/>
+    <hyperlink ref="H410" r:id="rId1040" xr:uid="{CDCDE12E-1420-4A2B-8F3A-DFB828182B55}"/>
+    <hyperlink ref="L410" r:id="rId1041" xr:uid="{28D9165D-CE4F-4DA8-9467-9095A959419E}"/>
+    <hyperlink ref="M410" r:id="rId1042" xr:uid="{4406979F-03B5-4F8C-82FF-7FC43F936034}"/>
+    <hyperlink ref="B411" r:id="rId1043" xr:uid="{E95B4B2B-B401-4C6A-BB51-131C3CD68BDB}"/>
+    <hyperlink ref="L411" r:id="rId1044" xr:uid="{FDF67677-08D7-468A-B077-EC634941D14F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>